<commit_message>
Update documentation for RheoBoard version 2
- Revised `CHANGELOG.md`, `README.md`, and `BuildYourOwn/README.md` to clarify the transition to a 3D-printed panel, removing references to the previous laser-cut design.
- Updated `okh-RheoBoard.yml` to reflect the current version and its status, ensuring consistency across documentation.
- Enhanced clarity regarding the assembly instructions and parts list, emphasizing the new design and providing updated links to relevant files.

These updates improve user understanding of the project's evolution and provide comprehensive guidance for building and using the RheoBoard.
</commit_message>
<xml_diff>
--- a/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
+++ b/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R365707313e7f429f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="R38c903e061744abb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="Rbc64fafccc8d4f5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R48e5bb8df6624937"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="Rd7655b6f73204586"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="Re857c47a2b054d67"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:M50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
@@ -160,7 +160,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RheoBoard105Accessories" displayName="RheoBoard105Accessories" ref="A1:G7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RheoBoard105Accessories" displayName="RheoBoard105Accessories" ref="A1:G8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Item"/>
     <x:tableColumn id="2" name="Quantity basis"/>
@@ -175,7 +175,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RheoBoard105SMT" displayName="RheoBoard105SMT" ref="A1:D44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RheoBoard105SMT" displayName="RheoBoard105SMT" ref="A1:D45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
@@ -475,12 +475,12 @@
       </x:c>
       <x:c r="M2" s="7" t="str"/>
     </x:row>
-    <x:row r="3" ht="53" customHeight="1">
+    <x:row r="3" ht="126" customHeight="1">
       <x:c r="A3" s="7" t="str">
         <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>C3,C4,C5,C23,C24,C25,C26,C30,C31,C33,C42,C44,C46,C47,C56,C59,C63</x:v>
+        <x:v>C3, C4, C5, C23, C24, C25, C26, C30, C31, C33, C42, C44, C46, C47, C56, C59, C63, C68, C69</x:v>
       </x:c>
       <x:c r="C3" s="7" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
@@ -489,14 +489,14 @@
         <x:v>C14663</x:v>
       </x:c>
       <x:c r="E3" s="8" t="n">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F3" s="9" t="n">
         <x:v>0.073</x:v>
       </x:c>
       <x:c r="G3" s="9" t="n">
         <x:f>IF(ISNUMBER(F3),E3*F3,"")</x:f>
-        <x:v>1.2409999999999999</x:v>
+        <x:v>1.387</x:v>
       </x:c>
       <x:c r="H3" s="7" t="str">
         <x:v>https://www.lcsc.com/product-detail/C14663.html</x:v>
@@ -511,7 +511,9 @@
       <x:c r="L3" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M3" s="7" t="str"/>
+      <x:c r="M3" s="7" t="str">
+        <x:v>C68/C69 added as local/host U13 supply bypass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="53" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -1172,7 +1174,9 @@
       <x:c r="L20" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M20" s="7" t="str"/>
+      <x:c r="M20" s="7" t="str">
+        <x:v>Standard Qwiic pin order: 1 GND, 2 3.3 V, 3 SDA, 4 SCL. J9 is the dedicated MASTER port; J1/J12/J17 power local SENSOR modules. J9 power/signal nets are separated by U13.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="53" customHeight="1">
       <x:c r="A21" s="11" t="str">
@@ -1294,7 +1298,7 @@
         <x:v>Manual THT</x:v>
       </x:c>
       <x:c r="M23" s="11" t="str">
-        <x:v>New master/mux header: pin 1 GND, pin 2 SDA, pin 3 SCL. Manual through-hole assembly.</x:v>
+        <x:v>LOCAL BUS SERVICE connector: GND/SDA/SCL, no power pin. Bypasses U13; use J9 for the USB/battery-powered Qwiic master.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="53" customHeight="1">
@@ -1458,7 +1462,7 @@
         <x:v>4K7/0603/1%</x:v>
       </x:c>
       <x:c r="B28" s="7" t="str">
-        <x:v>R11,R15,R20</x:v>
+        <x:v>R11, R15, R20, R82, R83</x:v>
       </x:c>
       <x:c r="C28" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
@@ -1467,14 +1471,14 @@
         <x:v>C23162</x:v>
       </x:c>
       <x:c r="E28" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F28" s="9" t="n">
         <x:v>0.001</x:v>
       </x:c>
       <x:c r="G28" s="9" t="n">
         <x:f>IF(ISNUMBER(F28),E28*F28,"")</x:f>
-        <x:v>0.003</x:v>
+        <x:v>0.005</x:v>
       </x:c>
       <x:c r="H28" s="7" t="str">
         <x:v>https://www.lcsc.com/product-detail/C23162.html</x:v>
@@ -1489,14 +1493,16 @@
       <x:c r="L28" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M28" s="7" t="str"/>
-    </x:row>
-    <x:row r="29" ht="53" customHeight="1">
+      <x:c r="M28" s="7" t="str">
+        <x:v>R82/R83 added as 4.7 kohm host SDA/SCL pullups; local R15/R20 retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="126" customHeight="1">
       <x:c r="A29" s="7" t="str">
         <x:v>10K/0603/1%</x:v>
       </x:c>
       <x:c r="B29" s="7" t="str">
-        <x:v>R13,R14,R16,R17,R18,R19,R22,R23,R29,R30,R31,R32,R33,R34,R37,R38,R51,R56</x:v>
+        <x:v>R13, R14, R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84</x:v>
       </x:c>
       <x:c r="C29" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
@@ -1505,14 +1511,14 @@
         <x:v>C25804</x:v>
       </x:c>
       <x:c r="E29" s="8" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F29" s="9" t="n">
         <x:v>0.014</x:v>
       </x:c>
       <x:c r="G29" s="9" t="n">
         <x:f>IF(ISNUMBER(F29),E29*F29,"")</x:f>
-        <x:v>0.252</x:v>
+        <x:v>0.266</x:v>
       </x:c>
       <x:c r="H29" s="7" t="str">
         <x:v>https://www.lcsc.com/product-detail/C25804.html</x:v>
@@ -1527,7 +1533,9 @@
       <x:c r="L29" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M29" s="7" t="str"/>
+      <x:c r="M29" s="7" t="str">
+        <x:v>R84 added from HOST_3V3 to GND for discharge (0.33 mA nominal).</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="53" customHeight="1">
       <x:c r="A30" s="7" t="str">
@@ -2292,6 +2300,45 @@
       </x:c>
       <x:c r="M49" s="7" t="str">
         <x:v>New auto-retry input eFuse; TI RPW0010A HotRod footprint, approximately 2 A limit / 13.8 V clamp.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="112" customHeight="1">
+      <x:c r="A50" s="7" t="str">
+        <x:v>TCA9517ADGKR</x:v>
+      </x:c>
+      <x:c r="B50" s="7" t="str">
+        <x:v>U13</x:v>
+      </x:c>
+      <x:c r="C50" s="7" t="str">
+        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
+      </x:c>
+      <x:c r="D50" s="7" t="str">
+        <x:v>C201698</x:v>
+      </x:c>
+      <x:c r="E50" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F50" s="10"/>
+      <x:c r="G50" s="9" t="str">
+        <x:f>IF(ISNUMBER(F50),E50*F50,"")</x:f>
+      </x:c>
+      <x:c r="H50" s="7" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C201698.html</x:v>
+      </x:c>
+      <x:c r="I50" s="7" t="str">
+        <x:v>https://www.ti.com/lit/ds/symlink/tca9517a.pdf</x:v>
+      </x:c>
+      <x:c r="J50" s="7" t="str">
+        <x:v>TCA9517ADGKR</x:v>
+      </x:c>
+      <x:c r="K50" s="7" t="str">
+        <x:v>Texas Instruments</x:v>
+      </x:c>
+      <x:c r="L50" s="7" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M50" s="7" t="str">
+        <x:v>Qwiic master interface: local bus on A, host on B. EN and VCCB use HOST_3V3; separate supplies, common GND. TI DGK land pattern: 1.4 x 0.45 mm pads, 0.65 mm pitch, 4.4 mm row-center span.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="30" customHeight="1">
@@ -2302,15 +2349,15 @@
       <x:c r="C51" s="14"/>
       <x:c r="D51" s="14"/>
       <x:c r="E51" s="14" t="n">
-        <x:f>SUM(E2:E49)</x:f>
-        <x:v>141</x:v>
+        <x:f>SUM(E2:E50)</x:f>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="F51" s="14" t="str">
         <x:v>Incomplete estimate</x:v>
       </x:c>
       <x:c r="G51" s="15" t="n">
-        <x:f>SUM(G2:G49)</x:f>
-        <x:v>55.456</x:v>
+        <x:f>SUM(G2:G50)</x:f>
+        <x:v>55.617999999999995</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="34" customHeight="1">
@@ -2337,7 +2384,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6927c6d7a7e4910"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2396359dc474a04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2401,12 +2448,12 @@
         <x:v>Existing specified valve retained. JST XH mating cable; verify supplied cable polarity. Header parts appear on main BOM separately.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="85" customHeight="1">
+    <x:row r="3" ht="154" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Master connector housing</x:v>
+        <x:v>Local service connector housing</x:v>
       </x:c>
       <x:c r="B3" s="3" t="str">
-        <x:v>1 per board</x:v>
+        <x:v>Optional: 1 per board</x:v>
       </x:c>
       <x:c r="C3" s="3" t="str">
         <x:v>JST</x:v>
@@ -2415,21 +2462,21 @@
         <x:v>EHR-3</x:v>
       </x:c>
       <x:c r="E3" s="3" t="str">
-        <x:v>Mating cable housing for J18</x:v>
+        <x:v>J18 local-bus service mating housing</x:v>
       </x:c>
       <x:c r="F3" s="3" t="str">
         <x:v>https://www.jst-mfg.com/product/pdf/eng/eEH.pdf</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Pin 1 GND, pin 2 SDA, pin 3 SCL. No 3.3 V wire. A professionally assembled matching cable may substitute for separate housing/contacts.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="85" customHeight="1">
+        <x:v>GND/SDA/SCL only; bypasses U13. The standard Qwiic master cable connects to J9.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="154" customHeight="1">
       <x:c r="A4" s="3" t="str">
-        <x:v>Master connector contacts</x:v>
+        <x:v>Local service connector contacts</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
-        <x:v>3 per board</x:v>
+        <x:v>Optional: 3 per housing</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
         <x:v>JST</x:v>
@@ -2438,16 +2485,16 @@
         <x:v>SEH-001T-P0.6</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str">
-        <x:v>Crimp contacts for EHR-3 housing</x:v>
+        <x:v>Contacts for optional J18 service harness</x:v>
       </x:c>
       <x:c r="F4" s="3" t="str">
         <x:v>https://www.jst-mfg.com/product/pdf/eng/eEH.pdf</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>Choose wire in the contact specification and use the appropriate crimp tooling. Verify end-to-end pin mapping before connection.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="85" customHeight="1">
+        <x:v>Select wire size and crimping method to JST specification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="154" customHeight="1">
       <x:c r="A5" s="3" t="str">
         <x:v>Eight-channel I2C multiplexer</x:v>
       </x:c>
@@ -2467,10 +2514,10 @@
         <x:v>https://www.adafruit.com/product/2717</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
-        <x:v>Working system assumption. Power mux from master 3.3 V; configure address 0x71 and select one channel at a time. Connect downstream GND/SDA/SCL only.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="85" customHeight="1">
+        <x:v>Address 0x71; exactly one channel enabled. Master 3.3 V/GND/channel SDA/SCL to J9; local rails stay separate. Product 2717 needs a Qwiic adapter harness. No upstream B-side repeater/rise-time accelerator. Total host pullup current &lt;=3 mA; selected-branch effective pullups &gt;=2.2 kohm including parallel module resistors/tolerance. Verify actual wiring and rise times.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="154" customHeight="1">
       <x:c r="A6" s="3" t="str">
         <x:v>12 V power supply</x:v>
       </x:c>
@@ -2493,31 +2540,56 @@
         <x:v>12 V, 2 A starting rating for specified loads; validate actual startup and simultaneous-load current. Board input fuse 2 A; do not increase load budget just because supply is larger.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="85" customHeight="1">
+    <x:row r="7" ht="154" customHeight="1">
       <x:c r="A7" s="3" t="str">
-        <x:v>Master controller</x:v>
+        <x:v>Qwiic master</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
         <x:v>1 per system</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
-        <x:v>To be selected</x:v>
+        <x:v>SparkFun</x:v>
       </x:c>
       <x:c r="D7" s="3" t="str">
-        <x:v>3.3 V logic I2C controller</x:v>
+        <x:v>WRL-15663 (ESP32 Thing Plus, Micro-B)</x:v>
       </x:c>
       <x:c r="E7" s="3" t="str">
-        <x:v>PWM, valves, button handling and pressure reads</x:v>
-      </x:c>
-      <x:c r="F7" s="3" t="str"/>
+        <x:v>USB/battery-powered I2C master; GPIO23 SDA, GPIO22 SCL</x:v>
+      </x:c>
+      <x:c r="F7" s="3" t="str">
+        <x:v>https://cdn.sparkfun.com/assets/6/d/c/6/c/ESP32_Thing_Plus_Schematic.pdf</x:v>
+      </x:c>
       <x:c r="G7" s="3" t="str">
-        <x:v>No controller on RheoBoard. Firmware must implement the documented register initialization and mux addressing. Existing DIY firmware is not a PCB release.</x:v>
+        <x:v>Connect standard four-wire Qwiic to J9 MASTER. Host 3.3 V powers only the host interface. Other Thing Plus variants require their own pin/power check. PCB-specific firmware initialization is required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="154" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>Standard Qwiic cable</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="str">
+        <x:v>1 per connection</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="str">
+        <x:v>Qwiic-compatible cable supplier</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="str">
+        <x:v>Four-wire JST SH 1.0 mm mating cable; length to suit</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="str">
+        <x:v>Master to J9, or local sensors to J1/J12/J17</x:v>
+      </x:c>
+      <x:c r="F8" s="3" t="str">
+        <x:v>https://www.sparkfun.com/qwiic</x:v>
+      </x:c>
+      <x:c r="G8" s="3" t="str">
+        <x:v>Pin 1 GND (black), 2 3.3 V (red), 3 SDA (blue), 4 SCL (yellow). Observe connector pin numbering; do not infer pin order from viewing direction.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43c3596e263f4d4b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b3d0d4779294d8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2565,7 +2637,7 @@
         <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B3" s="3" t="str">
-        <x:v>C3,C4,C5,C23,C24,C25,C26,C30,C31,C33,C42,C44,C46,C47,C56,C59,C63</x:v>
+        <x:v>C3, C4, C5, C23, C24, C25, C26, C30, C31, C33, C42, C44, C46, C47, C56, C59, C63, C68, C69</x:v>
       </x:c>
       <x:c r="C3" s="3" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
@@ -2873,7 +2945,7 @@
         <x:v>4K7/0603/1%</x:v>
       </x:c>
       <x:c r="B25" s="3" t="str">
-        <x:v>R11,R15,R20</x:v>
+        <x:v>R11, R15, R20, R82, R83</x:v>
       </x:c>
       <x:c r="C25" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
@@ -2887,7 +2959,7 @@
         <x:v>10K/0603/1%</x:v>
       </x:c>
       <x:c r="B26" s="3" t="str">
-        <x:v>R13,R14,R16,R17,R18,R19,R22,R23,R29,R30,R31,R32,R33,R34,R37,R38,R51,R56</x:v>
+        <x:v>R13, R14, R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84</x:v>
       </x:c>
       <x:c r="C26" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
@@ -3148,10 +3220,24 @@
         <x:v>C3662789</x:v>
       </x:c>
     </x:row>
+    <x:row r="45" ht="70" customHeight="1">
+      <x:c r="A45" s="3" t="str">
+        <x:v>TCA9517ADGKR</x:v>
+      </x:c>
+      <x:c r="B45" s="3" t="str">
+        <x:v>U13</x:v>
+      </x:c>
+      <x:c r="C45" s="3" t="str">
+        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
+      </x:c>
+      <x:c r="D45" s="3" t="str">
+        <x:v>C201698</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f7353b245c84904"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5fafd3e4a084324"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Remove redundant J18 header and update documentation for RheoBoard v1.05
- Removed the J18 local service header from the PCB design, as it is no longer needed.
- Updated the assembly instructions to reflect the removal of J18 and clarified the role of J3 as the local debug header.
- Revised the README and BOM to indicate the changes in the connector layout and part count.
- Adjusted the Gerber files and other manufacturing documents to ensure consistency with the updated design.

These changes streamline the design and improve the clarity of the documentation for users and manufacturers.
</commit_message>
<xml_diff>
--- a/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
+++ b/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R48e5bb8df6624937"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="Rd7655b6f73204586"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="Re857c47a2b054d67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R9c36f24d735a4c3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="Rad8e0848fc514f90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="R381aa90d17ac465b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:M50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
@@ -160,7 +160,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RheoBoard105Accessories" displayName="RheoBoard105Accessories" ref="A1:G8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="RheoBoard105Accessories" displayName="RheoBoard105Accessories" ref="A1:G6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Item"/>
     <x:tableColumn id="2" name="Quantity basis"/>
@@ -1263,118 +1263,117 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="53" customHeight="1">
-      <x:c r="A23" s="11" t="str">
-        <x:v>JST EH 3-pin 2.50mm</x:v>
-      </x:c>
-      <x:c r="B23" s="11" t="str">
-        <x:v>J18</x:v>
-      </x:c>
-      <x:c r="C23" s="11" t="str">
-        <x:v>Connector_JST:JST_EH_B3B-EH-A_1x03_P2.50mm_Vertical</x:v>
-      </x:c>
-      <x:c r="D23" s="11" t="str">
-        <x:v>C160259</x:v>
-      </x:c>
-      <x:c r="E23" s="12" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F23" s="10"/>
-      <x:c r="G23" s="13" t="str">
+      <x:c r="A23" s="7" t="str">
+        <x:v>4.7uH FXL0530-4R7-M</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="str">
+        <x:v>L1,L2,L5</x:v>
+      </x:c>
+      <x:c r="C23" s="7" t="str">
+        <x:v>Inductor_SMD:L_Changjiang_FXL0530</x:v>
+      </x:c>
+      <x:c r="D23" s="7" t="str">
+        <x:v>C177246</x:v>
+      </x:c>
+      <x:c r="E23" s="8" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F23" s="9" t="n">
+        <x:v>0.904</x:v>
+      </x:c>
+      <x:c r="G23" s="9" t="n">
         <x:f>IF(ISNUMBER(F23),E23*F23,"")</x:f>
-      </x:c>
-      <x:c r="H23" s="11" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C160259.html</x:v>
-      </x:c>
-      <x:c r="I23" s="11" t="str">
-        <x:v>https://www.jst-mfg.com/product/pdf/eng/eEH.pdf</x:v>
-      </x:c>
-      <x:c r="J23" s="11" t="str">
-        <x:v>B3B-EH-A(LF)(SN)</x:v>
-      </x:c>
-      <x:c r="K23" s="11" t="str">
-        <x:v>JST</x:v>
-      </x:c>
-      <x:c r="L23" s="11" t="str">
-        <x:v>Manual THT</x:v>
-      </x:c>
-      <x:c r="M23" s="11" t="str">
-        <x:v>LOCAL BUS SERVICE connector: GND/SDA/SCL, no power pin. Bypasses U13; use J9 for the USB/battery-powered Qwiic master.</x:v>
+        <x:v>2.712</x:v>
+      </x:c>
+      <x:c r="H23" s="7" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C177246.html</x:v>
+      </x:c>
+      <x:c r="I23" s="7"/>
+      <x:c r="J23" s="7" t="str">
+        <x:v>FXL0530-4R7-M</x:v>
+      </x:c>
+      <x:c r="K23" s="7" t="str">
+        <x:v>cjiang</x:v>
+      </x:c>
+      <x:c r="L23" s="7" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M23" s="7" t="str">
+        <x:v>FXL0530 pads match the selected inductor; old Bourns purchasing link removed.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="53" customHeight="1">
       <x:c r="A24" s="7" t="str">
-        <x:v>4.7uH FXL0530-4R7-M</x:v>
+        <x:v>AO3400A</x:v>
       </x:c>
       <x:c r="B24" s="7" t="str">
-        <x:v>L1,L2,L5</x:v>
+        <x:v>Q3,Q4,Q8,Q10</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
-        <x:v>Inductor_SMD:L_Changjiang_FXL0530</x:v>
+        <x:v>RheoBoard:AO3400A</x:v>
       </x:c>
       <x:c r="D24" s="7" t="str">
-        <x:v>C177246</x:v>
+        <x:v>C20917</x:v>
       </x:c>
       <x:c r="E24" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F24" s="9" t="n">
-        <x:v>0.904</x:v>
+        <x:v>0.322</x:v>
       </x:c>
       <x:c r="G24" s="9" t="n">
         <x:f>IF(ISNUMBER(F24),E24*F24,"")</x:f>
-        <x:v>2.712</x:v>
+        <x:v>1.288</x:v>
       </x:c>
       <x:c r="H24" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C177246.html</x:v>
-      </x:c>
-      <x:c r="I24" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C20917.html</x:v>
+      </x:c>
+      <x:c r="I24" s="7" t="str">
+        <x:v>https://www.aosmd.com/sites/default/files/res/data_sheets/AO3400A.pdf</x:v>
+      </x:c>
       <x:c r="J24" s="7" t="str">
-        <x:v>FXL0530-4R7-M</x:v>
+        <x:v>AO3400A</x:v>
       </x:c>
       <x:c r="K24" s="7" t="str">
-        <x:v>cjiang</x:v>
+        <x:v>AOS</x:v>
       </x:c>
       <x:c r="L24" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M24" s="7" t="str">
-        <x:v>FXL0530 pads match the selected inductor; old Bourns purchasing link removed.</x:v>
-      </x:c>
+      <x:c r="M24" s="7"/>
     </x:row>
     <x:row r="25" ht="53" customHeight="1">
       <x:c r="A25" s="7" t="str">
-        <x:v>AO3400A</x:v>
+        <x:v>100K/0603/1%</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
-        <x:v>Q3,Q4,Q8,Q10</x:v>
+        <x:v>R1,R4,R7</x:v>
       </x:c>
       <x:c r="C25" s="7" t="str">
-        <x:v>RheoBoard:AO3400A</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D25" s="7" t="str">
-        <x:v>C20917</x:v>
+        <x:v>C25803</x:v>
       </x:c>
       <x:c r="E25" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F25" s="9" t="n">
-        <x:v>0.322</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="G25" s="9" t="n">
         <x:f>IF(ISNUMBER(F25),E25*F25,"")</x:f>
-        <x:v>1.288</x:v>
+        <x:v>0.042</x:v>
       </x:c>
       <x:c r="H25" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C20917.html</x:v>
-      </x:c>
-      <x:c r="I25" s="7" t="str">
-        <x:v>https://www.aosmd.com/sites/default/files/res/data_sheets/AO3400A.pdf</x:v>
-      </x:c>
+        <x:v>https://www.lcsc.com/product-detail/C25803.html</x:v>
+      </x:c>
+      <x:c r="I25" s="7"/>
       <x:c r="J25" s="7" t="str">
-        <x:v>AO3400A</x:v>
+        <x:v>0603WAF1003T5E</x:v>
       </x:c>
       <x:c r="K25" s="7" t="str">
-        <x:v>AOS</x:v>
+        <x:v>UNI-ROYAL</x:v>
       </x:c>
       <x:c r="L25" s="7" t="str">
         <x:v>SMT</x:v>
@@ -1383,33 +1382,33 @@
     </x:row>
     <x:row r="26" ht="53" customHeight="1">
       <x:c r="A26" s="7" t="str">
-        <x:v>100K/0603/1%</x:v>
+        <x:v>2K2/0603/1%</x:v>
       </x:c>
       <x:c r="B26" s="7" t="str">
-        <x:v>R1,R4,R7</x:v>
+        <x:v>R10</x:v>
       </x:c>
       <x:c r="C26" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D26" s="7" t="str">
-        <x:v>C25803</x:v>
+        <x:v>C4190</x:v>
       </x:c>
       <x:c r="E26" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F26" s="9" t="n">
         <x:v>0.014</x:v>
       </x:c>
       <x:c r="G26" s="9" t="n">
         <x:f>IF(ISNUMBER(F26),E26*F26,"")</x:f>
-        <x:v>0.042</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="H26" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25803.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C4190.html</x:v>
       </x:c>
       <x:c r="I26" s="7" t="str"/>
       <x:c r="J26" s="7" t="str">
-        <x:v>0603WAF1003T5E</x:v>
+        <x:v>0603WAF2201T5E</x:v>
       </x:c>
       <x:c r="K26" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1421,33 +1420,33 @@
     </x:row>
     <x:row r="27" ht="53" customHeight="1">
       <x:c r="A27" s="7" t="str">
-        <x:v>2K2/0603/1%</x:v>
+        <x:v>4K7/0603/1%</x:v>
       </x:c>
       <x:c r="B27" s="7" t="str">
-        <x:v>R10</x:v>
+        <x:v>R11, R15, R20, R82, R83</x:v>
       </x:c>
       <x:c r="C27" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D27" s="7" t="str">
-        <x:v>C4190</x:v>
+        <x:v>C23162</x:v>
       </x:c>
       <x:c r="E27" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F27" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="G27" s="9" t="n">
         <x:f>IF(ISNUMBER(F27),E27*F27,"")</x:f>
-        <x:v>0.014</x:v>
+        <x:v>0.005</x:v>
       </x:c>
       <x:c r="H27" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C4190.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C23162.html</x:v>
       </x:c>
       <x:c r="I27" s="7" t="str"/>
       <x:c r="J27" s="7" t="str">
-        <x:v>0603WAF2201T5E</x:v>
+        <x:v>0603WAF4701T5E</x:v>
       </x:c>
       <x:c r="K27" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1455,37 +1454,39 @@
       <x:c r="L27" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M27" s="7" t="str"/>
-    </x:row>
-    <x:row r="28" ht="53" customHeight="1">
+      <x:c r="M27" s="7" t="str">
+        <x:v>R82/R83 added as 4.7 kohm host SDA/SCL pullups; local R15/R20 retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="126" customHeight="1">
       <x:c r="A28" s="7" t="str">
-        <x:v>4K7/0603/1%</x:v>
+        <x:v>10K/0603/1%</x:v>
       </x:c>
       <x:c r="B28" s="7" t="str">
-        <x:v>R11, R15, R20, R82, R83</x:v>
+        <x:v>R13, R14, R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84</x:v>
       </x:c>
       <x:c r="C28" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D28" s="7" t="str">
-        <x:v>C23162</x:v>
+        <x:v>C25804</x:v>
       </x:c>
       <x:c r="E28" s="8" t="n">
-        <x:v>5</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F28" s="9" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="G28" s="9" t="n">
         <x:f>IF(ISNUMBER(F28),E28*F28,"")</x:f>
-        <x:v>0.005</x:v>
+        <x:v>0.266</x:v>
       </x:c>
       <x:c r="H28" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C23162.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C25804.html</x:v>
       </x:c>
       <x:c r="I28" s="7" t="str"/>
       <x:c r="J28" s="7" t="str">
-        <x:v>0603WAF4701T5E</x:v>
+        <x:v>0603WAF1002T5E</x:v>
       </x:c>
       <x:c r="K28" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1494,38 +1495,38 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M28" s="7" t="str">
-        <x:v>R82/R83 added as 4.7 kohm host SDA/SCL pullups; local R15/R20 retained.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="126" customHeight="1">
+        <x:v>R84 added from HOST_3V3 to GND for discharge (0.33 mA nominal).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="53" customHeight="1">
       <x:c r="A29" s="7" t="str">
-        <x:v>10K/0603/1%</x:v>
+        <x:v>1k/0603/1%</x:v>
       </x:c>
       <x:c r="B29" s="7" t="str">
-        <x:v>R13, R14, R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84</x:v>
+        <x:v>R24,R25,R26,R39,R40,R54,R59,R75</x:v>
       </x:c>
       <x:c r="C29" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D29" s="7" t="str">
-        <x:v>C25804</x:v>
+        <x:v>C21190</x:v>
       </x:c>
       <x:c r="E29" s="8" t="n">
-        <x:v>19</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F29" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="G29" s="9" t="n">
         <x:f>IF(ISNUMBER(F29),E29*F29,"")</x:f>
-        <x:v>0.266</x:v>
+        <x:v>0.008</x:v>
       </x:c>
       <x:c r="H29" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25804.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C21190.html</x:v>
       </x:c>
       <x:c r="I29" s="7" t="str"/>
       <x:c r="J29" s="7" t="str">
-        <x:v>0603WAF1002T5E</x:v>
+        <x:v>0603WAF1001T5E</x:v>
       </x:c>
       <x:c r="K29" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1533,39 +1534,37 @@
       <x:c r="L29" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M29" s="7" t="str">
-        <x:v>R84 added from HOST_3V3 to GND for discharge (0.33 mA nominal).</x:v>
-      </x:c>
+      <x:c r="M29" s="7"/>
     </x:row>
     <x:row r="30" ht="53" customHeight="1">
       <x:c r="A30" s="7" t="str">
-        <x:v>1k/0603/1%</x:v>
+        <x:v>100R/0603/1%</x:v>
       </x:c>
       <x:c r="B30" s="7" t="str">
-        <x:v>R24,R25,R26,R39,R40,R54,R59,R75</x:v>
+        <x:v>R35,R36,R42,R55</x:v>
       </x:c>
       <x:c r="C30" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D30" s="7" t="str">
-        <x:v>C21190</x:v>
+        <x:v>C22775</x:v>
       </x:c>
       <x:c r="E30" s="8" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F30" s="9" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="G30" s="9" t="n">
         <x:f>IF(ISNUMBER(F30),E30*F30,"")</x:f>
-        <x:v>0.008</x:v>
+        <x:v>0.056</x:v>
       </x:c>
       <x:c r="H30" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C21190.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C22775.html</x:v>
       </x:c>
       <x:c r="I30" s="7" t="str"/>
       <x:c r="J30" s="7" t="str">
-        <x:v>0603WAF1001T5E</x:v>
+        <x:v>0603WAF1000T5E</x:v>
       </x:c>
       <x:c r="K30" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1577,33 +1576,33 @@
     </x:row>
     <x:row r="31" ht="53" customHeight="1">
       <x:c r="A31" s="7" t="str">
-        <x:v>100R/0603/1%</x:v>
+        <x:v>330/0603/1%</x:v>
       </x:c>
       <x:c r="B31" s="7" t="str">
-        <x:v>R35,R36,R42,R55</x:v>
+        <x:v>R44,R77</x:v>
       </x:c>
       <x:c r="C31" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D31" s="7" t="str">
-        <x:v>C22775</x:v>
+        <x:v>C23138</x:v>
       </x:c>
       <x:c r="E31" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F31" s="9" t="n">
         <x:v>0.014</x:v>
       </x:c>
       <x:c r="G31" s="9" t="n">
         <x:f>IF(ISNUMBER(F31),E31*F31,"")</x:f>
-        <x:v>0.056</x:v>
+        <x:v>0.028</x:v>
       </x:c>
       <x:c r="H31" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22775.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C23138.html</x:v>
       </x:c>
       <x:c r="I31" s="7" t="str"/>
       <x:c r="J31" s="7" t="str">
-        <x:v>0603WAF1000T5E</x:v>
+        <x:v>0603WAF3300T5E</x:v>
       </x:c>
       <x:c r="K31" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1615,111 +1614,111 @@
     </x:row>
     <x:row r="32" ht="53" customHeight="1">
       <x:c r="A32" s="7" t="str">
-        <x:v>330/0603/1%</x:v>
+        <x:v>196k ±1%</x:v>
       </x:c>
       <x:c r="B32" s="7" t="str">
-        <x:v>R44,R77</x:v>
+        <x:v>R45</x:v>
       </x:c>
       <x:c r="C32" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D32" s="7" t="str">
-        <x:v>C23138</x:v>
+        <x:v>C4203218</x:v>
       </x:c>
       <x:c r="E32" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F32" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="G32" s="9" t="n">
         <x:f>IF(ISNUMBER(F32),E32*F32,"")</x:f>
-        <x:v>0.028</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="H32" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C23138.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C4203218.html</x:v>
       </x:c>
       <x:c r="I32" s="7" t="str"/>
       <x:c r="J32" s="7" t="str">
-        <x:v>0603WAF3300T5E</x:v>
+        <x:v>CRCW0603196KFKEA</x:v>
       </x:c>
       <x:c r="K32" s="7" t="str">
-        <x:v>UNI-ROYAL</x:v>
+        <x:v>VISHAY</x:v>
       </x:c>
       <x:c r="L32" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M32" s="7" t="str"/>
+      <x:c r="M32" s="7" t="str">
+        <x:v>Schematic corrected to the assembled 196k value; pump rail approximately 4.52 V.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="53" customHeight="1">
       <x:c r="A33" s="7" t="str">
-        <x:v>196k ±1%</x:v>
+        <x:v>30K/0603/1%</x:v>
       </x:c>
       <x:c r="B33" s="7" t="str">
-        <x:v>R45</x:v>
+        <x:v>R46,R74,R76</x:v>
       </x:c>
       <x:c r="C33" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D33" s="7" t="str">
-        <x:v>C4203218</x:v>
+        <x:v>C22984</x:v>
       </x:c>
       <x:c r="E33" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F33" s="9" t="n">
-        <x:v>0.02</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="G33" s="9" t="n">
         <x:f>IF(ISNUMBER(F33),E33*F33,"")</x:f>
-        <x:v>0.02</x:v>
+        <x:v>0.042</x:v>
       </x:c>
       <x:c r="H33" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C4203218.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C22984.html</x:v>
       </x:c>
       <x:c r="I33" s="7" t="str"/>
       <x:c r="J33" s="7" t="str">
-        <x:v>CRCW0603196KFKEA</x:v>
+        <x:v>0603WAF3002T5E</x:v>
       </x:c>
       <x:c r="K33" s="7" t="str">
-        <x:v>VISHAY</x:v>
+        <x:v>UNI-ROYAL</x:v>
       </x:c>
       <x:c r="L33" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M33" s="7" t="str">
-        <x:v>Schematic corrected to the assembled 196k value; pump rail approximately 4.52 V.</x:v>
-      </x:c>
+      <x:c r="M33" s="7"/>
     </x:row>
     <x:row r="34" ht="53" customHeight="1">
       <x:c r="A34" s="7" t="str">
-        <x:v>30K/0603/1%</x:v>
+        <x:v>270K/0603/1%</x:v>
       </x:c>
       <x:c r="B34" s="7" t="str">
-        <x:v>R46,R74,R76</x:v>
+        <x:v>R60</x:v>
       </x:c>
       <x:c r="C34" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D34" s="7" t="str">
-        <x:v>C22984</x:v>
+        <x:v>C22965</x:v>
       </x:c>
       <x:c r="E34" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F34" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="G34" s="9" t="n">
         <x:f>IF(ISNUMBER(F34),E34*F34,"")</x:f>
-        <x:v>0.042</x:v>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="H34" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22984.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C22965.html</x:v>
       </x:c>
       <x:c r="I34" s="7" t="str"/>
       <x:c r="J34" s="7" t="str">
-        <x:v>0603WAF3002T5E</x:v>
+        <x:v>0603WAF2703T5E</x:v>
       </x:c>
       <x:c r="K34" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1731,36 +1730,36 @@
     </x:row>
     <x:row r="35" ht="53" customHeight="1">
       <x:c r="A35" s="7" t="str">
-        <x:v>270K/0603/1%</x:v>
+        <x:v>135k ±0.1%</x:v>
       </x:c>
       <x:c r="B35" s="7" t="str">
-        <x:v>R60</x:v>
+        <x:v>R61</x:v>
       </x:c>
       <x:c r="C35" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D35" s="7" t="str">
-        <x:v>C22965</x:v>
+        <x:v>C861113</x:v>
       </x:c>
       <x:c r="E35" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F35" s="9" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.06</x:v>
       </x:c>
       <x:c r="G35" s="9" t="n">
         <x:f>IF(ISNUMBER(F35),E35*F35,"")</x:f>
-        <x:v>0.001</x:v>
+        <x:v>0.06</x:v>
       </x:c>
       <x:c r="H35" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22965.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C861113.html</x:v>
       </x:c>
       <x:c r="I35" s="7" t="str"/>
       <x:c r="J35" s="7" t="str">
-        <x:v>0603WAF2703T5E</x:v>
+        <x:v>RT0603BRD07135KL</x:v>
       </x:c>
       <x:c r="K35" s="7" t="str">
-        <x:v>UNI-ROYAL</x:v>
+        <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="L35" s="7" t="str">
         <x:v>SMT</x:v>
@@ -1769,71 +1768,70 @@
     </x:row>
     <x:row r="36" ht="53" customHeight="1">
       <x:c r="A36" s="7" t="str">
-        <x:v>135k ±0.1%</x:v>
+        <x:v>549R ±1%</x:v>
       </x:c>
       <x:c r="B36" s="7" t="str">
-        <x:v>R61</x:v>
+        <x:v>R73</x:v>
       </x:c>
       <x:c r="C36" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D36" s="7" t="str">
-        <x:v>C861113</x:v>
+        <x:v>C23079</x:v>
       </x:c>
       <x:c r="E36" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F36" s="9" t="n">
-        <x:v>0.06</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="G36" s="9" t="n">
         <x:f>IF(ISNUMBER(F36),E36*F36,"")</x:f>
-        <x:v>0.06</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="H36" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C861113.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C23079.html</x:v>
       </x:c>
       <x:c r="I36" s="7" t="str"/>
       <x:c r="J36" s="7" t="str">
-        <x:v>RT0603BRD07135KL</x:v>
+        <x:v>0603WAF5490T5E</x:v>
       </x:c>
       <x:c r="K36" s="7" t="str">
-        <x:v>YAGEO</x:v>
+        <x:v>UNI-ROYAL</x:v>
       </x:c>
       <x:c r="L36" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M36" s="7" t="str"/>
+      <x:c r="M36" s="7" t="str">
+        <x:v>Schematic corrected to the assembled 549 ohm value.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="53" customHeight="1">
       <x:c r="A37" s="7" t="str">
-        <x:v>549R ±1%</x:v>
+        <x:v>680k ±1%</x:v>
       </x:c>
       <x:c r="B37" s="7" t="str">
-        <x:v>R73</x:v>
+        <x:v>R78</x:v>
       </x:c>
       <x:c r="C37" s="7" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D37" s="7" t="str">
-        <x:v>C23079</x:v>
+        <x:v>C25822</x:v>
       </x:c>
       <x:c r="E37" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F37" s="9" t="n">
-        <x:v>0.014</x:v>
-      </x:c>
-      <x:c r="G37" s="9" t="n">
+      <x:c r="F37" s="10"/>
+      <x:c r="G37" s="9" t="str">
         <x:f>IF(ISNUMBER(F37),E37*F37,"")</x:f>
-        <x:v>0.014</x:v>
       </x:c>
       <x:c r="H37" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C23079.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C25822.html</x:v>
       </x:c>
       <x:c r="I37" s="7" t="str"/>
       <x:c r="J37" s="7" t="str">
-        <x:v>0603WAF5490T5E</x:v>
+        <x:v>0603WAF6803T5E</x:v>
       </x:c>
       <x:c r="K37" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1841,36 +1839,37 @@
       <x:c r="L37" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M37" s="7" t="str">
-        <x:v>Schematic corrected to the assembled 549 ohm value.</x:v>
-      </x:c>
+      <x:c r="M37" s="7"/>
     </x:row>
     <x:row r="38" ht="53" customHeight="1">
       <x:c r="A38" s="7" t="str">
-        <x:v>680k ±1%</x:v>
+        <x:v>100K/0603/1%</x:v>
       </x:c>
       <x:c r="B38" s="7" t="str">
-        <x:v>R78</x:v>
+        <x:v>R79</x:v>
       </x:c>
       <x:c r="C38" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D38" s="7" t="str">
-        <x:v>C25822</x:v>
+        <x:v>C25803</x:v>
       </x:c>
       <x:c r="E38" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F38" s="10"/>
-      <x:c r="G38" s="9" t="str">
+      <x:c r="F38" s="9" t="n">
+        <x:v>0.014</x:v>
+      </x:c>
+      <x:c r="G38" s="9" t="n">
         <x:f>IF(ISNUMBER(F38),E38*F38,"")</x:f>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="H38" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25822.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C25803.html</x:v>
       </x:c>
       <x:c r="I38" s="7" t="str"/>
       <x:c r="J38" s="7" t="str">
-        <x:v>0603WAF6803T5E</x:v>
+        <x:v>0603WAF1003T5E</x:v>
       </x:c>
       <x:c r="K38" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1882,33 +1881,30 @@
     </x:row>
     <x:row r="39" ht="53" customHeight="1">
       <x:c r="A39" s="7" t="str">
-        <x:v>100K/0603/1%</x:v>
+        <x:v>390k ±1%</x:v>
       </x:c>
       <x:c r="B39" s="7" t="str">
-        <x:v>R79</x:v>
+        <x:v>R80</x:v>
       </x:c>
       <x:c r="C39" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D39" s="7" t="str">
-        <x:v>C25803</x:v>
+        <x:v>C2759410</x:v>
       </x:c>
       <x:c r="E39" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F39" s="9" t="n">
-        <x:v>0.014</x:v>
-      </x:c>
-      <x:c r="G39" s="9" t="n">
+      <x:c r="F39" s="10"/>
+      <x:c r="G39" s="9" t="str">
         <x:f>IF(ISNUMBER(F39),E39*F39,"")</x:f>
-        <x:v>0.014</x:v>
       </x:c>
       <x:c r="H39" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25803.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C2759410.html</x:v>
       </x:c>
       <x:c r="I39" s="7" t="str"/>
       <x:c r="J39" s="7" t="str">
-        <x:v>0603WAF1003T5E</x:v>
+        <x:v>HP03W5F3903T5E</x:v>
       </x:c>
       <x:c r="K39" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1920,16 +1916,16 @@
     </x:row>
     <x:row r="40" ht="53" customHeight="1">
       <x:c r="A40" s="7" t="str">
-        <x:v>390k ±1%</x:v>
+        <x:v>1.65k ±1%</x:v>
       </x:c>
       <x:c r="B40" s="7" t="str">
-        <x:v>R80</x:v>
+        <x:v>R81</x:v>
       </x:c>
       <x:c r="C40" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D40" s="7" t="str">
-        <x:v>C2759410</x:v>
+        <x:v>C22845</x:v>
       </x:c>
       <x:c r="E40" s="8" t="n">
         <x:v>1</x:v>
@@ -1939,11 +1935,11 @@
         <x:f>IF(ISNUMBER(F40),E40*F40,"")</x:f>
       </x:c>
       <x:c r="H40" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C2759410.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C22845.html</x:v>
       </x:c>
       <x:c r="I40" s="7" t="str"/>
       <x:c r="J40" s="7" t="str">
-        <x:v>HP03W5F3903T5E</x:v>
+        <x:v>0603WAF1651T5E</x:v>
       </x:c>
       <x:c r="K40" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1955,33 +1951,36 @@
     </x:row>
     <x:row r="41" ht="53" customHeight="1">
       <x:c r="A41" s="7" t="str">
-        <x:v>1.65k ±1%</x:v>
+        <x:v>TL3301NF160QG/P010515</x:v>
       </x:c>
       <x:c r="B41" s="7" t="str">
-        <x:v>R81</x:v>
+        <x:v>SW1,SW2,SW3,SW4</x:v>
       </x:c>
       <x:c r="C41" s="7" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
+        <x:v>RheoBoard:Tactile_Switch_4pad</x:v>
       </x:c>
       <x:c r="D41" s="7" t="str">
-        <x:v>C22845</x:v>
+        <x:v>C273527</x:v>
       </x:c>
       <x:c r="E41" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F41" s="10"/>
-      <x:c r="G41" s="9" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F41" s="9" t="n">
+        <x:v>0.183</x:v>
+      </x:c>
+      <x:c r="G41" s="9" t="n">
         <x:f>IF(ISNUMBER(F41),E41*F41,"")</x:f>
+        <x:v>0.732</x:v>
       </x:c>
       <x:c r="H41" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22845.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C273527.html</x:v>
       </x:c>
       <x:c r="I41" s="7" t="str"/>
       <x:c r="J41" s="7" t="str">
-        <x:v>0603WAF1651T5E</x:v>
+        <x:v>TL3301NF160QG/P010515</x:v>
       </x:c>
       <x:c r="K41" s="7" t="str">
-        <x:v>UNI-ROYAL</x:v>
+        <x:v>E-Switch</x:v>
       </x:c>
       <x:c r="L41" s="7" t="str">
         <x:v>SMT</x:v>
@@ -1990,36 +1989,38 @@
     </x:row>
     <x:row r="42" ht="53" customHeight="1">
       <x:c r="A42" s="7" t="str">
-        <x:v>TL3301NF160QG/P010515</x:v>
+        <x:v>TPS563203DRLR</x:v>
       </x:c>
       <x:c r="B42" s="7" t="str">
-        <x:v>SW1,SW2,SW3,SW4</x:v>
+        <x:v>U1,U2,U3</x:v>
       </x:c>
       <x:c r="C42" s="7" t="str">
-        <x:v>RheoBoard:Tactile_Switch_4pad</x:v>
+        <x:v>RheoBoard:TPS563203DRLR</x:v>
       </x:c>
       <x:c r="D42" s="7" t="str">
-        <x:v>C273527</x:v>
+        <x:v>C22445512</x:v>
       </x:c>
       <x:c r="E42" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F42" s="9" t="n">
-        <x:v>0.183</x:v>
+        <x:v>0.225</x:v>
       </x:c>
       <x:c r="G42" s="9" t="n">
         <x:f>IF(ISNUMBER(F42),E42*F42,"")</x:f>
-        <x:v>0.732</x:v>
+        <x:v>0.675</x:v>
       </x:c>
       <x:c r="H42" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C273527.html</x:v>
-      </x:c>
-      <x:c r="I42" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C22445512.html</x:v>
+      </x:c>
+      <x:c r="I42" s="7" t="str">
+        <x:v>https://www.ti.com/lit/gpn/tps563203</x:v>
+      </x:c>
       <x:c r="J42" s="7" t="str">
-        <x:v>TL3301NF160QG/P010515</x:v>
+        <x:v>TPS563203DRLR</x:v>
       </x:c>
       <x:c r="K42" s="7" t="str">
-        <x:v>E-Switch</x:v>
+        <x:v>TI</x:v>
       </x:c>
       <x:c r="L42" s="7" t="str">
         <x:v>SMT</x:v>
@@ -2028,35 +2029,35 @@
     </x:row>
     <x:row r="43" ht="53" customHeight="1">
       <x:c r="A43" s="7" t="str">
-        <x:v>TPS563203DRLR</x:v>
+        <x:v>TCA9534APWR</x:v>
       </x:c>
       <x:c r="B43" s="7" t="str">
-        <x:v>U1,U2,U3</x:v>
+        <x:v>U4</x:v>
       </x:c>
       <x:c r="C43" s="7" t="str">
-        <x:v>RheoBoard:TPS563203DRLR</x:v>
+        <x:v>RheoBoard:TCA9534APWR</x:v>
       </x:c>
       <x:c r="D43" s="7" t="str">
-        <x:v>C22445512</x:v>
+        <x:v>C206010</x:v>
       </x:c>
       <x:c r="E43" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F43" s="9" t="n">
-        <x:v>0.225</x:v>
+        <x:v>1.27</x:v>
       </x:c>
       <x:c r="G43" s="9" t="n">
         <x:f>IF(ISNUMBER(F43),E43*F43,"")</x:f>
-        <x:v>0.675</x:v>
+        <x:v>1.27</x:v>
       </x:c>
       <x:c r="H43" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22445512.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C206010.html</x:v>
       </x:c>
       <x:c r="I43" s="7" t="str">
-        <x:v>https://www.ti.com/lit/gpn/tps563203</x:v>
+        <x:v>https://www.ti.com/lit/ds/symlink/tca9534a.pdf</x:v>
       </x:c>
       <x:c r="J43" s="7" t="str">
-        <x:v>TPS563203DRLR</x:v>
+        <x:v>TCA9534APWR</x:v>
       </x:c>
       <x:c r="K43" s="7" t="str">
         <x:v>TI</x:v>
@@ -2066,80 +2067,80 @@
       </x:c>
       <x:c r="M43" s="7" t="str"/>
     </x:row>
-    <x:row r="44" ht="53" customHeight="1">
+    <x:row r="44" ht="68" customHeight="1">
       <x:c r="A44" s="7" t="str">
-        <x:v>TCA9534APWR</x:v>
+        <x:v>MPRLS0025PA00001A</x:v>
       </x:c>
       <x:c r="B44" s="7" t="str">
-        <x:v>U4</x:v>
+        <x:v>U5</x:v>
       </x:c>
       <x:c r="C44" s="7" t="str">
-        <x:v>RheoBoard:TCA9534APWR</x:v>
+        <x:v>RheoBoard:MPRLS0025PA00001A</x:v>
       </x:c>
       <x:c r="D44" s="7" t="str">
-        <x:v>C206010</x:v>
+        <x:v>C3257154</x:v>
       </x:c>
       <x:c r="E44" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F44" s="9" t="n">
-        <x:v>1.27</x:v>
+        <x:v>15.93</x:v>
       </x:c>
       <x:c r="G44" s="9" t="n">
         <x:f>IF(ISNUMBER(F44),E44*F44,"")</x:f>
-        <x:v>1.27</x:v>
+        <x:v>15.93</x:v>
       </x:c>
       <x:c r="H44" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C206010.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C3257154.html</x:v>
       </x:c>
       <x:c r="I44" s="7" t="str">
-        <x:v>https://www.ti.com/lit/ds/symlink/tca9534a.pdf</x:v>
+        <x:v>https://automation.honeywell.com/content/dam/honeywell-edam/sps/ast/en-us/campaigns/pressure-sensors/documents/sps-siot-mpr-series-datasheet-32332628-ciid-172626.pdf</x:v>
       </x:c>
       <x:c r="J44" s="7" t="str">
-        <x:v>TCA9534APWR</x:v>
+        <x:v>MPRLS0025PA00001A</x:v>
       </x:c>
       <x:c r="K44" s="7" t="str">
-        <x:v>TI</x:v>
+        <x:v>Honeywell</x:v>
       </x:c>
       <x:c r="L44" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M44" s="7" t="str"/>
     </x:row>
-    <x:row r="45" ht="68" customHeight="1">
+    <x:row r="45" ht="53" customHeight="1">
       <x:c r="A45" s="7" t="str">
-        <x:v>MPRLS0025PA00001A</x:v>
+        <x:v>PCA9685PW,118</x:v>
       </x:c>
       <x:c r="B45" s="7" t="str">
-        <x:v>U5</x:v>
+        <x:v>U7</x:v>
       </x:c>
       <x:c r="C45" s="7" t="str">
-        <x:v>RheoBoard:MPRLS0025PA00001A</x:v>
+        <x:v>RheoBoard:PCA9685</x:v>
       </x:c>
       <x:c r="D45" s="7" t="str">
-        <x:v>C3257154</x:v>
+        <x:v>C2678753</x:v>
       </x:c>
       <x:c r="E45" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F45" s="9" t="n">
-        <x:v>15.93</x:v>
+        <x:v>3.445</x:v>
       </x:c>
       <x:c r="G45" s="9" t="n">
         <x:f>IF(ISNUMBER(F45),E45*F45,"")</x:f>
-        <x:v>15.93</x:v>
+        <x:v>3.445</x:v>
       </x:c>
       <x:c r="H45" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C3257154.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C2678753.html</x:v>
       </x:c>
       <x:c r="I45" s="7" t="str">
-        <x:v>https://automation.honeywell.com/content/dam/honeywell-edam/sps/ast/en-us/campaigns/pressure-sensors/documents/sps-siot-mpr-series-datasheet-32332628-ciid-172626.pdf</x:v>
+        <x:v>https://www.nxp.com/docs/en/data-sheet/PCA9685.pdf</x:v>
       </x:c>
       <x:c r="J45" s="7" t="str">
-        <x:v>MPRLS0025PA00001A</x:v>
+        <x:v>PCA9685PW,118</x:v>
       </x:c>
       <x:c r="K45" s="7" t="str">
-        <x:v>Honeywell</x:v>
+        <x:v>NXP</x:v>
       </x:c>
       <x:c r="L45" s="7" t="str">
         <x:v>SMT</x:v>
@@ -2147,134 +2148,133 @@
       <x:c r="M45" s="7" t="str"/>
     </x:row>
     <x:row r="46" ht="53" customHeight="1">
-      <x:c r="A46" s="7" t="str">
-        <x:v>PCA9685PW,118</x:v>
-      </x:c>
-      <x:c r="B46" s="7" t="str">
-        <x:v>U7</x:v>
-      </x:c>
-      <x:c r="C46" s="7" t="str">
-        <x:v>RheoBoard:PCA9685</x:v>
-      </x:c>
-      <x:c r="D46" s="7" t="str">
-        <x:v>C2678753</x:v>
-      </x:c>
-      <x:c r="E46" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F46" s="9" t="n">
-        <x:v>3.445</x:v>
-      </x:c>
-      <x:c r="G46" s="9" t="n">
+      <x:c r="A46" s="11" t="str">
+        <x:v>ZR370-02PM / 4.5V / 2.5 LPM / ~500 mA</x:v>
+      </x:c>
+      <x:c r="B46" s="11" t="str">
+        <x:v>U8,U11</x:v>
+      </x:c>
+      <x:c r="C46" s="11" t="str">
+        <x:v>RheoBoard:PUMP</x:v>
+      </x:c>
+      <x:c r="D46" s="11"/>
+      <x:c r="E46" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F46" s="13" t="n">
+        <x:v>7.16</x:v>
+      </x:c>
+      <x:c r="G46" s="13" t="n">
         <x:f>IF(ISNUMBER(F46),E46*F46,"")</x:f>
-        <x:v>3.445</x:v>
-      </x:c>
-      <x:c r="H46" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C2678753.html</x:v>
-      </x:c>
-      <x:c r="I46" s="7" t="str">
-        <x:v>https://www.nxp.com/docs/en/data-sheet/PCA9685.pdf</x:v>
-      </x:c>
-      <x:c r="J46" s="7" t="str">
-        <x:v>PCA9685PW,118</x:v>
-      </x:c>
-      <x:c r="K46" s="7" t="str">
-        <x:v>NXP</x:v>
-      </x:c>
-      <x:c r="L46" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M46" s="7" t="str"/>
+        <x:v>14.32</x:v>
+      </x:c>
+      <x:c r="H46" s="11" t="str">
+        <x:v>https://www.adafruit.com/product/4699</x:v>
+      </x:c>
+      <x:c r="I46" s="11"/>
+      <x:c r="J46" s="11" t="str">
+        <x:v>ZR370-02PM</x:v>
+      </x:c>
+      <x:c r="K46" s="11" t="str">
+        <x:v>Supplier-specified</x:v>
+      </x:c>
+      <x:c r="L46" s="11" t="str">
+        <x:v>Manual pump fitting</x:v>
+      </x:c>
+      <x:c r="M46" s="11" t="str">
+        <x:v>Existing pump retained for intermittent use. Manual fitting; provide mechanical support.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="53" customHeight="1">
       <x:c r="A47" s="11" t="str">
-        <x:v>ZR370-02PM / 4.5V / 2.5 LPM / ~500 mA</x:v>
+        <x:v>JST XH 2-pin 2.50mm</x:v>
       </x:c>
       <x:c r="B47" s="11" t="str">
-        <x:v>U8,U11</x:v>
+        <x:v>U9,U10</x:v>
       </x:c>
       <x:c r="C47" s="11" t="str">
-        <x:v>RheoBoard:PUMP</x:v>
-      </x:c>
-      <x:c r="D47" s="11" t="str"/>
+        <x:v>RheoBoard:VALVE_v105</x:v>
+      </x:c>
+      <x:c r="D47" s="11" t="str">
+        <x:v>C158012</x:v>
+      </x:c>
       <x:c r="E47" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F47" s="13" t="n">
-        <x:v>7.16</x:v>
-      </x:c>
-      <x:c r="G47" s="13" t="n">
+      <x:c r="F47" s="10"/>
+      <x:c r="G47" s="13" t="str">
         <x:f>IF(ISNUMBER(F47),E47*F47,"")</x:f>
-        <x:v>14.32</x:v>
       </x:c>
       <x:c r="H47" s="11" t="str">
-        <x:v>https://www.adafruit.com/product/4699</x:v>
-      </x:c>
-      <x:c r="I47" s="11" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C158012.html</x:v>
+      </x:c>
+      <x:c r="I47" s="11" t="str">
+        <x:v>https://www.jst-mfg.com/product/pdf/eng/eXH.pdf</x:v>
+      </x:c>
       <x:c r="J47" s="11" t="str">
-        <x:v>ZR370-02PM</x:v>
+        <x:v>B2B-XH-A(LF)(SN)</x:v>
       </x:c>
       <x:c r="K47" s="11" t="str">
-        <x:v>Supplier-specified</x:v>
+        <x:v>JST</x:v>
       </x:c>
       <x:c r="L47" s="11" t="str">
-        <x:v>Manual pump fitting</x:v>
+        <x:v>Manual THT</x:v>
       </x:c>
       <x:c r="M47" s="11" t="str">
-        <x:v>Existing pump retained for intermittent use. Manual fitting; provide mechanical support.</x:v>
+        <x:v>Fitted JST XH header only. External valve is listed on Manual accessories. Manual through-hole assembly.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="53" customHeight="1">
-      <x:c r="A48" s="11" t="str">
-        <x:v>JST XH 2-pin 2.50mm</x:v>
-      </x:c>
-      <x:c r="B48" s="11" t="str">
-        <x:v>U9,U10</x:v>
-      </x:c>
-      <x:c r="C48" s="11" t="str">
-        <x:v>RheoBoard:VALVE_v105</x:v>
-      </x:c>
-      <x:c r="D48" s="11" t="str">
-        <x:v>C158012</x:v>
-      </x:c>
-      <x:c r="E48" s="12" t="n">
-        <x:v>2</x:v>
+      <x:c r="A48" s="7" t="str">
+        <x:v>TPS259472ARPWR</x:v>
+      </x:c>
+      <x:c r="B48" s="7" t="str">
+        <x:v>U12</x:v>
+      </x:c>
+      <x:c r="C48" s="7" t="str">
+        <x:v>RheoBoard:TI_RPW0010A_VQFN-HR_2x2mm</x:v>
+      </x:c>
+      <x:c r="D48" s="7" t="str">
+        <x:v>C3662789</x:v>
+      </x:c>
+      <x:c r="E48" s="8" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F48" s="10"/>
-      <x:c r="G48" s="13" t="str">
+      <x:c r="G48" s="9" t="str">
         <x:f>IF(ISNUMBER(F48),E48*F48,"")</x:f>
       </x:c>
-      <x:c r="H48" s="11" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C158012.html</x:v>
-      </x:c>
-      <x:c r="I48" s="11" t="str">
-        <x:v>https://www.jst-mfg.com/product/pdf/eng/eXH.pdf</x:v>
-      </x:c>
-      <x:c r="J48" s="11" t="str">
-        <x:v>B2B-XH-A(LF)(SN)</x:v>
-      </x:c>
-      <x:c r="K48" s="11" t="str">
-        <x:v>JST</x:v>
-      </x:c>
-      <x:c r="L48" s="11" t="str">
-        <x:v>Manual THT</x:v>
-      </x:c>
-      <x:c r="M48" s="11" t="str">
-        <x:v>Fitted JST XH header only. External valve is listed on Manual accessories. Manual through-hole assembly.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="53" customHeight="1">
+      <x:c r="H48" s="7" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C3662789.html</x:v>
+      </x:c>
+      <x:c r="I48" s="7" t="str">
+        <x:v>https://www.ti.com/lit/ds/symlink/tps25947.pdf</x:v>
+      </x:c>
+      <x:c r="J48" s="7" t="str">
+        <x:v>TPS259472ARPWR</x:v>
+      </x:c>
+      <x:c r="K48" s="7" t="str">
+        <x:v>Texas Instruments</x:v>
+      </x:c>
+      <x:c r="L48" s="7" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M48" s="7" t="str">
+        <x:v>New auto-retry input eFuse; TI RPW0010A HotRod footprint, approximately 2 A limit / 13.8 V clamp.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="112" customHeight="1">
       <x:c r="A49" s="7" t="str">
-        <x:v>TPS259472ARPWR</x:v>
+        <x:v>TCA9517ADGKR</x:v>
       </x:c>
       <x:c r="B49" s="7" t="str">
-        <x:v>U12</x:v>
+        <x:v>U13</x:v>
       </x:c>
       <x:c r="C49" s="7" t="str">
-        <x:v>RheoBoard:TI_RPW0010A_VQFN-HR_2x2mm</x:v>
+        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
       </x:c>
       <x:c r="D49" s="7" t="str">
-        <x:v>C3662789</x:v>
+        <x:v>C201698</x:v>
       </x:c>
       <x:c r="E49" s="8" t="n">
         <x:v>1</x:v>
@@ -2284,13 +2284,13 @@
         <x:f>IF(ISNUMBER(F49),E49*F49,"")</x:f>
       </x:c>
       <x:c r="H49" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C3662789.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C201698.html</x:v>
       </x:c>
       <x:c r="I49" s="7" t="str">
-        <x:v>https://www.ti.com/lit/ds/symlink/tps25947.pdf</x:v>
+        <x:v>https://www.ti.com/lit/ds/symlink/tca9517a.pdf</x:v>
       </x:c>
       <x:c r="J49" s="7" t="str">
-        <x:v>TPS259472ARPWR</x:v>
+        <x:v>TCA9517ADGKR</x:v>
       </x:c>
       <x:c r="K49" s="7" t="str">
         <x:v>Texas Instruments</x:v>
@@ -2299,66 +2299,42 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M49" s="7" t="str">
-        <x:v>New auto-retry input eFuse; TI RPW0010A HotRod footprint, approximately 2 A limit / 13.8 V clamp.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="112" customHeight="1">
-      <x:c r="A50" s="7" t="str">
-        <x:v>TCA9517ADGKR</x:v>
-      </x:c>
-      <x:c r="B50" s="7" t="str">
-        <x:v>U13</x:v>
-      </x:c>
-      <x:c r="C50" s="7" t="str">
-        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
-      </x:c>
-      <x:c r="D50" s="7" t="str">
-        <x:v>C201698</x:v>
-      </x:c>
-      <x:c r="E50" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F50" s="10"/>
-      <x:c r="G50" s="9" t="str">
-        <x:f>IF(ISNUMBER(F50),E50*F50,"")</x:f>
-      </x:c>
-      <x:c r="H50" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C201698.html</x:v>
-      </x:c>
-      <x:c r="I50" s="7" t="str">
-        <x:v>https://www.ti.com/lit/ds/symlink/tca9517a.pdf</x:v>
-      </x:c>
-      <x:c r="J50" s="7" t="str">
-        <x:v>TCA9517ADGKR</x:v>
-      </x:c>
-      <x:c r="K50" s="7" t="str">
-        <x:v>Texas Instruments</x:v>
-      </x:c>
-      <x:c r="L50" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M50" s="7" t="str">
         <x:v>Qwiic master interface: local bus on A, host on B. EN and VCCB use HOST_3V3; separate supplies, common GND. TI DGK land pattern: 1.4 x 0.45 mm pads, 0.65 mm pitch, 4.4 mm row-center span.</x:v>
       </x:c>
     </x:row>
+    <x:row r="50" ht="30" customHeight="1">
+      <x:c r="A50" s="14" t="str">
+        <x:v>Total fitted parts / incomplete priced subtotal</x:v>
+      </x:c>
+      <x:c r="B50" s="14"/>
+      <x:c r="C50" s="14"/>
+      <x:c r="D50" s="14"/>
+      <x:c r="E50" s="14" t="n">
+        <x:f>SUM(E2:E49)</x:f>
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="F50" s="14" t="str">
+        <x:v>Incomplete estimate</x:v>
+      </x:c>
+      <x:c r="G50" s="15" t="n">
+        <x:f>SUM(G2:G49)</x:f>
+        <x:v>55.617999999999995</x:v>
+      </x:c>
+      <x:c r="H50"/>
+      <x:c r="I50"/>
+      <x:c r="J50"/>
+      <x:c r="K50"/>
+      <x:c r="L50"/>
+      <x:c r="M50"/>
+    </x:row>
     <x:row r="51" ht="30" customHeight="1">
-      <x:c r="A51" s="14" t="str">
-        <x:v>Total fitted parts / incomplete priced subtotal</x:v>
-      </x:c>
-      <x:c r="B51" s="14"/>
-      <x:c r="C51" s="14"/>
-      <x:c r="D51" s="14"/>
-      <x:c r="E51" s="14" t="n">
-        <x:f>SUM(E2:E50)</x:f>
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="F51" s="14" t="str">
-        <x:v>Incomplete estimate</x:v>
-      </x:c>
-      <x:c r="G51" s="15" t="n">
-        <x:f>SUM(G2:G50)</x:f>
-        <x:v>55.617999999999995</x:v>
-      </x:c>
+      <x:c r="A51"/>
+      <x:c r="B51"/>
+      <x:c r="C51"/>
+      <x:c r="D51"/>
+      <x:c r="E51"/>
+      <x:c r="F51"/>
+      <x:c r="G51"/>
     </x:row>
     <x:row r="53" ht="34" customHeight="1">
       <x:c r="A53" s="16" t="str">
@@ -2384,7 +2360,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2396359dc474a04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7b14771b7ab43eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2450,146 +2426,118 @@
     </x:row>
     <x:row r="3" ht="154" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Local service connector housing</x:v>
+        <x:v>Eight-channel I2C multiplexer</x:v>
       </x:c>
       <x:c r="B3" s="3" t="str">
-        <x:v>Optional: 1 per board</x:v>
+        <x:v>1 per system, up to 8 boards</x:v>
       </x:c>
       <x:c r="C3" s="3" t="str">
-        <x:v>JST</x:v>
+        <x:v>Adafruit / Texas Instruments</x:v>
       </x:c>
       <x:c r="D3" s="3" t="str">
-        <x:v>EHR-3</x:v>
+        <x:v>Product 2717 / TCA9548A</x:v>
       </x:c>
       <x:c r="E3" s="3" t="str">
-        <x:v>J18 local-bus service mating housing</x:v>
+        <x:v>One independent RheoBoard per mux channel</x:v>
       </x:c>
       <x:c r="F3" s="3" t="str">
-        <x:v>https://www.jst-mfg.com/product/pdf/eng/eEH.pdf</x:v>
+        <x:v>https://www.adafruit.com/product/2717</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>GND/SDA/SCL only; bypasses U13. The standard Qwiic master cable connects to J9.</x:v>
+        <x:v>Address 0x71; exactly one channel enabled. Master 3.3 V/GND/channel SDA/SCL to J9; local rails stay separate. Product 2717 needs a Qwiic adapter harness. No upstream B-side repeater/rise-time accelerator. Total host pullup current &lt;=3 mA; selected-branch effective pullups &gt;=2.2 kohm including parallel module resistors/tolerance. Verify actual wiring and rise times.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="154" customHeight="1">
       <x:c r="A4" s="3" t="str">
-        <x:v>Local service connector contacts</x:v>
+        <x:v>12 V power supply</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
-        <x:v>Optional: 3 per housing</x:v>
+        <x:v>1 supply per board or budgeted distribution</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
-        <x:v>JST</x:v>
+        <x:v>To be selected</x:v>
       </x:c>
       <x:c r="D4" s="3" t="str">
-        <x:v>SEH-001T-P0.6</x:v>
+        <x:v>Regulated 12 V, center-positive, 5.5 × 2.5 mm plug</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str">
-        <x:v>Contacts for optional J18 service harness</x:v>
+        <x:v>Board input power</x:v>
       </x:c>
       <x:c r="F4" s="3" t="str">
-        <x:v>https://www.jst-mfg.com/product/pdf/eng/eEH.pdf</x:v>
+        <x:v>https://www.sameskydevices.com/product/resource/pj-082bh.pdf</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>Select wire size and crimping method to JST specification.</x:v>
+        <x:v>12 V, 2 A starting rating for specified loads; validate actual startup and simultaneous-load current. Board input fuse 2 A; do not increase load budget just because supply is larger.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="154" customHeight="1">
       <x:c r="A5" s="3" t="str">
-        <x:v>Eight-channel I2C multiplexer</x:v>
+        <x:v>Qwiic master</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>1 per system, up to 8 boards</x:v>
+        <x:v>1 per system</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
-        <x:v>Adafruit / Texas Instruments</x:v>
+        <x:v>SparkFun</x:v>
       </x:c>
       <x:c r="D5" s="3" t="str">
-        <x:v>Product 2717 / TCA9548A</x:v>
+        <x:v>WRL-15663 (ESP32 Thing Plus, Micro-B)</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
-        <x:v>One independent RheoBoard per mux channel</x:v>
+        <x:v>USB/battery-powered I2C master; GPIO23 SDA, GPIO22 SCL</x:v>
       </x:c>
       <x:c r="F5" s="3" t="str">
-        <x:v>https://www.adafruit.com/product/2717</x:v>
+        <x:v>https://cdn.sparkfun.com/assets/6/d/c/6/c/ESP32_Thing_Plus_Schematic.pdf</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
-        <x:v>Address 0x71; exactly one channel enabled. Master 3.3 V/GND/channel SDA/SCL to J9; local rails stay separate. Product 2717 needs a Qwiic adapter harness. No upstream B-side repeater/rise-time accelerator. Total host pullup current &lt;=3 mA; selected-branch effective pullups &gt;=2.2 kohm including parallel module resistors/tolerance. Verify actual wiring and rise times.</x:v>
+        <x:v>Connect standard four-wire Qwiic to J9 MASTER. Host 3.3 V powers only the host interface. Other Thing Plus variants require their own pin/power check. PCB-specific firmware initialization is required.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="154" customHeight="1">
       <x:c r="A6" s="3" t="str">
-        <x:v>12 V power supply</x:v>
+        <x:v>Standard Qwiic cable</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>1 supply per board or budgeted distribution</x:v>
+        <x:v>1 per connection</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
-        <x:v>To be selected</x:v>
+        <x:v>Qwiic-compatible cable supplier</x:v>
       </x:c>
       <x:c r="D6" s="3" t="str">
-        <x:v>Regulated 12 V, center-positive, 5.5 × 2.5 mm plug</x:v>
+        <x:v>Four-wire JST SH 1.0 mm mating cable; length to suit</x:v>
       </x:c>
       <x:c r="E6" s="3" t="str">
-        <x:v>Board input power</x:v>
+        <x:v>Master to J9, or local sensors to J1/J12/J17</x:v>
       </x:c>
       <x:c r="F6" s="3" t="str">
-        <x:v>https://www.sameskydevices.com/product/resource/pj-082bh.pdf</x:v>
+        <x:v>https://www.sparkfun.com/qwiic</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>12 V, 2 A starting rating for specified loads; validate actual startup and simultaneous-load current. Board input fuse 2 A; do not increase load budget just because supply is larger.</x:v>
+        <x:v>Pin 1 GND (black), 2 3.3 V (red), 3 SDA (blue), 4 SCL (yellow). Observe connector pin numbering; do not infer pin order from viewing direction.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="154" customHeight="1">
-      <x:c r="A7" s="3" t="str">
-        <x:v>Qwiic master</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="str">
-        <x:v>1 per system</x:v>
-      </x:c>
-      <x:c r="C7" s="3" t="str">
-        <x:v>SparkFun</x:v>
-      </x:c>
-      <x:c r="D7" s="3" t="str">
-        <x:v>WRL-15663 (ESP32 Thing Plus, Micro-B)</x:v>
-      </x:c>
-      <x:c r="E7" s="3" t="str">
-        <x:v>USB/battery-powered I2C master; GPIO23 SDA, GPIO22 SCL</x:v>
-      </x:c>
-      <x:c r="F7" s="3" t="str">
-        <x:v>https://cdn.sparkfun.com/assets/6/d/c/6/c/ESP32_Thing_Plus_Schematic.pdf</x:v>
-      </x:c>
-      <x:c r="G7" s="3" t="str">
-        <x:v>Connect standard four-wire Qwiic to J9 MASTER. Host 3.3 V powers only the host interface. Other Thing Plus variants require their own pin/power check. PCB-specific firmware initialization is required.</x:v>
-      </x:c>
+      <x:c r="A7"/>
+      <x:c r="B7"/>
+      <x:c r="C7"/>
+      <x:c r="D7"/>
+      <x:c r="E7"/>
+      <x:c r="F7"/>
+      <x:c r="G7"/>
     </x:row>
     <x:row r="8" ht="154" customHeight="1">
-      <x:c r="A8" s="3" t="str">
-        <x:v>Standard Qwiic cable</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="str">
-        <x:v>1 per connection</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="str">
-        <x:v>Qwiic-compatible cable supplier</x:v>
-      </x:c>
-      <x:c r="D8" s="3" t="str">
-        <x:v>Four-wire JST SH 1.0 mm mating cable; length to suit</x:v>
-      </x:c>
-      <x:c r="E8" s="3" t="str">
-        <x:v>Master to J9, or local sensors to J1/J12/J17</x:v>
-      </x:c>
-      <x:c r="F8" s="3" t="str">
-        <x:v>https://www.sparkfun.com/qwiic</x:v>
-      </x:c>
-      <x:c r="G8" s="3" t="str">
-        <x:v>Pin 1 GND (black), 2 3.3 V (red), 3 SDA (blue), 4 SCL (yellow). Observe connector pin numbering; do not infer pin order from viewing direction.</x:v>
-      </x:c>
+      <x:c r="A8"/>
+      <x:c r="B8"/>
+      <x:c r="C8"/>
+      <x:c r="D8"/>
+      <x:c r="E8"/>
+      <x:c r="F8"/>
+      <x:c r="G8"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b3d0d4779294d8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ead56bc8fcc47cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3237,7 +3185,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5fafd3e4a084324"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R683616b9a51c4778"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update RheoBoard v1.05 design files and documentation
- Revised the assembly and bringup instructions to clarify the inspection process for components, including the new Q11 MOSFET and D37 zener diode.
- Updated the revision notes to reflect the acceptance of prototype risks related to U5's reset strategy and valve voltage margins.
- Enhanced the BOM to include the new reverse-polarity stage components and updated part counts.
- Adjusted manufacturing files to ensure consistency with the latest design changes, including the removal of obsolete Gerber files.

These changes improve the clarity, usability, and accuracy of the RheoBoard project files and documentation.
</commit_message>
<xml_diff>
--- a/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
+++ b/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R9c36f24d735a4c3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="Rad8e0848fc514f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="R381aa90d17ac465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rcd21091360504211"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="R9d30e2348e654d9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="R51fbe10935c6473f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -41,7 +41,7 @@
       <x:name val="Times New Roman"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -68,6 +68,11 @@
         <x:fgColor rgb="FF4F81BD"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -81,7 +86,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -131,6 +136,9 @@
     <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -139,7 +147,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:M50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
@@ -175,7 +183,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RheoBoard105SMT" displayName="RheoBoard105SMT" ref="A1:D45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RheoBoard105SMT" displayName="RheoBoard105SMT" ref="A1:D46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
@@ -901,42 +909,41 @@
     </x:row>
     <x:row r="14" ht="53" customHeight="1">
       <x:c r="A14" s="7" t="str">
-        <x:v>B540C-13-F</x:v>
+        <x:v>DMP6023LE-13</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>D1</x:v>
+        <x:v>Q11</x:v>
       </x:c>
       <x:c r="C14" s="7" t="str">
-        <x:v>Diode_SMD:D_SMC</x:v>
+        <x:v>Package_TO_SOT_SMD:SOT-223-3_TabPin2</x:v>
       </x:c>
       <x:c r="D14" s="7" t="str">
-        <x:v>C72264</x:v>
+        <x:v>C154901</x:v>
       </x:c>
       <x:c r="E14" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F14" s="9" t="n">
-        <x:v>0.438</x:v>
-      </x:c>
-      <x:c r="G14" s="9" t="n">
+      <x:c r="F14" s="19"/>
+      <x:c r="G14" s="9" t="str">
         <x:f>IF(ISNUMBER(F14),E14*F14,"")</x:f>
-        <x:v>0.438</x:v>
       </x:c>
       <x:c r="H14" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C72264.html</x:v>
-      </x:c>
-      <x:c r="I14" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C154901.html</x:v>
+      </x:c>
+      <x:c r="I14" s="7" t="str">
+        <x:v>https://www.diodes.com/datasheet/download/DMP6023LE.pdf</x:v>
+      </x:c>
       <x:c r="J14" s="7" t="str">
-        <x:v>B540C-13-F</x:v>
+        <x:v>DMP6023LE-13</x:v>
       </x:c>
       <x:c r="K14" s="7" t="str">
-        <x:v>DIODES</x:v>
+        <x:v>Diodes Incorporated</x:v>
       </x:c>
       <x:c r="L14" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M14" s="7" t="str">
-        <x:v>SMC package and cathode mark now match B540C-13-F.</x:v>
+        <x:v>Replaces D1 with lower-loss reverse-polarity protection. 1 gate, 2 drain/tab to fused input, 3 source to VIN_RAW.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="53" customHeight="1">
@@ -1463,7 +1470,7 @@
         <x:v>10K/0603/1%</x:v>
       </x:c>
       <x:c r="B28" s="7" t="str">
-        <x:v>R13, R14, R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84</x:v>
+        <x:v>R13, R14, R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84, R85</x:v>
       </x:c>
       <x:c r="C28" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
@@ -1472,14 +1479,14 @@
         <x:v>C25804</x:v>
       </x:c>
       <x:c r="E28" s="8" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F28" s="9" t="n">
         <x:v>0.014</x:v>
       </x:c>
       <x:c r="G28" s="9" t="n">
         <x:f>IF(ISNUMBER(F28),E28*F28,"")</x:f>
-        <x:v>0.266</x:v>
+        <x:v>0.28</x:v>
       </x:c>
       <x:c r="H28" s="7" t="str">
         <x:v>https://www.lcsc.com/product-detail/C25804.html</x:v>
@@ -1495,7 +1502,7 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M28" s="7" t="str">
-        <x:v>R84 added from HOST_3V3 to GND for discharge (0.33 mA nominal).</x:v>
+        <x:v>R84 discharges HOST_3V3. R85 pulls Q11 gate to GND for reverse-polarity protection.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="53" customHeight="1">
@@ -2302,65 +2309,125 @@
         <x:v>Qwiic master interface: local bus on A, host on B. EN and VCCB use HOST_3V3; separate supplies, common GND. TI DGK land pattern: 1.4 x 0.45 mm pads, 0.65 mm pitch, 4.4 mm row-center span.</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="30" customHeight="1">
-      <x:c r="A50" s="14" t="str">
+    <x:row r="50" ht="83" customHeight="1">
+      <x:c r="A50" s="7" t="str">
+        <x:v>BZT52C10-7-F</x:v>
+      </x:c>
+      <x:c r="B50" s="7" t="str">
+        <x:v>D37</x:v>
+      </x:c>
+      <x:c r="C50" s="7" t="str">
+        <x:v>Diode_SMD:D_SOD-123</x:v>
+      </x:c>
+      <x:c r="D50" s="7" t="str">
+        <x:v>C155227</x:v>
+      </x:c>
+      <x:c r="E50" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F50" s="10"/>
+      <x:c r="G50" s="9" t="str">
+        <x:f>IF(ISNUMBER(F50),E50*F50,"")</x:f>
+      </x:c>
+      <x:c r="H50" s="7" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C155227.html</x:v>
+      </x:c>
+      <x:c r="I50" s="7" t="str">
+        <x:v>https://www.diodes.com/datasheet/download/BZT52Cxx.pdf</x:v>
+      </x:c>
+      <x:c r="J50" s="7" t="str">
+        <x:v>BZT52C10-7-F</x:v>
+      </x:c>
+      <x:c r="K50" s="7" t="str">
+        <x:v>Diodes Incorporated</x:v>
+      </x:c>
+      <x:c r="L50" s="7" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M50" s="7" t="str">
+        <x:v>Q11 gate-source clamp. Cathode to VIN_RAW/source; anode to gate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="30" customHeight="1">
+      <x:c r="A51" s="14" t="str">
         <x:v>Total fitted parts / incomplete priced subtotal</x:v>
       </x:c>
-      <x:c r="B50" s="14"/>
-      <x:c r="C50" s="14"/>
-      <x:c r="D50" s="14"/>
-      <x:c r="E50" s="14" t="n">
-        <x:f>SUM(E2:E49)</x:f>
-        <x:v>146</x:v>
-      </x:c>
-      <x:c r="F50" s="14" t="str">
+      <x:c r="B51" s="14"/>
+      <x:c r="C51" s="14"/>
+      <x:c r="D51" s="14"/>
+      <x:c r="E51" s="14" t="n">
+        <x:f>SUM(E2:E50)</x:f>
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="F51" s="14" t="str">
         <x:v>Incomplete estimate</x:v>
       </x:c>
-      <x:c r="G50" s="15" t="n">
-        <x:f>SUM(G2:G49)</x:f>
-        <x:v>55.617999999999995</x:v>
-      </x:c>
-      <x:c r="H50"/>
-      <x:c r="I50"/>
-      <x:c r="J50"/>
-      <x:c r="K50"/>
-      <x:c r="L50"/>
-      <x:c r="M50"/>
-    </x:row>
-    <x:row r="51" ht="30" customHeight="1">
-      <x:c r="A51"/>
-      <x:c r="B51"/>
-      <x:c r="C51"/>
-      <x:c r="D51"/>
-      <x:c r="E51"/>
-      <x:c r="F51"/>
-      <x:c r="G51"/>
+      <x:c r="G51" s="15" t="n">
+        <x:f>SUM(G2:G50)</x:f>
+        <x:v>55.194</x:v>
+      </x:c>
+      <x:c r="H51"/>
+      <x:c r="I51"/>
+      <x:c r="J51"/>
+      <x:c r="K51"/>
+      <x:c r="L51"/>
+      <x:c r="M51"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52"/>
+      <x:c r="B52"/>
+      <x:c r="C52"/>
+      <x:c r="D52"/>
+      <x:c r="E52"/>
+      <x:c r="F52"/>
+      <x:c r="G52"/>
+      <x:c r="H52"/>
+      <x:c r="I52"/>
+      <x:c r="J52"/>
+      <x:c r="K52"/>
+      <x:c r="L52"/>
+      <x:c r="M52"/>
     </x:row>
     <x:row r="53" ht="34" customHeight="1">
-      <x:c r="A53" s="16" t="str">
+      <x:c r="A53"/>
+      <x:c r="B53"/>
+      <x:c r="C53"/>
+      <x:c r="D53"/>
+      <x:c r="E53"/>
+      <x:c r="F53"/>
+      <x:c r="G53"/>
+      <x:c r="H53"/>
+      <x:c r="I53"/>
+      <x:c r="J53"/>
+      <x:c r="K53"/>
+      <x:c r="L53"/>
+      <x:c r="M53"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="16" t="str">
         <x:v>Prices are retained from the original workbook only where the selected part is unchanged. New parts have blank prices. This subtotal is incomplete and is not a JLCPCB quotation; obtain a fresh quote for v1.05.</x:v>
       </x:c>
-      <x:c r="B53" s="16"/>
-      <x:c r="C53" s="16"/>
-      <x:c r="D53" s="16"/>
-      <x:c r="E53" s="16"/>
-      <x:c r="F53" s="16"/>
-      <x:c r="G53" s="16"/>
-      <x:c r="H53" s="16"/>
-      <x:c r="I53" s="16"/>
-      <x:c r="J53" s="16"/>
-      <x:c r="K53" s="16"/>
-      <x:c r="L53" s="16"/>
-      <x:c r="M53" s="16"/>
+      <x:c r="B54" s="16"/>
+      <x:c r="C54" s="16"/>
+      <x:c r="D54" s="16"/>
+      <x:c r="E54" s="16"/>
+      <x:c r="F54" s="16"/>
+      <x:c r="G54" s="16"/>
+      <x:c r="H54" s="16"/>
+      <x:c r="I54" s="16"/>
+      <x:c r="J54" s="16"/>
+      <x:c r="K54" s="16"/>
+      <x:c r="L54" s="16"/>
+      <x:c r="M54" s="16"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A51:D51"/>
-    <x:mergeCell ref="A53:M53"/>
+    <x:mergeCell ref="A52:D52"/>
+    <x:mergeCell ref="A54:M54"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7b14771b7ab43eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra94a2ddbbbb343d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2537,7 +2604,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ead56bc8fcc47cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7db9df7c5530470e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2736,16 +2803,16 @@
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="3" t="str">
-        <x:v>B540C-13-F</x:v>
+        <x:v>DMP6023LE-13</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
-        <x:v>D1</x:v>
+        <x:v>Q11</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
-        <x:v>Diode_SMD:D_SMC</x:v>
+        <x:v>Package_TO_SOT_SMD:SOT-223-3_TabPin2</x:v>
       </x:c>
       <x:c r="D14" s="3" t="str">
-        <x:v>C72264</x:v>
+        <x:v>C154901</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
@@ -2907,7 +2974,7 @@
         <x:v>10K/0603/1%</x:v>
       </x:c>
       <x:c r="B26" s="3" t="str">
-        <x:v>R13, R14, R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84</x:v>
+        <x:v>R13, R14, R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84, R85</x:v>
       </x:c>
       <x:c r="C26" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
@@ -3182,10 +3249,24 @@
         <x:v>C201698</x:v>
       </x:c>
     </x:row>
+    <x:row r="46" ht="70" customHeight="1">
+      <x:c r="A46" s="3" t="str">
+        <x:v>BZT52C10-7-F</x:v>
+      </x:c>
+      <x:c r="B46" s="3" t="str">
+        <x:v>D37</x:v>
+      </x:c>
+      <x:c r="C46" s="3" t="str">
+        <x:v>Diode_SMD:D_SOD-123</x:v>
+      </x:c>
+      <x:c r="D46" s="3" t="str">
+        <x:v>C155227</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R683616b9a51c4778"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4025bb32a59f468d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update RheoBoard v1.05 documentation and design files
- Enhanced ASSEMBLY_AND_BRINGUP.md to include details about the new J19 button GPIO header and its connection to the ESP32.
- Revised README.md to reflect the removal of U4 and the consolidation of actuator control in U7 PCA9685, clarifying the button interface requirements.
- Updated REVISION_NOTES.md to document the removal of the TCA9534 and the addition of the J19 header, along with the corresponding changes in the BOM.
- Adjusted BOM files to reflect the updated part counts and configurations, including the addition of manually fitted components.

These changes improve the clarity and usability of the RheoBoard project documentation and design files.
</commit_message>
<xml_diff>
--- a/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
+++ b/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rcd21091360504211"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="R9d30e2348e654d9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="R51fbe10935c6473f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rdb7370b51d894220"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="R793197d3893f4a53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="R858b91da9fdd4677"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -41,7 +41,7 @@
       <x:name val="Times New Roman"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -73,6 +73,11 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -86,7 +91,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="21">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -139,6 +144,9 @@
     <x:xf numFmtId="201" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -147,7 +155,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:M50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:M48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
@@ -168,7 +176,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="RheoBoard105Accessories" displayName="RheoBoard105Accessories" ref="A1:G6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="RheoBoard105Accessories" displayName="RheoBoard105Accessories" ref="A1:G7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Item"/>
     <x:tableColumn id="2" name="Quantity basis"/>
@@ -183,7 +191,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RheoBoard105SMT" displayName="RheoBoard105SMT" ref="A1:D46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="RheoBoard105SMT" displayName="RheoBoard105SMT" ref="A1:D43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
@@ -450,7 +458,7 @@
         <x:v>10uF 25V X5R ±10%</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>C1,C2,C8,C9,C15,C16</x:v>
+        <x:v>C1, C2, C8, C9, C15, C16</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
         <x:v>Capacitor_SMD:C_0805_2012Metric_Pad1.18x1.45mm_HandSolder</x:v>
@@ -471,7 +479,7 @@
       <x:c r="H2" s="7" t="str">
         <x:v>https://www.lcsc.com/product-detail/C5448891.html</x:v>
       </x:c>
-      <x:c r="I2" s="7" t="str"/>
+      <x:c r="I2" s="7"/>
       <x:c r="J2" s="7" t="str">
         <x:v>TCC0805X5R106K250FT</x:v>
       </x:c>
@@ -481,14 +489,14 @@
       <x:c r="L2" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M2" s="7" t="str"/>
+      <x:c r="M2" s="7"/>
     </x:row>
     <x:row r="3" ht="126" customHeight="1">
       <x:c r="A3" s="7" t="str">
         <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>C3, C4, C5, C23, C24, C25, C26, C30, C31, C33, C42, C44, C46, C47, C56, C59, C63, C68, C69</x:v>
+        <x:v>C3, C4, C5, C23, C24, C25, C26, C30, C31, C33, C42, C44, C46, C56, C59, C63, C68, C69</x:v>
       </x:c>
       <x:c r="C3" s="7" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
@@ -497,19 +505,19 @@
         <x:v>C14663</x:v>
       </x:c>
       <x:c r="E3" s="8" t="n">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F3" s="9" t="n">
         <x:v>0.073</x:v>
       </x:c>
       <x:c r="G3" s="9" t="n">
         <x:f>IF(ISNUMBER(F3),E3*F3,"")</x:f>
-        <x:v>1.387</x:v>
+        <x:v>1.3139999999999998</x:v>
       </x:c>
       <x:c r="H3" s="7" t="str">
         <x:v>https://www.lcsc.com/product-detail/C14663.html</x:v>
       </x:c>
-      <x:c r="I3" s="7" t="str"/>
+      <x:c r="I3" s="7"/>
       <x:c r="J3" s="7" t="str">
         <x:v>CC0603KRX7R9BB104</x:v>
       </x:c>
@@ -525,71 +533,71 @@
     </x:row>
     <x:row r="4" ht="53" customHeight="1">
       <x:c r="A4" s="7" t="str">
-        <x:v>10nF 50V ±10%</x:v>
+        <x:v>1nF 50V X7R ±5%</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>C22</x:v>
+        <x:v>C27</x:v>
       </x:c>
       <x:c r="C4" s="7" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D4" s="7" t="str">
-        <x:v>C57112</x:v>
+        <x:v>C5360811</x:v>
       </x:c>
       <x:c r="E4" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>0.92</x:v>
+        <x:v>0.052</x:v>
       </x:c>
       <x:c r="G4" s="9" t="n">
         <x:f>IF(ISNUMBER(F4),E4*F4,"")</x:f>
-        <x:v>0.92</x:v>
+        <x:v>0.052</x:v>
       </x:c>
       <x:c r="H4" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C57112.html</x:v>
-      </x:c>
-      <x:c r="I4" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C5360811.html</x:v>
+      </x:c>
+      <x:c r="I4" s="7"/>
       <x:c r="J4" s="7" t="str">
-        <x:v>0603B103K500NT</x:v>
+        <x:v>TCC0603X7R102J500CT</x:v>
       </x:c>
       <x:c r="K4" s="7" t="str">
-        <x:v>FH</x:v>
+        <x:v>CCTC</x:v>
       </x:c>
       <x:c r="L4" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M4" s="7" t="str"/>
+      <x:c r="M4" s="7"/>
     </x:row>
     <x:row r="5" ht="53" customHeight="1">
       <x:c r="A5" s="7" t="str">
-        <x:v>1nF 50V X7R ±5%</x:v>
+        <x:v>10uF 25V X5R ±10%</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>C27</x:v>
+        <x:v>C28, C29</x:v>
       </x:c>
       <x:c r="C5" s="7" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D5" s="7" t="str">
-        <x:v>C5360811</x:v>
+        <x:v>C7393892</x:v>
       </x:c>
       <x:c r="E5" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>0.052</x:v>
+        <x:v>0.165</x:v>
       </x:c>
       <x:c r="G5" s="9" t="n">
         <x:f>IF(ISNUMBER(F5),E5*F5,"")</x:f>
-        <x:v>0.052</x:v>
+        <x:v>0.33</x:v>
       </x:c>
       <x:c r="H5" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C5360811.html</x:v>
-      </x:c>
-      <x:c r="I5" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C7393892.html</x:v>
+      </x:c>
+      <x:c r="I5" s="7"/>
       <x:c r="J5" s="7" t="str">
-        <x:v>TCC0603X7R102J500CT</x:v>
+        <x:v>TCC0603X5R106K250CT</x:v>
       </x:c>
       <x:c r="K5" s="7" t="str">
         <x:v>CCTC</x:v>
@@ -597,173 +605,172 @@
       <x:c r="L5" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M5" s="7" t="str"/>
+      <x:c r="M5" s="7"/>
     </x:row>
     <x:row r="6" ht="53" customHeight="1">
       <x:c r="A6" s="7" t="str">
-        <x:v>10uF 25V X5R ±10%</x:v>
+        <x:v>22uF 50V ±20%</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>C28,C29</x:v>
+        <x:v>C32, C34, C43, C45</x:v>
       </x:c>
       <x:c r="C6" s="7" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
+        <x:v>Capacitor_SMD:CP_Elec_6.3x5.8</x:v>
       </x:c>
       <x:c r="D6" s="7" t="str">
-        <x:v>C7393892</x:v>
+        <x:v>C128458</x:v>
       </x:c>
       <x:c r="E6" s="8" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F6" s="9" t="n">
-        <x:v>0.165</x:v>
-      </x:c>
-      <x:c r="G6" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F6" s="10"/>
+      <x:c r="G6" s="9" t="str">
         <x:f>IF(ISNUMBER(F6),E6*F6,"")</x:f>
-        <x:v>0.33</x:v>
       </x:c>
       <x:c r="H6" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C7393892.html</x:v>
-      </x:c>
-      <x:c r="I6" s="7" t="str"/>
+        <x:v>https://industrial.panasonic.com/ww/products/pt/aluminum-cap-smd/models/EEEFK1H220P</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="str">
+        <x:v>https://industrial.panasonic.com/cdbs/www-data/pdf/RDE0000/ABA0000C776.pdf</x:v>
+      </x:c>
       <x:c r="J6" s="7" t="str">
-        <x:v>TCC0603X5R106K250CT</x:v>
+        <x:v>EEEFK1H220P</x:v>
       </x:c>
       <x:c r="K6" s="7" t="str">
-        <x:v>CCTC</x:v>
+        <x:v>Panasonic</x:v>
       </x:c>
       <x:c r="L6" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M6" s="7" t="str"/>
+      <x:c r="M6" s="7" t="str">
+        <x:v>Reduced from 100uF to 22uF; each pump/valve rail is approximately 88.3uF nominal. Bench transient validation remains required.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="53" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>22uF 50V ±20%</x:v>
+        <x:v>22uF 25V X5R ±20%</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>C32,C34,C43,C45</x:v>
+        <x:v>C52, C53, C54, C57, C60, C61</x:v>
       </x:c>
       <x:c r="C7" s="7" t="str">
-        <x:v>Capacitor_SMD:CP_Elec_6.3x5.8</x:v>
+        <x:v>Capacitor_SMD:C_0805_2012Metric_Pad1.18x1.45mm_HandSolder</x:v>
       </x:c>
       <x:c r="D7" s="7" t="str">
-        <x:v>C128458</x:v>
+        <x:v>C20416420</x:v>
       </x:c>
       <x:c r="E7" s="8" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F7" s="10"/>
-      <x:c r="G7" s="9" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="n">
         <x:f>IF(ISNUMBER(F7),E7*F7,"")</x:f>
+        <x:v>1.296</x:v>
       </x:c>
       <x:c r="H7" s="7" t="str">
-        <x:v>https://industrial.panasonic.com/ww/products/pt/aluminum-cap-smd/models/EEEFK1H220P</x:v>
-      </x:c>
-      <x:c r="I7" s="7" t="str">
-        <x:v>https://industrial.panasonic.com/cdbs/www-data/pdf/RDE0000/ABA0000C776.pdf</x:v>
-      </x:c>
+        <x:v>https://www.lcsc.com/product-detail/C20416420.html</x:v>
+      </x:c>
+      <x:c r="I7" s="7"/>
       <x:c r="J7" s="7" t="str">
-        <x:v>EEEFK1H220P</x:v>
+        <x:v>TCC0805X5R226M250FT</x:v>
       </x:c>
       <x:c r="K7" s="7" t="str">
-        <x:v>Panasonic</x:v>
+        <x:v>CCTC</x:v>
       </x:c>
       <x:c r="L7" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M7" s="7" t="str">
-        <x:v>Reduced from 100uF to 22uF; each pump/valve rail is approximately 88.3uF nominal. Bench transient validation remains required.</x:v>
-      </x:c>
+      <x:c r="M7" s="7"/>
     </x:row>
     <x:row r="8" ht="53" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>22uF 25V X5R ±20%</x:v>
+        <x:v>18pF 50V C0G ±2%</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>C52,C53,C54,C57,C60,C61</x:v>
+        <x:v>C55, C58, C62</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
-        <x:v>Capacitor_SMD:C_0805_2012Metric_Pad1.18x1.45mm_HandSolder</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D8" s="7" t="str">
-        <x:v>C20416420</x:v>
+        <x:v>C2169079</x:v>
       </x:c>
       <x:c r="E8" s="8" t="n">
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>0.216</x:v>
+        <x:v>0.043</x:v>
       </x:c>
       <x:c r="G8" s="9" t="n">
         <x:f>IF(ISNUMBER(F8),E8*F8,"")</x:f>
-        <x:v>1.296</x:v>
+        <x:v>0.129</x:v>
       </x:c>
       <x:c r="H8" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C20416420.html</x:v>
-      </x:c>
-      <x:c r="I8" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C2169079.html</x:v>
+      </x:c>
+      <x:c r="I8" s="7"/>
       <x:c r="J8" s="7" t="str">
-        <x:v>TCC0805X5R226M250FT</x:v>
+        <x:v>VJ0603A180GXACW1BC</x:v>
       </x:c>
       <x:c r="K8" s="7" t="str">
-        <x:v>CCTC</x:v>
+        <x:v>VISHAY</x:v>
       </x:c>
       <x:c r="L8" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M8" s="7" t="str"/>
+      <x:c r="M8" s="7"/>
     </x:row>
     <x:row r="9" ht="53" customHeight="1">
       <x:c r="A9" s="7" t="str">
-        <x:v>18pF 50V C0G ±2%</x:v>
+        <x:v>3.3nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>C55,C58,C62</x:v>
+        <x:v>C64</x:v>
       </x:c>
       <x:c r="C9" s="7" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D9" s="7" t="str">
-        <x:v>C2169079</x:v>
+        <x:v>C107088</x:v>
       </x:c>
       <x:c r="E9" s="8" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F9" s="9" t="n">
-        <x:v>0.043</x:v>
-      </x:c>
-      <x:c r="G9" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F9" s="10"/>
+      <x:c r="G9" s="9" t="str">
         <x:f>IF(ISNUMBER(F9),E9*F9,"")</x:f>
-        <x:v>0.129</x:v>
       </x:c>
       <x:c r="H9" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C2169079.html</x:v>
-      </x:c>
-      <x:c r="I9" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C107088.html</x:v>
+      </x:c>
+      <x:c r="I9" s="7"/>
       <x:c r="J9" s="7" t="str">
-        <x:v>VJ0603A180GXACW1BC</x:v>
+        <x:v>CC0603KRX7R9BB332</x:v>
       </x:c>
       <x:c r="K9" s="7" t="str">
-        <x:v>VISHAY</x:v>
+        <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="L9" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M9" s="7" t="str"/>
+      <x:c r="M9" s="7" t="str">
+        <x:v>New controlled-startup timing capacitor for U12.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="53" customHeight="1">
       <x:c r="A10" s="7" t="str">
-        <x:v>3.3nF 50V X7R ±10%</x:v>
+        <x:v>1uF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>C64</x:v>
+        <x:v>C65</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:C_0805_2012Metric</x:v>
       </x:c>
       <x:c r="D10" s="7" t="str">
-        <x:v>C107088</x:v>
+        <x:v>C91185</x:v>
       </x:c>
       <x:c r="E10" s="8" t="n">
         <x:v>1</x:v>
@@ -773,11 +780,13 @@
         <x:f>IF(ISNUMBER(F10),E10*F10,"")</x:f>
       </x:c>
       <x:c r="H10" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C107088.html</x:v>
-      </x:c>
-      <x:c r="I10" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C91185.html</x:v>
+      </x:c>
+      <x:c r="I10" s="7" t="str">
+        <x:v>https://www.yageogroup.com/download/specsheet/CC0805KKX7R9BB105</x:v>
+      </x:c>
       <x:c r="J10" s="7" t="str">
-        <x:v>CC0603KRX7R9BB332</x:v>
+        <x:v>CC0805KKX7R9BB105</x:v>
       </x:c>
       <x:c r="K10" s="7" t="str">
         <x:v>YAGEO</x:v>
@@ -786,37 +795,38 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M10" s="7" t="str">
-        <x:v>New controlled-startup timing capacitor for U12.</x:v>
+        <x:v>New local input bypass for U12; place beside IN/GND.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="53" customHeight="1">
       <x:c r="A11" s="7" t="str">
-        <x:v>1uF 50V X7R ±10%</x:v>
+        <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>C65</x:v>
+        <x:v>C66</x:v>
       </x:c>
       <x:c r="C11" s="7" t="str">
-        <x:v>Capacitor_SMD:C_0805_2012Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D11" s="7" t="str">
-        <x:v>C91185</x:v>
+        <x:v>C14663</x:v>
       </x:c>
       <x:c r="E11" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F11" s="10"/>
-      <x:c r="G11" s="9" t="str">
+      <x:c r="F11" s="9" t="n">
+        <x:v>0.073</x:v>
+      </x:c>
+      <x:c r="G11" s="9" t="n">
         <x:f>IF(ISNUMBER(F11),E11*F11,"")</x:f>
+        <x:v>0.073</x:v>
       </x:c>
       <x:c r="H11" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C91185.html</x:v>
-      </x:c>
-      <x:c r="I11" s="7" t="str">
-        <x:v>https://www.yageogroup.com/download/specsheet/CC0805KKX7R9BB105</x:v>
-      </x:c>
+        <x:v>https://www.lcsc.com/product-detail/C14663.html</x:v>
+      </x:c>
+      <x:c r="I11" s="7"/>
       <x:c r="J11" s="7" t="str">
-        <x:v>CC0805KKX7R9BB105</x:v>
+        <x:v>CC0603KRX7R9BB104</x:v>
       </x:c>
       <x:c r="K11" s="7" t="str">
         <x:v>YAGEO</x:v>
@@ -825,38 +835,37 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M11" s="7" t="str">
-        <x:v>New local input bypass for U12; place beside IN/GND.</x:v>
+        <x:v>New local input high-frequency bypass for U12.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="53" customHeight="1">
       <x:c r="A12" s="7" t="str">
-        <x:v>100nF 50V X7R ±10%</x:v>
+        <x:v>4.7uF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>C66</x:v>
+        <x:v>C67</x:v>
       </x:c>
       <x:c r="C12" s="7" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:C_1206_3216Metric</x:v>
       </x:c>
       <x:c r="D12" s="7" t="str">
-        <x:v>C14663</x:v>
+        <x:v>C132170</x:v>
       </x:c>
       <x:c r="E12" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F12" s="9" t="n">
-        <x:v>0.073</x:v>
-      </x:c>
-      <x:c r="G12" s="9" t="n">
+      <x:c r="F12" s="10"/>
+      <x:c r="G12" s="9" t="str">
         <x:f>IF(ISNUMBER(F12),E12*F12,"")</x:f>
-        <x:v>0.073</x:v>
       </x:c>
       <x:c r="H12" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C14663.html</x:v>
-      </x:c>
-      <x:c r="I12" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C132170.html</x:v>
+      </x:c>
+      <x:c r="I12" s="7" t="str">
+        <x:v>https://www.yageogroup.com/download/specsheet/CC1206KKX7R9BB475</x:v>
+      </x:c>
       <x:c r="J12" s="7" t="str">
-        <x:v>CC0603KRX7R9BB104</x:v>
+        <x:v>CC1206KKX7R9BB475</x:v>
       </x:c>
       <x:c r="K12" s="7" t="str">
         <x:v>YAGEO</x:v>
@@ -865,21 +874,21 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M12" s="7" t="str">
-        <x:v>New local input high-frequency bypass for U12.</x:v>
+        <x:v>New local output bypass for U12; place beside OUT/GND.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="53" customHeight="1">
       <x:c r="A13" s="7" t="str">
-        <x:v>4.7uF 50V X7R ±10%</x:v>
+        <x:v>DMP6023LE-13</x:v>
       </x:c>
       <x:c r="B13" s="7" t="str">
-        <x:v>C67</x:v>
+        <x:v>Q11</x:v>
       </x:c>
       <x:c r="C13" s="7" t="str">
-        <x:v>Capacitor_SMD:C_1206_3216Metric</x:v>
+        <x:v>Package_TO_SOT_SMD:SOT-223-3_TabPin2</x:v>
       </x:c>
       <x:c r="D13" s="7" t="str">
-        <x:v>C132170</x:v>
+        <x:v>C154901</x:v>
       </x:c>
       <x:c r="E13" s="8" t="n">
         <x:v>1</x:v>
@@ -889,460 +898,459 @@
         <x:f>IF(ISNUMBER(F13),E13*F13,"")</x:f>
       </x:c>
       <x:c r="H13" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C132170.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C154901.html</x:v>
       </x:c>
       <x:c r="I13" s="7" t="str">
-        <x:v>https://www.yageogroup.com/download/specsheet/CC1206KKX7R9BB475</x:v>
+        <x:v>https://www.diodes.com/datasheet/download/DMP6023LE.pdf</x:v>
       </x:c>
       <x:c r="J13" s="7" t="str">
-        <x:v>CC1206KKX7R9BB475</x:v>
+        <x:v>DMP6023LE-13</x:v>
       </x:c>
       <x:c r="K13" s="7" t="str">
-        <x:v>YAGEO</x:v>
+        <x:v>Diodes Incorporated</x:v>
       </x:c>
       <x:c r="L13" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M13" s="7" t="str">
-        <x:v>New local output bypass for U12; place beside OUT/GND.</x:v>
+        <x:v>Replaces D1 with lower-loss reverse-polarity protection. 1 gate, 2 drain/tab to fused input, 3 source to VIN_RAW.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="53" customHeight="1">
       <x:c r="A14" s="7" t="str">
-        <x:v>DMP6023LE-13</x:v>
+        <x:v>LED_Red</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>Q11</x:v>
+        <x:v>D6, D7, D8, D13, D14, D15, D17, D19</x:v>
       </x:c>
       <x:c r="C14" s="7" t="str">
-        <x:v>Package_TO_SOT_SMD:SOT-223-3_TabPin2</x:v>
+        <x:v>LED_SMD:LED_0603_1608Metric_Pad1.05x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D14" s="7" t="str">
-        <x:v>C154901</x:v>
+        <x:v>C434419</x:v>
       </x:c>
       <x:c r="E14" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F14" s="19"/>
-      <x:c r="G14" s="9" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F14" s="9" t="n">
+        <x:v>0.098</x:v>
+      </x:c>
+      <x:c r="G14" s="9" t="n">
         <x:f>IF(ISNUMBER(F14),E14*F14,"")</x:f>
+        <x:v>0.784</x:v>
       </x:c>
       <x:c r="H14" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C154901.html</x:v>
-      </x:c>
-      <x:c r="I14" s="7" t="str">
-        <x:v>https://www.diodes.com/datasheet/download/DMP6023LE.pdf</x:v>
-      </x:c>
+        <x:v>https://www.lcsc.com/product-detail/C434419.html</x:v>
+      </x:c>
+      <x:c r="I14" s="7"/>
       <x:c r="J14" s="7" t="str">
-        <x:v>DMP6023LE-13</x:v>
+        <x:v>SZYY0603R</x:v>
       </x:c>
       <x:c r="K14" s="7" t="str">
-        <x:v>Diodes Incorporated</x:v>
+        <x:v>Yongyu Photoelectric</x:v>
       </x:c>
       <x:c r="L14" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M14" s="7" t="str">
-        <x:v>Replaces D1 with lower-loss reverse-polarity protection. 1 gate, 2 drain/tab to fused input, 3 source to VIN_RAW.</x:v>
-      </x:c>
+      <x:c r="M14" s="7"/>
     </x:row>
     <x:row r="15" ht="53" customHeight="1">
       <x:c r="A15" s="7" t="str">
-        <x:v>LED_Red</x:v>
+        <x:v>SS34</x:v>
       </x:c>
       <x:c r="B15" s="7" t="str">
-        <x:v>D6,D7,D8,D13,D14,D15,D17,D19</x:v>
+        <x:v>D11, D12, D16, D18</x:v>
       </x:c>
       <x:c r="C15" s="7" t="str">
-        <x:v>LED_SMD:LED_0603_1608Metric_Pad1.05x0.95mm_HandSolder</x:v>
+        <x:v>Diode_SMD:D_SMA</x:v>
       </x:c>
       <x:c r="D15" s="7" t="str">
-        <x:v>C434419</x:v>
+        <x:v>C115205</x:v>
       </x:c>
       <x:c r="E15" s="8" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F15" s="9" t="n">
-        <x:v>0.098</x:v>
+        <x:v>0.467</x:v>
       </x:c>
       <x:c r="G15" s="9" t="n">
         <x:f>IF(ISNUMBER(F15),E15*F15,"")</x:f>
-        <x:v>0.784</x:v>
+        <x:v>1.868</x:v>
       </x:c>
       <x:c r="H15" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C434419.html</x:v>
-      </x:c>
-      <x:c r="I15" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C115205.html</x:v>
+      </x:c>
+      <x:c r="I15" s="7"/>
       <x:c r="J15" s="7" t="str">
-        <x:v>SZYY0603R</x:v>
+        <x:v>SS34</x:v>
       </x:c>
       <x:c r="K15" s="7" t="str">
-        <x:v>Yongyu Photoelectric</x:v>
+        <x:v>Jingdao Microelectronics</x:v>
       </x:c>
       <x:c r="L15" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M15" s="7" t="str"/>
+      <x:c r="M15" s="7" t="str">
+        <x:v>SMA footprint and polarity mark match selected Jingdao SS34.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="53" customHeight="1">
       <x:c r="A16" s="7" t="str">
-        <x:v>SS34</x:v>
+        <x:v>LED_Red</x:v>
       </x:c>
       <x:c r="B16" s="7" t="str">
-        <x:v>D11,D12,D16,D18</x:v>
+        <x:v>D33, D34, D35</x:v>
       </x:c>
       <x:c r="C16" s="7" t="str">
-        <x:v>Diode_SMD:D_SMA</x:v>
+        <x:v>LED_SMD:LED_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D16" s="7" t="str">
-        <x:v>C115205</x:v>
+        <x:v>C434419</x:v>
       </x:c>
       <x:c r="E16" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F16" s="9" t="n">
-        <x:v>0.467</x:v>
+        <x:v>0.098</x:v>
       </x:c>
       <x:c r="G16" s="9" t="n">
         <x:f>IF(ISNUMBER(F16),E16*F16,"")</x:f>
-        <x:v>1.868</x:v>
+        <x:v>0.29400000000000004</x:v>
       </x:c>
       <x:c r="H16" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C115205.html</x:v>
-      </x:c>
-      <x:c r="I16" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C434419.html</x:v>
+      </x:c>
+      <x:c r="I16" s="7"/>
       <x:c r="J16" s="7" t="str">
-        <x:v>SS34</x:v>
+        <x:v>SZYY0603R</x:v>
       </x:c>
       <x:c r="K16" s="7" t="str">
-        <x:v>Jingdao Microelectronics</x:v>
+        <x:v>Yongyu Photoelectric</x:v>
       </x:c>
       <x:c r="L16" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M16" s="7" t="str">
-        <x:v>SMA footprint and polarity mark match selected Jingdao SS34.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="53" customHeight="1">
+      <x:c r="M16" s="7"/>
+    </x:row>
+    <x:row r="17" ht="83" customHeight="1">
       <x:c r="A17" s="7" t="str">
-        <x:v>LED_Red</x:v>
+        <x:v>SMBJ13A</x:v>
       </x:c>
       <x:c r="B17" s="7" t="str">
-        <x:v>D33,D34,D35</x:v>
+        <x:v>D36</x:v>
       </x:c>
       <x:c r="C17" s="7" t="str">
-        <x:v>LED_SMD:LED_0603_1608Metric</x:v>
+        <x:v>Diode_SMD:D_SMB</x:v>
       </x:c>
       <x:c r="D17" s="7" t="str">
-        <x:v>C434419</x:v>
+        <x:v>C151252</x:v>
       </x:c>
       <x:c r="E17" s="8" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F17" s="9" t="n">
-        <x:v>0.098</x:v>
-      </x:c>
-      <x:c r="G17" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F17" s="10"/>
+      <x:c r="G17" s="9" t="str">
         <x:f>IF(ISNUMBER(F17),E17*F17,"")</x:f>
-        <x:v>0.29400000000000004</x:v>
       </x:c>
       <x:c r="H17" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C434419.html</x:v>
-      </x:c>
-      <x:c r="I17" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C151252.html</x:v>
+      </x:c>
+      <x:c r="I17" s="7" t="str">
+        <x:v>https://m.littelfuse.com/~/media/electronics/datasheets/tvs_diodes/littelfuse_tvs_diode_smbj_datasheet.pdf.pdf</x:v>
+      </x:c>
       <x:c r="J17" s="7" t="str">
-        <x:v>SZYY0603R</x:v>
+        <x:v>SMBJ13A</x:v>
       </x:c>
       <x:c r="K17" s="7" t="str">
-        <x:v>Yongyu Photoelectric</x:v>
+        <x:v>Littelfuse</x:v>
       </x:c>
       <x:c r="L17" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M17" s="7" t="str"/>
-    </x:row>
-    <x:row r="18" ht="83" customHeight="1">
+      <x:c r="M17" s="7" t="str">
+        <x:v>Catalog attribute table incorrectly lists 14V/23.2V while selected manufacturer MPN is SMBJ13A. Require exact MPN SMBJ13A, 13V standoff, 21.5V clamp at 28A per manufacturer table; inspect supplier approval. Not a substitute for eFuse.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="53" customHeight="1">
       <x:c r="A18" s="7" t="str">
-        <x:v>SMBJ13A</x:v>
+        <x:v>2A time-delay JFC1032-1200TS</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>D36</x:v>
+        <x:v>F1</x:v>
       </x:c>
       <x:c r="C18" s="7" t="str">
-        <x:v>Diode_SMD:D_SMB</x:v>
+        <x:v>RheoBoard:Fuse_JDT_JFC1032TS_10.25x3.2mm</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
-        <x:v>C151252</x:v>
+        <x:v>C53035082</x:v>
       </x:c>
       <x:c r="E18" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F18" s="10"/>
-      <x:c r="G18" s="9" t="str">
+      <x:c r="F18" s="9" t="n">
+        <x:v>1.45</x:v>
+      </x:c>
+      <x:c r="G18" s="9" t="n">
         <x:f>IF(ISNUMBER(F18),E18*F18,"")</x:f>
+        <x:v>1.45</x:v>
       </x:c>
       <x:c r="H18" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C151252.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C53035082.html</x:v>
       </x:c>
       <x:c r="I18" s="7" t="str">
-        <x:v>https://m.littelfuse.com/~/media/electronics/datasheets/tvs_diodes/littelfuse_tvs_diode_smbj_datasheet.pdf.pdf</x:v>
+        <x:v>https://www.jdtfuse.com/upload/PDF/JFC1032TS.pdf</x:v>
       </x:c>
       <x:c r="J18" s="7" t="str">
-        <x:v>SMBJ13A</x:v>
+        <x:v>JFC1032-1200TS</x:v>
       </x:c>
       <x:c r="K18" s="7" t="str">
-        <x:v>Littelfuse</x:v>
+        <x:v>JDTfuse</x:v>
       </x:c>
       <x:c r="L18" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M18" s="7" t="str">
-        <x:v>Catalog attribute table incorrectly lists 14V/23.2V while selected manufacturer MPN is SMBJ13A. Require exact MPN SMBJ13A, 13V standoff, 21.5V clamp at 28A per manufacturer table; inspect supplier approval. Not a substitute for eFuse.</x:v>
+        <x:v>Corrected centered origin and JDT land pattern. Check the new placement preview.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="53" customHeight="1">
       <x:c r="A19" s="7" t="str">
-        <x:v>2A time-delay JFC1032-1200TS</x:v>
+        <x:v>JST SH 4-pin 1.00mm</x:v>
       </x:c>
       <x:c r="B19" s="7" t="str">
-        <x:v>F1</x:v>
+        <x:v>J1, J9, J12, J17</x:v>
       </x:c>
       <x:c r="C19" s="7" t="str">
-        <x:v>RheoBoard:Fuse_JDT_JFC1032TS_10.25x3.2mm</x:v>
+        <x:v>Connector_JST:JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</x:v>
       </x:c>
       <x:c r="D19" s="7" t="str">
-        <x:v>C53035082</x:v>
+        <x:v>C160404</x:v>
       </x:c>
       <x:c r="E19" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F19" s="9" t="n">
-        <x:v>1.45</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="G19" s="9" t="n">
         <x:f>IF(ISNUMBER(F19),E19*F19,"")</x:f>
-        <x:v>1.45</x:v>
+        <x:v>2.4</x:v>
       </x:c>
       <x:c r="H19" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C53035082.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C160404.html</x:v>
       </x:c>
       <x:c r="I19" s="7" t="str">
-        <x:v>https://www.jdtfuse.com/upload/PDF/JFC1032TS.pdf</x:v>
+        <x:v>https://www.jst-mfg.com/product/pdf/eng/eSH.pdf</x:v>
       </x:c>
       <x:c r="J19" s="7" t="str">
-        <x:v>JFC1032-1200TS</x:v>
+        <x:v>SM04B-SRSS-TB(LF)(SN)</x:v>
       </x:c>
       <x:c r="K19" s="7" t="str">
-        <x:v>JDTfuse</x:v>
+        <x:v>JST</x:v>
       </x:c>
       <x:c r="L19" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M19" s="7" t="str">
-        <x:v>Corrected centered origin and JDT land pattern. Check the new placement preview.</x:v>
+        <x:v>Standard Qwiic pin order: 1 GND, 2 3.3 V, 3 SDA, 4 SCL. J9 is the dedicated MASTER port; J1/J12/J17 power local SENSOR modules. J9 power/signal nets are separated by U13.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="53" customHeight="1">
-      <x:c r="A20" s="7" t="str">
-        <x:v>JST SH 4-pin 1.00mm</x:v>
-      </x:c>
-      <x:c r="B20" s="7" t="str">
-        <x:v>J1,J9,J12,J17</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="str">
-        <x:v>Connector_JST:JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</x:v>
-      </x:c>
-      <x:c r="D20" s="7" t="str">
-        <x:v>C160404</x:v>
-      </x:c>
-      <x:c r="E20" s="8" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F20" s="9" t="n">
-        <x:v>0.6</x:v>
-      </x:c>
-      <x:c r="G20" s="9" t="n">
+      <x:c r="A20" s="11" t="str">
+        <x:v>PJ-082BH</x:v>
+      </x:c>
+      <x:c r="B20" s="11" t="str">
+        <x:v>J2</x:v>
+      </x:c>
+      <x:c r="C20" s="11" t="str">
+        <x:v>RheoBoard:PJ-082BH</x:v>
+      </x:c>
+      <x:c r="D20" s="11" t="str">
+        <x:v>C3094233</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F20" s="13" t="n">
+        <x:v>1.58</x:v>
+      </x:c>
+      <x:c r="G20" s="13" t="n">
         <x:f>IF(ISNUMBER(F20),E20*F20,"")</x:f>
-        <x:v>2.4</x:v>
-      </x:c>
-      <x:c r="H20" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C160404.html</x:v>
-      </x:c>
-      <x:c r="I20" s="7" t="str">
-        <x:v>https://www.jst-mfg.com/product/pdf/eng/eSH.pdf</x:v>
-      </x:c>
-      <x:c r="J20" s="7" t="str">
-        <x:v>SM04B-SRSS-TB(LF)(SN)</x:v>
-      </x:c>
-      <x:c r="K20" s="7" t="str">
-        <x:v>JST</x:v>
-      </x:c>
-      <x:c r="L20" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M20" s="7" t="str">
-        <x:v>Standard Qwiic pin order: 1 GND, 2 3.3 V, 3 SDA, 4 SCL. J9 is the dedicated MASTER port; J1/J12/J17 power local SENSOR modules. J9 power/signal nets are separated by U13.</x:v>
+        <x:v>1.58</x:v>
+      </x:c>
+      <x:c r="H20" s="11" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C3094233.html</x:v>
+      </x:c>
+      <x:c r="I20" s="11" t="str">
+        <x:v>https://www.sameskydevices.com/product/resource/pj-082bh.pdf</x:v>
+      </x:c>
+      <x:c r="J20" s="11" t="str">
+        <x:v>PJ-082BH</x:v>
+      </x:c>
+      <x:c r="K20" s="11" t="str">
+        <x:v>CUI</x:v>
+      </x:c>
+      <x:c r="L20" s="11" t="str">
+        <x:v>Manual THT</x:v>
+      </x:c>
+      <x:c r="M20" s="11" t="str">
+        <x:v>Manual through-hole assembly. Center-positive 12 V, 5.5 x 2.5 mm mating plug.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="53" customHeight="1">
       <x:c r="A21" s="11" t="str">
-        <x:v>PJ-082BH</x:v>
+        <x:v>JST EH 4-pin 2.50mm</x:v>
       </x:c>
       <x:c r="B21" s="11" t="str">
-        <x:v>J2</x:v>
+        <x:v>J3</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
-        <x:v>RheoBoard:PJ-082BH</x:v>
+        <x:v>Connector_JST:JST_EH_B4B-EH-A_1x04_P2.50mm_Vertical</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
-        <x:v>C3094233</x:v>
+        <x:v>C160258</x:v>
       </x:c>
       <x:c r="E21" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F21" s="13" t="n">
-        <x:v>1.58</x:v>
+        <x:v>0.139</x:v>
       </x:c>
       <x:c r="G21" s="13" t="n">
         <x:f>IF(ISNUMBER(F21),E21*F21,"")</x:f>
-        <x:v>1.58</x:v>
+        <x:v>0.139</x:v>
       </x:c>
       <x:c r="H21" s="11" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C3094233.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C160258.html</x:v>
       </x:c>
       <x:c r="I21" s="11" t="str">
-        <x:v>https://www.sameskydevices.com/product/resource/pj-082bh.pdf</x:v>
+        <x:v>https://www.jst-mfg.com/product/pdf/eng/eEH.pdf</x:v>
       </x:c>
       <x:c r="J21" s="11" t="str">
-        <x:v>PJ-082BH</x:v>
+        <x:v>B4B-EH-A(LF)(SN)</x:v>
       </x:c>
       <x:c r="K21" s="11" t="str">
-        <x:v>CUI</x:v>
+        <x:v>JST</x:v>
       </x:c>
       <x:c r="L21" s="11" t="str">
         <x:v>Manual THT</x:v>
       </x:c>
       <x:c r="M21" s="11" t="str">
-        <x:v>Manual through-hole assembly. Center-positive 12 V, 5.5 x 2.5 mm mating plug.</x:v>
+        <x:v>Manual through-hole assembly. Pin 2 supplies local 3.3 V to peripherals.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="53" customHeight="1">
-      <x:c r="A22" s="11" t="str">
-        <x:v>JST EH 4-pin 2.50mm</x:v>
-      </x:c>
-      <x:c r="B22" s="11" t="str">
-        <x:v>J3</x:v>
-      </x:c>
-      <x:c r="C22" s="11" t="str">
-        <x:v>Connector_JST:JST_EH_B4B-EH-A_1x04_P2.50mm_Vertical</x:v>
-      </x:c>
-      <x:c r="D22" s="11" t="str">
-        <x:v>C160258</x:v>
-      </x:c>
-      <x:c r="E22" s="12" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F22" s="13" t="n">
-        <x:v>0.139</x:v>
-      </x:c>
-      <x:c r="G22" s="13" t="n">
+      <x:c r="A22" s="7" t="str">
+        <x:v>4.7uH FXL0530-4R7-M</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="str">
+        <x:v>L1, L2, L5</x:v>
+      </x:c>
+      <x:c r="C22" s="7" t="str">
+        <x:v>Inductor_SMD:L_Changjiang_FXL0530</x:v>
+      </x:c>
+      <x:c r="D22" s="7" t="str">
+        <x:v>C177246</x:v>
+      </x:c>
+      <x:c r="E22" s="8" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F22" s="9" t="n">
+        <x:v>0.904</x:v>
+      </x:c>
+      <x:c r="G22" s="9" t="n">
         <x:f>IF(ISNUMBER(F22),E22*F22,"")</x:f>
-        <x:v>0.139</x:v>
-      </x:c>
-      <x:c r="H22" s="11" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C160258.html</x:v>
-      </x:c>
-      <x:c r="I22" s="11" t="str">
-        <x:v>https://www.jst-mfg.com/product/pdf/eng/eEH.pdf</x:v>
-      </x:c>
-      <x:c r="J22" s="11" t="str">
-        <x:v>B4B-EH-A(LF)(SN)</x:v>
-      </x:c>
-      <x:c r="K22" s="11" t="str">
-        <x:v>JST</x:v>
-      </x:c>
-      <x:c r="L22" s="11" t="str">
-        <x:v>Manual THT</x:v>
-      </x:c>
-      <x:c r="M22" s="11" t="str">
-        <x:v>Manual through-hole assembly. Pin 2 supplies local 3.3 V to peripherals.</x:v>
+        <x:v>2.712</x:v>
+      </x:c>
+      <x:c r="H22" s="7" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C177246.html</x:v>
+      </x:c>
+      <x:c r="I22" s="7"/>
+      <x:c r="J22" s="7" t="str">
+        <x:v>FXL0530-4R7-M</x:v>
+      </x:c>
+      <x:c r="K22" s="7" t="str">
+        <x:v>cjiang</x:v>
+      </x:c>
+      <x:c r="L22" s="7" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M22" s="7" t="str">
+        <x:v>FXL0530 pads match the selected inductor; old Bourns purchasing link removed.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="53" customHeight="1">
       <x:c r="A23" s="7" t="str">
-        <x:v>4.7uH FXL0530-4R7-M</x:v>
+        <x:v>AO3400A</x:v>
       </x:c>
       <x:c r="B23" s="7" t="str">
-        <x:v>L1,L2,L5</x:v>
+        <x:v>Q3, Q4, Q8, Q10</x:v>
       </x:c>
       <x:c r="C23" s="7" t="str">
-        <x:v>Inductor_SMD:L_Changjiang_FXL0530</x:v>
+        <x:v>RheoBoard:AO3400A</x:v>
       </x:c>
       <x:c r="D23" s="7" t="str">
-        <x:v>C177246</x:v>
+        <x:v>C20917</x:v>
       </x:c>
       <x:c r="E23" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F23" s="9" t="n">
-        <x:v>0.904</x:v>
+        <x:v>0.322</x:v>
       </x:c>
       <x:c r="G23" s="9" t="n">
         <x:f>IF(ISNUMBER(F23),E23*F23,"")</x:f>
-        <x:v>2.712</x:v>
+        <x:v>1.288</x:v>
       </x:c>
       <x:c r="H23" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C177246.html</x:v>
-      </x:c>
-      <x:c r="I23" s="7"/>
+        <x:v>https://www.lcsc.com/product-detail/C20917.html</x:v>
+      </x:c>
+      <x:c r="I23" s="7" t="str">
+        <x:v>https://www.aosmd.com/sites/default/files/res/data_sheets/AO3400A.pdf</x:v>
+      </x:c>
       <x:c r="J23" s="7" t="str">
-        <x:v>FXL0530-4R7-M</x:v>
+        <x:v>AO3400A</x:v>
       </x:c>
       <x:c r="K23" s="7" t="str">
-        <x:v>cjiang</x:v>
+        <x:v>AOS</x:v>
       </x:c>
       <x:c r="L23" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M23" s="7" t="str">
-        <x:v>FXL0530 pads match the selected inductor; old Bourns purchasing link removed.</x:v>
-      </x:c>
+      <x:c r="M23" s="7"/>
     </x:row>
     <x:row r="24" ht="53" customHeight="1">
       <x:c r="A24" s="7" t="str">
-        <x:v>AO3400A</x:v>
+        <x:v>100K/0603/1%</x:v>
       </x:c>
       <x:c r="B24" s="7" t="str">
-        <x:v>Q3,Q4,Q8,Q10</x:v>
+        <x:v>R1, R4, R7</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
-        <x:v>RheoBoard:AO3400A</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D24" s="7" t="str">
-        <x:v>C20917</x:v>
+        <x:v>C25803</x:v>
       </x:c>
       <x:c r="E24" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F24" s="9" t="n">
-        <x:v>0.322</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="G24" s="9" t="n">
         <x:f>IF(ISNUMBER(F24),E24*F24,"")</x:f>
-        <x:v>1.288</x:v>
+        <x:v>0.042</x:v>
       </x:c>
       <x:c r="H24" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C20917.html</x:v>
-      </x:c>
-      <x:c r="I24" s="7" t="str">
-        <x:v>https://www.aosmd.com/sites/default/files/res/data_sheets/AO3400A.pdf</x:v>
-      </x:c>
+        <x:v>https://www.lcsc.com/product-detail/C25803.html</x:v>
+      </x:c>
+      <x:c r="I24" s="7"/>
       <x:c r="J24" s="7" t="str">
-        <x:v>AO3400A</x:v>
+        <x:v>0603WAF1003T5E</x:v>
       </x:c>
       <x:c r="K24" s="7" t="str">
-        <x:v>AOS</x:v>
+        <x:v>UNI-ROYAL</x:v>
       </x:c>
       <x:c r="L24" s="7" t="str">
         <x:v>SMT</x:v>
@@ -1351,33 +1359,33 @@
     </x:row>
     <x:row r="25" ht="53" customHeight="1">
       <x:c r="A25" s="7" t="str">
-        <x:v>100K/0603/1%</x:v>
+        <x:v>4K7/0603/1%</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
-        <x:v>R1,R4,R7</x:v>
+        <x:v>R15, R20, R82, R83</x:v>
       </x:c>
       <x:c r="C25" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D25" s="7" t="str">
-        <x:v>C25803</x:v>
+        <x:v>C23162</x:v>
       </x:c>
       <x:c r="E25" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F25" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="G25" s="9" t="n">
         <x:f>IF(ISNUMBER(F25),E25*F25,"")</x:f>
-        <x:v>0.042</x:v>
+        <x:v>0.004</x:v>
       </x:c>
       <x:c r="H25" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25803.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C23162.html</x:v>
       </x:c>
       <x:c r="I25" s="7"/>
       <x:c r="J25" s="7" t="str">
-        <x:v>0603WAF1003T5E</x:v>
+        <x:v>0603WAF4701T5E</x:v>
       </x:c>
       <x:c r="K25" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1385,37 +1393,39 @@
       <x:c r="L25" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M25" s="7" t="str"/>
-    </x:row>
-    <x:row r="26" ht="53" customHeight="1">
+      <x:c r="M25" s="7" t="str">
+        <x:v>R82/R83 added as 4.7 kohm host SDA/SCL pullups; local R15/R20 retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="126" customHeight="1">
       <x:c r="A26" s="7" t="str">
-        <x:v>2K2/0603/1%</x:v>
+        <x:v>10K/0603/1%</x:v>
       </x:c>
       <x:c r="B26" s="7" t="str">
-        <x:v>R10</x:v>
+        <x:v>R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84, R85</x:v>
       </x:c>
       <x:c r="C26" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D26" s="7" t="str">
-        <x:v>C4190</x:v>
+        <x:v>C25804</x:v>
       </x:c>
       <x:c r="E26" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F26" s="9" t="n">
         <x:v>0.014</x:v>
       </x:c>
       <x:c r="G26" s="9" t="n">
         <x:f>IF(ISNUMBER(F26),E26*F26,"")</x:f>
-        <x:v>0.014</x:v>
+        <x:v>0.252</x:v>
       </x:c>
       <x:c r="H26" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C4190.html</x:v>
-      </x:c>
-      <x:c r="I26" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C25804.html</x:v>
+      </x:c>
+      <x:c r="I26" s="7"/>
       <x:c r="J26" s="7" t="str">
-        <x:v>0603WAF2201T5E</x:v>
+        <x:v>0603WAF1002T5E</x:v>
       </x:c>
       <x:c r="K26" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1423,37 +1433,39 @@
       <x:c r="L26" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M26" s="7" t="str"/>
+      <x:c r="M26" s="7" t="str">
+        <x:v>R16–R19 pull the button signals to HOST_3V3 from J9. R84 discharges HOST_3V3. R85 pulls Q11 gate to GND.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="53" customHeight="1">
       <x:c r="A27" s="7" t="str">
-        <x:v>4K7/0603/1%</x:v>
+        <x:v>1k/0603/1%</x:v>
       </x:c>
       <x:c r="B27" s="7" t="str">
-        <x:v>R11, R15, R20, R82, R83</x:v>
+        <x:v>R24, R25, R26, R39, R40, R54, R59, R75</x:v>
       </x:c>
       <x:c r="C27" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D27" s="7" t="str">
-        <x:v>C23162</x:v>
+        <x:v>C21190</x:v>
       </x:c>
       <x:c r="E27" s="8" t="n">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F27" s="9" t="n">
         <x:v>0.001</x:v>
       </x:c>
       <x:c r="G27" s="9" t="n">
         <x:f>IF(ISNUMBER(F27),E27*F27,"")</x:f>
-        <x:v>0.005</x:v>
+        <x:v>0.008</x:v>
       </x:c>
       <x:c r="H27" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C23162.html</x:v>
-      </x:c>
-      <x:c r="I27" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C21190.html</x:v>
+      </x:c>
+      <x:c r="I27" s="7"/>
       <x:c r="J27" s="7" t="str">
-        <x:v>0603WAF4701T5E</x:v>
+        <x:v>0603WAF1001T5E</x:v>
       </x:c>
       <x:c r="K27" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1461,39 +1473,37 @@
       <x:c r="L27" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M27" s="7" t="str">
-        <x:v>R82/R83 added as 4.7 kohm host SDA/SCL pullups; local R15/R20 retained.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="126" customHeight="1">
+      <x:c r="M27" s="7"/>
+    </x:row>
+    <x:row r="28" ht="53" customHeight="1">
       <x:c r="A28" s="7" t="str">
-        <x:v>10K/0603/1%</x:v>
+        <x:v>100R/0603/1%</x:v>
       </x:c>
       <x:c r="B28" s="7" t="str">
-        <x:v>R13, R14, R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84, R85</x:v>
+        <x:v>R35, R36, R42, R55</x:v>
       </x:c>
       <x:c r="C28" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D28" s="7" t="str">
-        <x:v>C25804</x:v>
+        <x:v>C22775</x:v>
       </x:c>
       <x:c r="E28" s="8" t="n">
-        <x:v>20</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F28" s="9" t="n">
         <x:v>0.014</x:v>
       </x:c>
       <x:c r="G28" s="9" t="n">
         <x:f>IF(ISNUMBER(F28),E28*F28,"")</x:f>
-        <x:v>0.28</x:v>
+        <x:v>0.056</x:v>
       </x:c>
       <x:c r="H28" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25804.html</x:v>
-      </x:c>
-      <x:c r="I28" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C22775.html</x:v>
+      </x:c>
+      <x:c r="I28" s="7"/>
       <x:c r="J28" s="7" t="str">
-        <x:v>0603WAF1002T5E</x:v>
+        <x:v>0603WAF1000T5E</x:v>
       </x:c>
       <x:c r="K28" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1501,39 +1511,37 @@
       <x:c r="L28" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M28" s="7" t="str">
-        <x:v>R84 discharges HOST_3V3. R85 pulls Q11 gate to GND for reverse-polarity protection.</x:v>
-      </x:c>
+      <x:c r="M28" s="7"/>
     </x:row>
     <x:row r="29" ht="53" customHeight="1">
       <x:c r="A29" s="7" t="str">
-        <x:v>1k/0603/1%</x:v>
+        <x:v>330/0603/1%</x:v>
       </x:c>
       <x:c r="B29" s="7" t="str">
-        <x:v>R24,R25,R26,R39,R40,R54,R59,R75</x:v>
+        <x:v>R44, R77</x:v>
       </x:c>
       <x:c r="C29" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D29" s="7" t="str">
-        <x:v>C21190</x:v>
+        <x:v>C23138</x:v>
       </x:c>
       <x:c r="E29" s="8" t="n">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F29" s="9" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="G29" s="9" t="n">
         <x:f>IF(ISNUMBER(F29),E29*F29,"")</x:f>
-        <x:v>0.008</x:v>
+        <x:v>0.028</x:v>
       </x:c>
       <x:c r="H29" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C21190.html</x:v>
-      </x:c>
-      <x:c r="I29" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C23138.html</x:v>
+      </x:c>
+      <x:c r="I29" s="7"/>
       <x:c r="J29" s="7" t="str">
-        <x:v>0603WAF1001T5E</x:v>
+        <x:v>0603WAF3300T5E</x:v>
       </x:c>
       <x:c r="K29" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1545,71 +1553,73 @@
     </x:row>
     <x:row r="30" ht="53" customHeight="1">
       <x:c r="A30" s="7" t="str">
-        <x:v>100R/0603/1%</x:v>
+        <x:v>196k ±1%</x:v>
       </x:c>
       <x:c r="B30" s="7" t="str">
-        <x:v>R35,R36,R42,R55</x:v>
+        <x:v>R45</x:v>
       </x:c>
       <x:c r="C30" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D30" s="7" t="str">
-        <x:v>C22775</x:v>
+        <x:v>C4203218</x:v>
       </x:c>
       <x:c r="E30" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F30" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="G30" s="9" t="n">
         <x:f>IF(ISNUMBER(F30),E30*F30,"")</x:f>
-        <x:v>0.056</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="H30" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22775.html</x:v>
-      </x:c>
-      <x:c r="I30" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C4203218.html</x:v>
+      </x:c>
+      <x:c r="I30" s="7"/>
       <x:c r="J30" s="7" t="str">
-        <x:v>0603WAF1000T5E</x:v>
+        <x:v>CRCW0603196KFKEA</x:v>
       </x:c>
       <x:c r="K30" s="7" t="str">
-        <x:v>UNI-ROYAL</x:v>
+        <x:v>VISHAY</x:v>
       </x:c>
       <x:c r="L30" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M30" s="7" t="str"/>
+      <x:c r="M30" s="7" t="str">
+        <x:v>Schematic corrected to the assembled 196k value; pump rail approximately 4.52 V.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="53" customHeight="1">
       <x:c r="A31" s="7" t="str">
-        <x:v>330/0603/1%</x:v>
+        <x:v>30K/0603/1%</x:v>
       </x:c>
       <x:c r="B31" s="7" t="str">
-        <x:v>R44,R77</x:v>
+        <x:v>R46, R74, R76</x:v>
       </x:c>
       <x:c r="C31" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D31" s="7" t="str">
-        <x:v>C23138</x:v>
+        <x:v>C22984</x:v>
       </x:c>
       <x:c r="E31" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F31" s="9" t="n">
         <x:v>0.014</x:v>
       </x:c>
       <x:c r="G31" s="9" t="n">
         <x:f>IF(ISNUMBER(F31),E31*F31,"")</x:f>
-        <x:v>0.028</x:v>
+        <x:v>0.042</x:v>
       </x:c>
       <x:c r="H31" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C23138.html</x:v>
-      </x:c>
-      <x:c r="I31" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C22984.html</x:v>
+      </x:c>
+      <x:c r="I31" s="7"/>
       <x:c r="J31" s="7" t="str">
-        <x:v>0603WAF3300T5E</x:v>
+        <x:v>0603WAF3002T5E</x:v>
       </x:c>
       <x:c r="K31" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1617,80 +1627,78 @@
       <x:c r="L31" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M31" s="7" t="str"/>
+      <x:c r="M31" s="7"/>
     </x:row>
     <x:row r="32" ht="53" customHeight="1">
       <x:c r="A32" s="7" t="str">
-        <x:v>196k ±1%</x:v>
+        <x:v>270K/0603/1%</x:v>
       </x:c>
       <x:c r="B32" s="7" t="str">
-        <x:v>R45</x:v>
+        <x:v>R60</x:v>
       </x:c>
       <x:c r="C32" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D32" s="7" t="str">
-        <x:v>C4203218</x:v>
+        <x:v>C22965</x:v>
       </x:c>
       <x:c r="E32" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F32" s="9" t="n">
-        <x:v>0.02</x:v>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="G32" s="9" t="n">
         <x:f>IF(ISNUMBER(F32),E32*F32,"")</x:f>
-        <x:v>0.02</x:v>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="H32" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C4203218.html</x:v>
-      </x:c>
-      <x:c r="I32" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C22965.html</x:v>
+      </x:c>
+      <x:c r="I32" s="7"/>
       <x:c r="J32" s="7" t="str">
-        <x:v>CRCW0603196KFKEA</x:v>
+        <x:v>0603WAF2703T5E</x:v>
       </x:c>
       <x:c r="K32" s="7" t="str">
-        <x:v>VISHAY</x:v>
+        <x:v>UNI-ROYAL</x:v>
       </x:c>
       <x:c r="L32" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M32" s="7" t="str">
-        <x:v>Schematic corrected to the assembled 196k value; pump rail approximately 4.52 V.</x:v>
-      </x:c>
+      <x:c r="M32" s="7"/>
     </x:row>
     <x:row r="33" ht="53" customHeight="1">
       <x:c r="A33" s="7" t="str">
-        <x:v>30K/0603/1%</x:v>
+        <x:v>135k ±0.1%</x:v>
       </x:c>
       <x:c r="B33" s="7" t="str">
-        <x:v>R46,R74,R76</x:v>
+        <x:v>R61</x:v>
       </x:c>
       <x:c r="C33" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D33" s="7" t="str">
-        <x:v>C22984</x:v>
+        <x:v>C861113</x:v>
       </x:c>
       <x:c r="E33" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F33" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.06</x:v>
       </x:c>
       <x:c r="G33" s="9" t="n">
         <x:f>IF(ISNUMBER(F33),E33*F33,"")</x:f>
-        <x:v>0.042</x:v>
+        <x:v>0.06</x:v>
       </x:c>
       <x:c r="H33" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22984.html</x:v>
-      </x:c>
-      <x:c r="I33" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C861113.html</x:v>
+      </x:c>
+      <x:c r="I33" s="7"/>
       <x:c r="J33" s="7" t="str">
-        <x:v>0603WAF3002T5E</x:v>
+        <x:v>RT0603BRD07135KL</x:v>
       </x:c>
       <x:c r="K33" s="7" t="str">
-        <x:v>UNI-ROYAL</x:v>
+        <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="L33" s="7" t="str">
         <x:v>SMT</x:v>
@@ -1699,33 +1707,33 @@
     </x:row>
     <x:row r="34" ht="53" customHeight="1">
       <x:c r="A34" s="7" t="str">
-        <x:v>270K/0603/1%</x:v>
+        <x:v>549R ±1%</x:v>
       </x:c>
       <x:c r="B34" s="7" t="str">
-        <x:v>R60</x:v>
+        <x:v>R73</x:v>
       </x:c>
       <x:c r="C34" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D34" s="7" t="str">
-        <x:v>C22965</x:v>
+        <x:v>C23079</x:v>
       </x:c>
       <x:c r="E34" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F34" s="9" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="G34" s="9" t="n">
         <x:f>IF(ISNUMBER(F34),E34*F34,"")</x:f>
-        <x:v>0.001</x:v>
+        <x:v>0.014</x:v>
       </x:c>
       <x:c r="H34" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22965.html</x:v>
-      </x:c>
-      <x:c r="I34" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C23079.html</x:v>
+      </x:c>
+      <x:c r="I34" s="7"/>
       <x:c r="J34" s="7" t="str">
-        <x:v>0603WAF2703T5E</x:v>
+        <x:v>0603WAF5490T5E</x:v>
       </x:c>
       <x:c r="K34" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1733,58 +1741,57 @@
       <x:c r="L34" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M34" s="7" t="str"/>
+      <x:c r="M34" s="7" t="str">
+        <x:v>Schematic corrected to the assembled 549 ohm value.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="53" customHeight="1">
       <x:c r="A35" s="7" t="str">
-        <x:v>135k ±0.1%</x:v>
+        <x:v>680k ±1%</x:v>
       </x:c>
       <x:c r="B35" s="7" t="str">
-        <x:v>R61</x:v>
+        <x:v>R78</x:v>
       </x:c>
       <x:c r="C35" s="7" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D35" s="7" t="str">
-        <x:v>C861113</x:v>
+        <x:v>C25822</x:v>
       </x:c>
       <x:c r="E35" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F35" s="9" t="n">
-        <x:v>0.06</x:v>
-      </x:c>
-      <x:c r="G35" s="9" t="n">
+      <x:c r="F35" s="10"/>
+      <x:c r="G35" s="9" t="str">
         <x:f>IF(ISNUMBER(F35),E35*F35,"")</x:f>
-        <x:v>0.06</x:v>
       </x:c>
       <x:c r="H35" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C861113.html</x:v>
-      </x:c>
-      <x:c r="I35" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C25822.html</x:v>
+      </x:c>
+      <x:c r="I35" s="7"/>
       <x:c r="J35" s="7" t="str">
-        <x:v>RT0603BRD07135KL</x:v>
+        <x:v>0603WAF6803T5E</x:v>
       </x:c>
       <x:c r="K35" s="7" t="str">
-        <x:v>YAGEO</x:v>
+        <x:v>UNI-ROYAL</x:v>
       </x:c>
       <x:c r="L35" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M35" s="7" t="str"/>
+      <x:c r="M35" s="7"/>
     </x:row>
     <x:row r="36" ht="53" customHeight="1">
       <x:c r="A36" s="7" t="str">
-        <x:v>549R ±1%</x:v>
+        <x:v>100K/0603/1%</x:v>
       </x:c>
       <x:c r="B36" s="7" t="str">
-        <x:v>R73</x:v>
+        <x:v>R79</x:v>
       </x:c>
       <x:c r="C36" s="7" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D36" s="7" t="str">
-        <x:v>C23079</x:v>
+        <x:v>C25803</x:v>
       </x:c>
       <x:c r="E36" s="8" t="n">
         <x:v>1</x:v>
@@ -1797,11 +1804,11 @@
         <x:v>0.014</x:v>
       </x:c>
       <x:c r="H36" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C23079.html</x:v>
-      </x:c>
-      <x:c r="I36" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C25803.html</x:v>
+      </x:c>
+      <x:c r="I36" s="7"/>
       <x:c r="J36" s="7" t="str">
-        <x:v>0603WAF5490T5E</x:v>
+        <x:v>0603WAF1003T5E</x:v>
       </x:c>
       <x:c r="K36" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1809,22 +1816,20 @@
       <x:c r="L36" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M36" s="7" t="str">
-        <x:v>Schematic corrected to the assembled 549 ohm value.</x:v>
-      </x:c>
+      <x:c r="M36" s="7"/>
     </x:row>
     <x:row r="37" ht="53" customHeight="1">
       <x:c r="A37" s="7" t="str">
-        <x:v>680k ±1%</x:v>
+        <x:v>390k ±1%</x:v>
       </x:c>
       <x:c r="B37" s="7" t="str">
-        <x:v>R78</x:v>
+        <x:v>R80</x:v>
       </x:c>
       <x:c r="C37" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D37" s="7" t="str">
-        <x:v>C25822</x:v>
+        <x:v>C2759410</x:v>
       </x:c>
       <x:c r="E37" s="8" t="n">
         <x:v>1</x:v>
@@ -1834,11 +1839,11 @@
         <x:f>IF(ISNUMBER(F37),E37*F37,"")</x:f>
       </x:c>
       <x:c r="H37" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25822.html</x:v>
-      </x:c>
-      <x:c r="I37" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C2759410.html</x:v>
+      </x:c>
+      <x:c r="I37" s="7"/>
       <x:c r="J37" s="7" t="str">
-        <x:v>0603WAF6803T5E</x:v>
+        <x:v>HP03W5F3903T5E</x:v>
       </x:c>
       <x:c r="K37" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1850,33 +1855,30 @@
     </x:row>
     <x:row r="38" ht="53" customHeight="1">
       <x:c r="A38" s="7" t="str">
-        <x:v>100K/0603/1%</x:v>
+        <x:v>1.65k ±1%</x:v>
       </x:c>
       <x:c r="B38" s="7" t="str">
-        <x:v>R79</x:v>
+        <x:v>R81</x:v>
       </x:c>
       <x:c r="C38" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D38" s="7" t="str">
-        <x:v>C25803</x:v>
+        <x:v>C22845</x:v>
       </x:c>
       <x:c r="E38" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F38" s="9" t="n">
-        <x:v>0.014</x:v>
-      </x:c>
-      <x:c r="G38" s="9" t="n">
+      <x:c r="F38" s="10"/>
+      <x:c r="G38" s="9" t="str">
         <x:f>IF(ISNUMBER(F38),E38*F38,"")</x:f>
-        <x:v>0.014</x:v>
       </x:c>
       <x:c r="H38" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25803.html</x:v>
-      </x:c>
-      <x:c r="I38" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C22845.html</x:v>
+      </x:c>
+      <x:c r="I38" s="7"/>
       <x:c r="J38" s="7" t="str">
-        <x:v>0603WAF1003T5E</x:v>
+        <x:v>0603WAF1651T5E</x:v>
       </x:c>
       <x:c r="K38" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1884,488 +1886,445 @@
       <x:c r="L38" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M38" s="7" t="str"/>
+      <x:c r="M38" s="7"/>
     </x:row>
     <x:row r="39" ht="53" customHeight="1">
       <x:c r="A39" s="7" t="str">
-        <x:v>390k ±1%</x:v>
+        <x:v>TL3301NF160QG/P010515</x:v>
       </x:c>
       <x:c r="B39" s="7" t="str">
-        <x:v>R80</x:v>
+        <x:v>SW1, SW2, SW3, SW4</x:v>
       </x:c>
       <x:c r="C39" s="7" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
+        <x:v>RheoBoard:Tactile_Switch_4pad</x:v>
       </x:c>
       <x:c r="D39" s="7" t="str">
-        <x:v>C2759410</x:v>
+        <x:v>C273527</x:v>
       </x:c>
       <x:c r="E39" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F39" s="10"/>
-      <x:c r="G39" s="9" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F39" s="9" t="n">
+        <x:v>0.183</x:v>
+      </x:c>
+      <x:c r="G39" s="9" t="n">
         <x:f>IF(ISNUMBER(F39),E39*F39,"")</x:f>
+        <x:v>0.732</x:v>
       </x:c>
       <x:c r="H39" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C2759410.html</x:v>
-      </x:c>
-      <x:c r="I39" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C273527.html</x:v>
+      </x:c>
+      <x:c r="I39" s="7"/>
       <x:c r="J39" s="7" t="str">
-        <x:v>HP03W5F3903T5E</x:v>
+        <x:v>TL3301NF160QG/P010515</x:v>
       </x:c>
       <x:c r="K39" s="7" t="str">
-        <x:v>UNI-ROYAL</x:v>
+        <x:v>E-Switch</x:v>
       </x:c>
       <x:c r="L39" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M39" s="7" t="str"/>
+      <x:c r="M39" s="7"/>
     </x:row>
     <x:row r="40" ht="53" customHeight="1">
       <x:c r="A40" s="7" t="str">
-        <x:v>1.65k ±1%</x:v>
+        <x:v>TPS563203DRLR</x:v>
       </x:c>
       <x:c r="B40" s="7" t="str">
-        <x:v>R81</x:v>
+        <x:v>U1, U2, U3</x:v>
       </x:c>
       <x:c r="C40" s="7" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
+        <x:v>RheoBoard:TPS563203DRLR</x:v>
       </x:c>
       <x:c r="D40" s="7" t="str">
-        <x:v>C22845</x:v>
+        <x:v>C22445512</x:v>
       </x:c>
       <x:c r="E40" s="8" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F40" s="9" t="n">
+        <x:v>0.225</x:v>
+      </x:c>
+      <x:c r="G40" s="9" t="n">
+        <x:f>IF(ISNUMBER(F40),E40*F40,"")</x:f>
+        <x:v>0.675</x:v>
+      </x:c>
+      <x:c r="H40" s="7" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C22445512.html</x:v>
+      </x:c>
+      <x:c r="I40" s="7" t="str">
+        <x:v>https://www.ti.com/lit/gpn/tps563203</x:v>
+      </x:c>
+      <x:c r="J40" s="7" t="str">
+        <x:v>TPS563203DRLR</x:v>
+      </x:c>
+      <x:c r="K40" s="7" t="str">
+        <x:v>TI</x:v>
+      </x:c>
+      <x:c r="L40" s="7" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M40" s="7"/>
+    </x:row>
+    <x:row r="41" ht="68" customHeight="1">
+      <x:c r="A41" s="7" t="str">
+        <x:v>MPRLS0025PA00001A</x:v>
+      </x:c>
+      <x:c r="B41" s="7" t="str">
+        <x:v>U5</x:v>
+      </x:c>
+      <x:c r="C41" s="7" t="str">
+        <x:v>RheoBoard:MPRLS0025PA00001A</x:v>
+      </x:c>
+      <x:c r="D41" s="7" t="str">
+        <x:v>C3257154</x:v>
+      </x:c>
+      <x:c r="E41" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F40" s="10"/>
-      <x:c r="G40" s="9" t="str">
-        <x:f>IF(ISNUMBER(F40),E40*F40,"")</x:f>
-      </x:c>
-      <x:c r="H40" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22845.html</x:v>
-      </x:c>
-      <x:c r="I40" s="7" t="str"/>
-      <x:c r="J40" s="7" t="str">
-        <x:v>0603WAF1651T5E</x:v>
-      </x:c>
-      <x:c r="K40" s="7" t="str">
-        <x:v>UNI-ROYAL</x:v>
-      </x:c>
-      <x:c r="L40" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M40" s="7" t="str"/>
-    </x:row>
-    <x:row r="41" ht="53" customHeight="1">
-      <x:c r="A41" s="7" t="str">
-        <x:v>TL3301NF160QG/P010515</x:v>
-      </x:c>
-      <x:c r="B41" s="7" t="str">
-        <x:v>SW1,SW2,SW3,SW4</x:v>
-      </x:c>
-      <x:c r="C41" s="7" t="str">
-        <x:v>RheoBoard:Tactile_Switch_4pad</x:v>
-      </x:c>
-      <x:c r="D41" s="7" t="str">
-        <x:v>C273527</x:v>
-      </x:c>
-      <x:c r="E41" s="8" t="n">
-        <x:v>4</x:v>
-      </x:c>
       <x:c r="F41" s="9" t="n">
-        <x:v>0.183</x:v>
+        <x:v>15.93</x:v>
       </x:c>
       <x:c r="G41" s="9" t="n">
         <x:f>IF(ISNUMBER(F41),E41*F41,"")</x:f>
-        <x:v>0.732</x:v>
+        <x:v>15.93</x:v>
       </x:c>
       <x:c r="H41" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C273527.html</x:v>
-      </x:c>
-      <x:c r="I41" s="7" t="str"/>
+        <x:v>https://www.lcsc.com/product-detail/C3257154.html</x:v>
+      </x:c>
+      <x:c r="I41" s="7" t="str">
+        <x:v>https://automation.honeywell.com/content/dam/honeywell-edam/sps/ast/en-us/campaigns/pressure-sensors/documents/sps-siot-mpr-series-datasheet-32332628-ciid-172626.pdf</x:v>
+      </x:c>
       <x:c r="J41" s="7" t="str">
-        <x:v>TL3301NF160QG/P010515</x:v>
+        <x:v>MPRLS0025PA00001A</x:v>
       </x:c>
       <x:c r="K41" s="7" t="str">
-        <x:v>E-Switch</x:v>
+        <x:v>Honeywell</x:v>
       </x:c>
       <x:c r="L41" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M41" s="7" t="str"/>
+      <x:c r="M41" s="7"/>
     </x:row>
     <x:row r="42" ht="53" customHeight="1">
       <x:c r="A42" s="7" t="str">
-        <x:v>TPS563203DRLR</x:v>
+        <x:v>PCA9685PW,118</x:v>
       </x:c>
       <x:c r="B42" s="7" t="str">
-        <x:v>U1,U2,U3</x:v>
+        <x:v>U7</x:v>
       </x:c>
       <x:c r="C42" s="7" t="str">
-        <x:v>RheoBoard:TPS563203DRLR</x:v>
+        <x:v>RheoBoard:PCA9685</x:v>
       </x:c>
       <x:c r="D42" s="7" t="str">
-        <x:v>C22445512</x:v>
+        <x:v>C2678753</x:v>
       </x:c>
       <x:c r="E42" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F42" s="9" t="n">
-        <x:v>0.225</x:v>
+        <x:v>3.445</x:v>
       </x:c>
       <x:c r="G42" s="9" t="n">
         <x:f>IF(ISNUMBER(F42),E42*F42,"")</x:f>
-        <x:v>0.675</x:v>
+        <x:v>3.445</x:v>
       </x:c>
       <x:c r="H42" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22445512.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C2678753.html</x:v>
       </x:c>
       <x:c r="I42" s="7" t="str">
-        <x:v>https://www.ti.com/lit/gpn/tps563203</x:v>
+        <x:v>https://www.nxp.com/docs/en/data-sheet/PCA9685.pdf</x:v>
       </x:c>
       <x:c r="J42" s="7" t="str">
-        <x:v>TPS563203DRLR</x:v>
+        <x:v>PCA9685PW,118</x:v>
       </x:c>
       <x:c r="K42" s="7" t="str">
-        <x:v>TI</x:v>
+        <x:v>NXP</x:v>
       </x:c>
       <x:c r="L42" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M42" s="7" t="str"/>
+      <x:c r="M42" s="7" t="str">
+        <x:v>Pumps LED0/1, indicators LED2–4, valves LED5/6 using FULL ON/OFF. TCA9534 removed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="53" customHeight="1">
-      <x:c r="A43" s="7" t="str">
-        <x:v>TCA9534APWR</x:v>
-      </x:c>
-      <x:c r="B43" s="7" t="str">
-        <x:v>U4</x:v>
-      </x:c>
-      <x:c r="C43" s="7" t="str">
-        <x:v>RheoBoard:TCA9534APWR</x:v>
-      </x:c>
-      <x:c r="D43" s="7" t="str">
-        <x:v>C206010</x:v>
-      </x:c>
-      <x:c r="E43" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F43" s="9" t="n">
-        <x:v>1.27</x:v>
-      </x:c>
-      <x:c r="G43" s="9" t="n">
+      <x:c r="A43" s="11" t="str">
+        <x:v>ZR370-02PM / 4.5V / 2.5 LPM / ~500 mA</x:v>
+      </x:c>
+      <x:c r="B43" s="11" t="str">
+        <x:v>U8, U11</x:v>
+      </x:c>
+      <x:c r="C43" s="11" t="str">
+        <x:v>RheoBoard:PUMP</x:v>
+      </x:c>
+      <x:c r="D43" s="11"/>
+      <x:c r="E43" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F43" s="13" t="n">
+        <x:v>7.16</x:v>
+      </x:c>
+      <x:c r="G43" s="13" t="n">
         <x:f>IF(ISNUMBER(F43),E43*F43,"")</x:f>
-        <x:v>1.27</x:v>
-      </x:c>
-      <x:c r="H43" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C206010.html</x:v>
-      </x:c>
-      <x:c r="I43" s="7" t="str">
-        <x:v>https://www.ti.com/lit/ds/symlink/tca9534a.pdf</x:v>
-      </x:c>
-      <x:c r="J43" s="7" t="str">
-        <x:v>TCA9534APWR</x:v>
-      </x:c>
-      <x:c r="K43" s="7" t="str">
-        <x:v>TI</x:v>
-      </x:c>
-      <x:c r="L43" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M43" s="7" t="str"/>
-    </x:row>
-    <x:row r="44" ht="68" customHeight="1">
-      <x:c r="A44" s="7" t="str">
-        <x:v>MPRLS0025PA00001A</x:v>
-      </x:c>
-      <x:c r="B44" s="7" t="str">
-        <x:v>U5</x:v>
-      </x:c>
-      <x:c r="C44" s="7" t="str">
-        <x:v>RheoBoard:MPRLS0025PA00001A</x:v>
-      </x:c>
-      <x:c r="D44" s="7" t="str">
-        <x:v>C3257154</x:v>
-      </x:c>
-      <x:c r="E44" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F44" s="9" t="n">
-        <x:v>15.93</x:v>
-      </x:c>
-      <x:c r="G44" s="9" t="n">
+        <x:v>14.32</x:v>
+      </x:c>
+      <x:c r="H43" s="11" t="str">
+        <x:v>https://www.adafruit.com/product/4699</x:v>
+      </x:c>
+      <x:c r="I43" s="11"/>
+      <x:c r="J43" s="11" t="str">
+        <x:v>ZR370-02PM</x:v>
+      </x:c>
+      <x:c r="K43" s="11" t="str">
+        <x:v>Supplier-specified</x:v>
+      </x:c>
+      <x:c r="L43" s="11" t="str">
+        <x:v>Manual pump fitting</x:v>
+      </x:c>
+      <x:c r="M43" s="11" t="str">
+        <x:v>Existing pump retained for intermittent use. Manual fitting; provide mechanical support.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="53" customHeight="1">
+      <x:c r="A44" s="11" t="str">
+        <x:v>JST XH 2-pin 2.50mm</x:v>
+      </x:c>
+      <x:c r="B44" s="11" t="str">
+        <x:v>U9, U10</x:v>
+      </x:c>
+      <x:c r="C44" s="11" t="str">
+        <x:v>RheoBoard:VALVE_v105</x:v>
+      </x:c>
+      <x:c r="D44" s="11" t="str">
+        <x:v>C158012</x:v>
+      </x:c>
+      <x:c r="E44" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F44" s="10"/>
+      <x:c r="G44" s="13" t="str">
         <x:f>IF(ISNUMBER(F44),E44*F44,"")</x:f>
-        <x:v>15.93</x:v>
-      </x:c>
-      <x:c r="H44" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C3257154.html</x:v>
-      </x:c>
-      <x:c r="I44" s="7" t="str">
-        <x:v>https://automation.honeywell.com/content/dam/honeywell-edam/sps/ast/en-us/campaigns/pressure-sensors/documents/sps-siot-mpr-series-datasheet-32332628-ciid-172626.pdf</x:v>
-      </x:c>
-      <x:c r="J44" s="7" t="str">
-        <x:v>MPRLS0025PA00001A</x:v>
-      </x:c>
-      <x:c r="K44" s="7" t="str">
-        <x:v>Honeywell</x:v>
-      </x:c>
-      <x:c r="L44" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M44" s="7" t="str"/>
+      </x:c>
+      <x:c r="H44" s="11" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C158012.html</x:v>
+      </x:c>
+      <x:c r="I44" s="11" t="str">
+        <x:v>https://www.jst-mfg.com/product/pdf/eng/eXH.pdf</x:v>
+      </x:c>
+      <x:c r="J44" s="11" t="str">
+        <x:v>B2B-XH-A(LF)(SN)</x:v>
+      </x:c>
+      <x:c r="K44" s="11" t="str">
+        <x:v>JST</x:v>
+      </x:c>
+      <x:c r="L44" s="11" t="str">
+        <x:v>Manual THT</x:v>
+      </x:c>
+      <x:c r="M44" s="11" t="str">
+        <x:v>Fitted JST XH header only. External valve is listed on Manual accessories. Manual through-hole assembly.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="53" customHeight="1">
       <x:c r="A45" s="7" t="str">
-        <x:v>PCA9685PW,118</x:v>
+        <x:v>TPS259472ARPWR</x:v>
       </x:c>
       <x:c r="B45" s="7" t="str">
-        <x:v>U7</x:v>
+        <x:v>U12</x:v>
       </x:c>
       <x:c r="C45" s="7" t="str">
-        <x:v>RheoBoard:PCA9685</x:v>
+        <x:v>RheoBoard:TI_RPW0010A_VQFN-HR_2x2mm</x:v>
       </x:c>
       <x:c r="D45" s="7" t="str">
-        <x:v>C2678753</x:v>
+        <x:v>C3662789</x:v>
       </x:c>
       <x:c r="E45" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F45" s="9" t="n">
-        <x:v>3.445</x:v>
-      </x:c>
-      <x:c r="G45" s="9" t="n">
+      <x:c r="F45" s="10"/>
+      <x:c r="G45" s="9" t="str">
         <x:f>IF(ISNUMBER(F45),E45*F45,"")</x:f>
-        <x:v>3.445</x:v>
       </x:c>
       <x:c r="H45" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C2678753.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C3662789.html</x:v>
       </x:c>
       <x:c r="I45" s="7" t="str">
-        <x:v>https://www.nxp.com/docs/en/data-sheet/PCA9685.pdf</x:v>
+        <x:v>https://www.ti.com/lit/ds/symlink/tps25947.pdf</x:v>
       </x:c>
       <x:c r="J45" s="7" t="str">
-        <x:v>PCA9685PW,118</x:v>
+        <x:v>TPS259472ARPWR</x:v>
       </x:c>
       <x:c r="K45" s="7" t="str">
-        <x:v>NXP</x:v>
+        <x:v>Texas Instruments</x:v>
       </x:c>
       <x:c r="L45" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M45" s="7" t="str"/>
-    </x:row>
-    <x:row r="46" ht="53" customHeight="1">
-      <x:c r="A46" s="11" t="str">
-        <x:v>ZR370-02PM / 4.5V / 2.5 LPM / ~500 mA</x:v>
-      </x:c>
-      <x:c r="B46" s="11" t="str">
-        <x:v>U8,U11</x:v>
-      </x:c>
-      <x:c r="C46" s="11" t="str">
-        <x:v>RheoBoard:PUMP</x:v>
-      </x:c>
-      <x:c r="D46" s="11"/>
-      <x:c r="E46" s="12" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F46" s="13" t="n">
-        <x:v>7.16</x:v>
-      </x:c>
-      <x:c r="G46" s="13" t="n">
+      <x:c r="M45" s="7" t="str">
+        <x:v>New auto-retry input eFuse; TI RPW0010A HotRod footprint, approximately 2 A limit / 13.8 V clamp.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="112" customHeight="1">
+      <x:c r="A46" s="7" t="str">
+        <x:v>TCA9517ADGKR</x:v>
+      </x:c>
+      <x:c r="B46" s="7" t="str">
+        <x:v>U13</x:v>
+      </x:c>
+      <x:c r="C46" s="7" t="str">
+        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
+      </x:c>
+      <x:c r="D46" s="7" t="str">
+        <x:v>C201698</x:v>
+      </x:c>
+      <x:c r="E46" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F46" s="10"/>
+      <x:c r="G46" s="9" t="str">
         <x:f>IF(ISNUMBER(F46),E46*F46,"")</x:f>
-        <x:v>14.32</x:v>
-      </x:c>
-      <x:c r="H46" s="11" t="str">
-        <x:v>https://www.adafruit.com/product/4699</x:v>
-      </x:c>
-      <x:c r="I46" s="11"/>
-      <x:c r="J46" s="11" t="str">
-        <x:v>ZR370-02PM</x:v>
-      </x:c>
-      <x:c r="K46" s="11" t="str">
-        <x:v>Supplier-specified</x:v>
-      </x:c>
-      <x:c r="L46" s="11" t="str">
-        <x:v>Manual pump fitting</x:v>
-      </x:c>
-      <x:c r="M46" s="11" t="str">
-        <x:v>Existing pump retained for intermittent use. Manual fitting; provide mechanical support.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="53" customHeight="1">
-      <x:c r="A47" s="11" t="str">
-        <x:v>JST XH 2-pin 2.50mm</x:v>
-      </x:c>
-      <x:c r="B47" s="11" t="str">
-        <x:v>U9,U10</x:v>
-      </x:c>
-      <x:c r="C47" s="11" t="str">
-        <x:v>RheoBoard:VALVE_v105</x:v>
-      </x:c>
-      <x:c r="D47" s="11" t="str">
-        <x:v>C158012</x:v>
-      </x:c>
-      <x:c r="E47" s="12" t="n">
-        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H46" s="7" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C201698.html</x:v>
+      </x:c>
+      <x:c r="I46" s="7" t="str">
+        <x:v>https://www.ti.com/lit/ds/symlink/tca9517a.pdf</x:v>
+      </x:c>
+      <x:c r="J46" s="7" t="str">
+        <x:v>TCA9517ADGKR</x:v>
+      </x:c>
+      <x:c r="K46" s="7" t="str">
+        <x:v>Texas Instruments</x:v>
+      </x:c>
+      <x:c r="L46" s="7" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M46" s="7" t="str">
+        <x:v>Qwiic master interface: local bus on A, host on B. EN and VCCB use HOST_3V3; separate supplies, common GND. TI DGK land pattern: 1.4 x 0.45 mm pads, 0.65 mm pitch, 4.4 mm row-center span.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="83" customHeight="1">
+      <x:c r="A47" s="7" t="str">
+        <x:v>BZT52C10-7-F</x:v>
+      </x:c>
+      <x:c r="B47" s="7" t="str">
+        <x:v>D37</x:v>
+      </x:c>
+      <x:c r="C47" s="7" t="str">
+        <x:v>Diode_SMD:D_SOD-123</x:v>
+      </x:c>
+      <x:c r="D47" s="7" t="str">
+        <x:v>C155227</x:v>
+      </x:c>
+      <x:c r="E47" s="8" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F47" s="10"/>
-      <x:c r="G47" s="13" t="str">
+      <x:c r="G47" s="9" t="str">
         <x:f>IF(ISNUMBER(F47),E47*F47,"")</x:f>
       </x:c>
-      <x:c r="H47" s="11" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C158012.html</x:v>
-      </x:c>
-      <x:c r="I47" s="11" t="str">
-        <x:v>https://www.jst-mfg.com/product/pdf/eng/eXH.pdf</x:v>
-      </x:c>
-      <x:c r="J47" s="11" t="str">
-        <x:v>B2B-XH-A(LF)(SN)</x:v>
-      </x:c>
-      <x:c r="K47" s="11" t="str">
-        <x:v>JST</x:v>
-      </x:c>
-      <x:c r="L47" s="11" t="str">
-        <x:v>Manual THT</x:v>
-      </x:c>
-      <x:c r="M47" s="11" t="str">
-        <x:v>Fitted JST XH header only. External valve is listed on Manual accessories. Manual through-hole assembly.</x:v>
+      <x:c r="H47" s="7" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C155227.html</x:v>
+      </x:c>
+      <x:c r="I47" s="7" t="str">
+        <x:v>https://www.diodes.com/datasheet/download/BZT52Cxx.pdf</x:v>
+      </x:c>
+      <x:c r="J47" s="7" t="str">
+        <x:v>BZT52C10-7-F</x:v>
+      </x:c>
+      <x:c r="K47" s="7" t="str">
+        <x:v>Diodes Incorporated</x:v>
+      </x:c>
+      <x:c r="L47" s="7" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M47" s="7" t="str">
+        <x:v>Q11 gate-source clamp. Cathode to VIN_RAW/source; anode to gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="53" customHeight="1">
-      <x:c r="A48" s="7" t="str">
-        <x:v>TPS259472ARPWR</x:v>
-      </x:c>
-      <x:c r="B48" s="7" t="str">
-        <x:v>U12</x:v>
-      </x:c>
-      <x:c r="C48" s="7" t="str">
-        <x:v>RheoBoard:TI_RPW0010A_VQFN-HR_2x2mm</x:v>
-      </x:c>
-      <x:c r="D48" s="7" t="str">
-        <x:v>C3662789</x:v>
-      </x:c>
-      <x:c r="E48" s="8" t="n">
+      <x:c r="A48" s="11" t="str">
+        <x:v>Button GPIO 1x05 2.54mm</x:v>
+      </x:c>
+      <x:c r="B48" s="11" t="str">
+        <x:v>J19</x:v>
+      </x:c>
+      <x:c r="C48" s="11" t="str">
+        <x:v>Connector_PinHeader_2.54mm:PinHeader_1x05_P2.54mm_Vertical</x:v>
+      </x:c>
+      <x:c r="D48" s="11"/>
+      <x:c r="E48" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F48" s="10"/>
-      <x:c r="G48" s="9" t="str">
+      <x:c r="F48" s="20"/>
+      <x:c r="G48" s="13" t="str">
         <x:f>IF(ISNUMBER(F48),E48*F48,"")</x:f>
       </x:c>
-      <x:c r="H48" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C3662789.html</x:v>
-      </x:c>
-      <x:c r="I48" s="7" t="str">
-        <x:v>https://www.ti.com/lit/ds/symlink/tps25947.pdf</x:v>
-      </x:c>
-      <x:c r="J48" s="7" t="str">
-        <x:v>TPS259472ARPWR</x:v>
-      </x:c>
-      <x:c r="K48" s="7" t="str">
-        <x:v>Texas Instruments</x:v>
-      </x:c>
-      <x:c r="L48" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M48" s="7" t="str">
-        <x:v>New auto-retry input eFuse; TI RPW0010A HotRod footprint, approximately 2 A limit / 13.8 V clamp.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="112" customHeight="1">
-      <x:c r="A49" s="7" t="str">
-        <x:v>TCA9517ADGKR</x:v>
-      </x:c>
-      <x:c r="B49" s="7" t="str">
-        <x:v>U13</x:v>
-      </x:c>
-      <x:c r="C49" s="7" t="str">
-        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
-      </x:c>
-      <x:c r="D49" s="7" t="str">
-        <x:v>C201698</x:v>
-      </x:c>
-      <x:c r="E49" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F49" s="10"/>
-      <x:c r="G49" s="9" t="str">
-        <x:f>IF(ISNUMBER(F49),E49*F49,"")</x:f>
-      </x:c>
-      <x:c r="H49" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C201698.html</x:v>
-      </x:c>
-      <x:c r="I49" s="7" t="str">
-        <x:v>https://www.ti.com/lit/ds/symlink/tca9517a.pdf</x:v>
-      </x:c>
-      <x:c r="J49" s="7" t="str">
-        <x:v>TCA9517ADGKR</x:v>
-      </x:c>
-      <x:c r="K49" s="7" t="str">
-        <x:v>Texas Instruments</x:v>
-      </x:c>
-      <x:c r="L49" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M49" s="7" t="str">
-        <x:v>Qwiic master interface: local bus on A, host on B. EN and VCCB use HOST_3V3; separate supplies, common GND. TI DGK land pattern: 1.4 x 0.45 mm pads, 0.65 mm pitch, 4.4 mm row-center span.</x:v>
-      </x:c>
+      <x:c r="H48" s="11" t="str">
+        <x:v>https://www.adafruit.com/product/392</x:v>
+      </x:c>
+      <x:c r="I48" s="11"/>
+      <x:c r="J48" s="11" t="str">
+        <x:v>392, cut to 5 positions</x:v>
+      </x:c>
+      <x:c r="K48" s="11" t="str">
+        <x:v>Adafruit or equivalent</x:v>
+      </x:c>
+      <x:c r="L48" s="11" t="str">
+        <x:v>Manual</x:v>
+      </x:c>
+      <x:c r="M48" s="11" t="str">
+        <x:v>Straight 2.54mm male header. Pin1 GND,2 SW1,3 SW2,4 SW3,5 SW4. Buttons need separate GPIO cable and host power through J9.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="30" customHeight="1">
+      <x:c r="A49" s="14" t="str">
+        <x:v>Total fitted parts / incomplete priced subtotal</x:v>
+      </x:c>
+      <x:c r="B49" s="14"/>
+      <x:c r="C49" s="14"/>
+      <x:c r="D49" s="14"/>
+      <x:c r="E49" s="14" t="n">
+        <x:f>SUM(E2:E48)</x:f>
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="F49" s="14" t="str">
+        <x:v>Incomplete estimate</x:v>
+      </x:c>
+      <x:c r="G49" s="15" t="n">
+        <x:f>SUM(G2:G48)</x:f>
+        <x:v>52.888</x:v>
+      </x:c>
+      <x:c r="H49"/>
+      <x:c r="I49"/>
+      <x:c r="J49"/>
+      <x:c r="K49"/>
+      <x:c r="L49"/>
+      <x:c r="M49"/>
     </x:row>
     <x:row r="50" ht="83" customHeight="1">
-      <x:c r="A50" s="7" t="str">
-        <x:v>BZT52C10-7-F</x:v>
-      </x:c>
-      <x:c r="B50" s="7" t="str">
-        <x:v>D37</x:v>
-      </x:c>
-      <x:c r="C50" s="7" t="str">
-        <x:v>Diode_SMD:D_SOD-123</x:v>
-      </x:c>
-      <x:c r="D50" s="7" t="str">
-        <x:v>C155227</x:v>
-      </x:c>
-      <x:c r="E50" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F50" s="10"/>
-      <x:c r="G50" s="9" t="str">
-        <x:f>IF(ISNUMBER(F50),E50*F50,"")</x:f>
-      </x:c>
-      <x:c r="H50" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C155227.html</x:v>
-      </x:c>
-      <x:c r="I50" s="7" t="str">
-        <x:v>https://www.diodes.com/datasheet/download/BZT52Cxx.pdf</x:v>
-      </x:c>
-      <x:c r="J50" s="7" t="str">
-        <x:v>BZT52C10-7-F</x:v>
-      </x:c>
-      <x:c r="K50" s="7" t="str">
-        <x:v>Diodes Incorporated</x:v>
-      </x:c>
-      <x:c r="L50" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M50" s="7" t="str">
-        <x:v>Q11 gate-source clamp. Cathode to VIN_RAW/source; anode to gate.</x:v>
-      </x:c>
+      <x:c r="A50"/>
+      <x:c r="B50"/>
+      <x:c r="C50"/>
+      <x:c r="D50"/>
+      <x:c r="E50"/>
+      <x:c r="F50"/>
+      <x:c r="G50"/>
+      <x:c r="H50"/>
+      <x:c r="I50"/>
+      <x:c r="J50"/>
+      <x:c r="K50"/>
+      <x:c r="L50"/>
+      <x:c r="M50"/>
     </x:row>
     <x:row r="51" ht="30" customHeight="1">
-      <x:c r="A51" s="14" t="str">
-        <x:v>Total fitted parts / incomplete priced subtotal</x:v>
-      </x:c>
-      <x:c r="B51" s="14"/>
-      <x:c r="C51" s="14"/>
-      <x:c r="D51" s="14"/>
-      <x:c r="E51" s="14" t="n">
-        <x:f>SUM(E2:E50)</x:f>
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="F51" s="14" t="str">
-        <x:v>Incomplete estimate</x:v>
-      </x:c>
-      <x:c r="G51" s="15" t="n">
-        <x:f>SUM(G2:G50)</x:f>
-        <x:v>55.194</x:v>
-      </x:c>
+      <x:c r="A51"/>
+      <x:c r="B51"/>
+      <x:c r="C51"/>
+      <x:c r="D51"/>
+      <x:c r="E51"/>
+      <x:c r="F51"/>
+      <x:c r="G51"/>
       <x:c r="H51"/>
       <x:c r="I51"/>
       <x:c r="J51"/>
@@ -2373,20 +2332,22 @@
       <x:c r="L51"/>
       <x:c r="M51"/>
     </x:row>
-    <x:row r="52">
-      <x:c r="A52"/>
-      <x:c r="B52"/>
-      <x:c r="C52"/>
-      <x:c r="D52"/>
-      <x:c r="E52"/>
-      <x:c r="F52"/>
-      <x:c r="G52"/>
-      <x:c r="H52"/>
-      <x:c r="I52"/>
-      <x:c r="J52"/>
-      <x:c r="K52"/>
-      <x:c r="L52"/>
-      <x:c r="M52"/>
+    <x:row r="52" ht="36" customHeight="1">
+      <x:c r="A52" s="16" t="str">
+        <x:v>Prices are retained from the original workbook only where the selected part is unchanged. New parts have blank prices. This subtotal is incomplete and is not a JLCPCB quotation; obtain a fresh quote for v1.05.</x:v>
+      </x:c>
+      <x:c r="B52" s="16"/>
+      <x:c r="C52" s="16"/>
+      <x:c r="D52" s="16"/>
+      <x:c r="E52" s="16"/>
+      <x:c r="F52" s="16"/>
+      <x:c r="G52" s="16"/>
+      <x:c r="H52" s="16"/>
+      <x:c r="I52" s="16"/>
+      <x:c r="J52" s="16"/>
+      <x:c r="K52" s="16"/>
+      <x:c r="L52" s="16"/>
+      <x:c r="M52" s="16"/>
     </x:row>
     <x:row r="53" ht="34" customHeight="1">
       <x:c r="A53"/>
@@ -2404,30 +2365,27 @@
       <x:c r="M53"/>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="16" t="str">
-        <x:v>Prices are retained from the original workbook only where the selected part is unchanged. New parts have blank prices. This subtotal is incomplete and is not a JLCPCB quotation; obtain a fresh quote for v1.05.</x:v>
-      </x:c>
-      <x:c r="B54" s="16"/>
-      <x:c r="C54" s="16"/>
-      <x:c r="D54" s="16"/>
-      <x:c r="E54" s="16"/>
-      <x:c r="F54" s="16"/>
-      <x:c r="G54" s="16"/>
-      <x:c r="H54" s="16"/>
-      <x:c r="I54" s="16"/>
-      <x:c r="J54" s="16"/>
-      <x:c r="K54" s="16"/>
-      <x:c r="L54" s="16"/>
-      <x:c r="M54" s="16"/>
+      <x:c r="A54"/>
+      <x:c r="B54"/>
+      <x:c r="C54"/>
+      <x:c r="D54"/>
+      <x:c r="E54"/>
+      <x:c r="F54"/>
+      <x:c r="G54"/>
+      <x:c r="H54"/>
+      <x:c r="I54"/>
+      <x:c r="J54"/>
+      <x:c r="K54"/>
+      <x:c r="L54"/>
+      <x:c r="M54"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A52:D52"/>
-    <x:mergeCell ref="A54:M54"/>
+    <x:mergeCell ref="A52:M52"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra94a2ddbbbb343d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1b68d8db98b494a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2557,7 +2515,7 @@
         <x:v>https://cdn.sparkfun.com/assets/6/d/c/6/c/ESP32_Thing_Plus_Schematic.pdf</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
-        <x:v>Connect standard four-wire Qwiic to J9 MASTER. Host 3.3 V powers only the host interface. Other Thing Plus variants require their own pin/power check. PCB-specific firmware initialization is required.</x:v>
+        <x:v>Connect four-wire Qwiic to J9 MASTER. Host3V3 powers U13 host interface and R16–R19 button pullups. J19 needs a separate four-GPIO + GND cable. PCB-specific firmware required.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="154" customHeight="1">
@@ -2584,13 +2542,27 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="154" customHeight="1">
-      <x:c r="A7"/>
-      <x:c r="B7"/>
-      <x:c r="C7"/>
-      <x:c r="D7"/>
-      <x:c r="E7"/>
-      <x:c r="F7"/>
-      <x:c r="G7"/>
+      <x:c r="A7" s="3" t="str">
+        <x:v>Button GPIO cable</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="str">
+        <x:v>5 leads per board using its buttons</x:v>
+      </x:c>
+      <x:c r="C7" s="3" t="str">
+        <x:v>Adafruit or equivalent</x:v>
+      </x:c>
+      <x:c r="D7" s="3" t="str">
+        <x:v>1950: use 5 of 20 female/female 150mm jumpers</x:v>
+      </x:c>
+      <x:c r="E7" s="3" t="str">
+        <x:v>J19 buttons to ESP32 GPIO32,33,25,26 and GND</x:v>
+      </x:c>
+      <x:c r="F7" s="3" t="str">
+        <x:v>https://www.adafruit.com/product/1950</x:v>
+      </x:c>
+      <x:c r="G7" s="3" t="str">
+        <x:v>J19 pin1 GND;2 GPIO32;3 GPIO33;4 GPIO25(A1);5 GPIO26(A0). Requires male headers on ESP32. Both this cable and Qwiic/J9 are needed; no power wire on J19.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="154" customHeight="1">
       <x:c r="A8"/>
@@ -2604,7 +2576,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7db9df7c5530470e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5c51e6e2deb4589"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2638,7 +2610,7 @@
         <x:v>10uF 25V X5R ±10%</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>C1,C2,C8,C9,C15,C16</x:v>
+        <x:v>C1, C2, C8, C9, C15, C16</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
         <x:v>Capacitor_SMD:C_0805_2012Metric_Pad1.18x1.45mm_HandSolder</x:v>
@@ -2652,7 +2624,7 @@
         <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B3" s="3" t="str">
-        <x:v>C3, C4, C5, C23, C24, C25, C26, C30, C31, C33, C42, C44, C46, C47, C56, C59, C63, C68, C69</x:v>
+        <x:v>C3, C4, C5, C23, C24, C25, C26, C30, C31, C33, C42, C44, C46, C56, C59, C63, C68, C69</x:v>
       </x:c>
       <x:c r="C3" s="3" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
@@ -2663,610 +2635,586 @@
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="3" t="str">
-        <x:v>10nF 50V ±10%</x:v>
+        <x:v>1nF 50V X7R ±5%</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
-        <x:v>C22</x:v>
+        <x:v>C27</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D4" s="3" t="str">
-        <x:v>C57112</x:v>
+        <x:v>C5360811</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="3" t="str">
-        <x:v>1nF 50V X7R ±5%</x:v>
+        <x:v>10uF 25V X5R ±10%</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>C27</x:v>
+        <x:v>C28, C29</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D5" s="3" t="str">
-        <x:v>C5360811</x:v>
+        <x:v>C7393892</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="3" t="str">
-        <x:v>10uF 25V X5R ±10%</x:v>
+        <x:v>22uF 50V ±20%</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>C28,C29</x:v>
+        <x:v>C32, C34, C43, C45</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
+        <x:v>Capacitor_SMD:CP_Elec_6.3x5.8</x:v>
       </x:c>
       <x:c r="D6" s="3" t="str">
-        <x:v>C7393892</x:v>
+        <x:v>C128458</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="3" t="str">
-        <x:v>22uF 50V ±20%</x:v>
+        <x:v>22uF 25V X5R ±20%</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
-        <x:v>C32,C34,C43,C45</x:v>
+        <x:v>C52, C53, C54, C57, C60, C61</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
-        <x:v>Capacitor_SMD:CP_Elec_6.3x5.8</x:v>
+        <x:v>Capacitor_SMD:C_0805_2012Metric_Pad1.18x1.45mm_HandSolder</x:v>
       </x:c>
       <x:c r="D7" s="3" t="str">
-        <x:v>C128458</x:v>
+        <x:v>C20416420</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="3" t="str">
-        <x:v>22uF 25V X5R ±20%</x:v>
+        <x:v>18pF 50V C0G ±2%</x:v>
       </x:c>
       <x:c r="B8" s="3" t="str">
-        <x:v>C52,C53,C54,C57,C60,C61</x:v>
+        <x:v>C55, C58, C62</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
-        <x:v>Capacitor_SMD:C_0805_2012Metric_Pad1.18x1.45mm_HandSolder</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D8" s="3" t="str">
-        <x:v>C20416420</x:v>
+        <x:v>C2169079</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="3" t="str">
-        <x:v>18pF 50V C0G ±2%</x:v>
+        <x:v>3.3nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
-        <x:v>C55,C58,C62</x:v>
+        <x:v>C64</x:v>
       </x:c>
       <x:c r="C9" s="3" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D9" s="3" t="str">
-        <x:v>C2169079</x:v>
+        <x:v>C107088</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="3" t="str">
-        <x:v>3.3nF 50V X7R ±10%</x:v>
+        <x:v>1uF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>C64</x:v>
+        <x:v>C65</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:C_0805_2012Metric</x:v>
       </x:c>
       <x:c r="D10" s="3" t="str">
-        <x:v>C107088</x:v>
+        <x:v>C91185</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="3" t="str">
-        <x:v>1uF 50V X7R ±10%</x:v>
+        <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
-        <x:v>C65</x:v>
+        <x:v>C66</x:v>
       </x:c>
       <x:c r="C11" s="3" t="str">
-        <x:v>Capacitor_SMD:C_0805_2012Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D11" s="3" t="str">
-        <x:v>C91185</x:v>
+        <x:v>C14663</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="3" t="str">
-        <x:v>100nF 50V X7R ±10%</x:v>
+        <x:v>4.7uF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
-        <x:v>C66</x:v>
+        <x:v>C67</x:v>
       </x:c>
       <x:c r="C12" s="3" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:C_1206_3216Metric</x:v>
       </x:c>
       <x:c r="D12" s="3" t="str">
-        <x:v>C14663</x:v>
+        <x:v>C132170</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="3" t="str">
-        <x:v>4.7uF 50V X7R ±10%</x:v>
+        <x:v>DMP6023LE-13</x:v>
       </x:c>
       <x:c r="B13" s="3" t="str">
-        <x:v>C67</x:v>
+        <x:v>Q11</x:v>
       </x:c>
       <x:c r="C13" s="3" t="str">
-        <x:v>Capacitor_SMD:C_1206_3216Metric</x:v>
+        <x:v>Package_TO_SOT_SMD:SOT-223-3_TabPin2</x:v>
       </x:c>
       <x:c r="D13" s="3" t="str">
-        <x:v>C132170</x:v>
+        <x:v>C154901</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="3" t="str">
-        <x:v>DMP6023LE-13</x:v>
+        <x:v>LED_Red</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
-        <x:v>Q11</x:v>
+        <x:v>D6, D7, D8, D13, D14, D15, D17, D19</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
-        <x:v>Package_TO_SOT_SMD:SOT-223-3_TabPin2</x:v>
+        <x:v>LED_SMD:LED_0603_1608Metric_Pad1.05x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D14" s="3" t="str">
-        <x:v>C154901</x:v>
+        <x:v>C434419</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="3" t="str">
-        <x:v>LED_Red</x:v>
+        <x:v>SS34</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
-        <x:v>D6,D7,D8,D13,D14,D15,D17,D19</x:v>
+        <x:v>D11, D12, D16, D18</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
-        <x:v>LED_SMD:LED_0603_1608Metric_Pad1.05x0.95mm_HandSolder</x:v>
+        <x:v>Diode_SMD:D_SMA</x:v>
       </x:c>
       <x:c r="D15" s="3" t="str">
-        <x:v>C434419</x:v>
+        <x:v>C115205</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="3" t="str">
-        <x:v>SS34</x:v>
+        <x:v>LED_Red</x:v>
       </x:c>
       <x:c r="B16" s="3" t="str">
-        <x:v>D11,D12,D16,D18</x:v>
+        <x:v>D33, D34, D35</x:v>
       </x:c>
       <x:c r="C16" s="3" t="str">
-        <x:v>Diode_SMD:D_SMA</x:v>
+        <x:v>LED_SMD:LED_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D16" s="3" t="str">
-        <x:v>C115205</x:v>
+        <x:v>C434419</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="3" t="str">
-        <x:v>LED_Red</x:v>
+        <x:v>SMBJ13A</x:v>
       </x:c>
       <x:c r="B17" s="3" t="str">
-        <x:v>D33,D34,D35</x:v>
+        <x:v>D36</x:v>
       </x:c>
       <x:c r="C17" s="3" t="str">
-        <x:v>LED_SMD:LED_0603_1608Metric</x:v>
+        <x:v>Diode_SMD:D_SMB</x:v>
       </x:c>
       <x:c r="D17" s="3" t="str">
-        <x:v>C434419</x:v>
+        <x:v>C151252</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="3" t="str">
-        <x:v>SMBJ13A</x:v>
+        <x:v>2A time-delay JFC1032-1200TS</x:v>
       </x:c>
       <x:c r="B18" s="3" t="str">
-        <x:v>D36</x:v>
+        <x:v>F1</x:v>
       </x:c>
       <x:c r="C18" s="3" t="str">
-        <x:v>Diode_SMD:D_SMB</x:v>
+        <x:v>RheoBoard:Fuse_JDT_JFC1032TS_10.25x3.2mm</x:v>
       </x:c>
       <x:c r="D18" s="3" t="str">
-        <x:v>C151252</x:v>
+        <x:v>C53035082</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" s="3" t="str">
-        <x:v>2A time-delay JFC1032-1200TS</x:v>
+        <x:v>JST SH 4-pin 1.00mm</x:v>
       </x:c>
       <x:c r="B19" s="3" t="str">
-        <x:v>F1</x:v>
+        <x:v>J1, J9, J12, J17</x:v>
       </x:c>
       <x:c r="C19" s="3" t="str">
-        <x:v>RheoBoard:Fuse_JDT_JFC1032TS_10.25x3.2mm</x:v>
+        <x:v>Connector_JST:JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</x:v>
       </x:c>
       <x:c r="D19" s="3" t="str">
-        <x:v>C53035082</x:v>
+        <x:v>C160404</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
       <x:c r="A20" s="3" t="str">
-        <x:v>JST SH 4-pin 1.00mm</x:v>
+        <x:v>4.7uH FXL0530-4R7-M</x:v>
       </x:c>
       <x:c r="B20" s="3" t="str">
-        <x:v>J1,J9,J12,J17</x:v>
+        <x:v>L1, L2, L5</x:v>
       </x:c>
       <x:c r="C20" s="3" t="str">
-        <x:v>Connector_JST:JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</x:v>
+        <x:v>Inductor_SMD:L_Changjiang_FXL0530</x:v>
       </x:c>
       <x:c r="D20" s="3" t="str">
-        <x:v>C160404</x:v>
+        <x:v>C177246</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
       <x:c r="A21" s="3" t="str">
-        <x:v>4.7uH FXL0530-4R7-M</x:v>
+        <x:v>AO3400A</x:v>
       </x:c>
       <x:c r="B21" s="3" t="str">
-        <x:v>L1,L2,L5</x:v>
+        <x:v>Q3, Q4, Q8, Q10</x:v>
       </x:c>
       <x:c r="C21" s="3" t="str">
-        <x:v>Inductor_SMD:L_Changjiang_FXL0530</x:v>
+        <x:v>RheoBoard:AO3400A</x:v>
       </x:c>
       <x:c r="D21" s="3" t="str">
-        <x:v>C177246</x:v>
+        <x:v>C20917</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" s="3" t="str">
-        <x:v>AO3400A</x:v>
+        <x:v>100K/0603/1%</x:v>
       </x:c>
       <x:c r="B22" s="3" t="str">
-        <x:v>Q3,Q4,Q8,Q10</x:v>
+        <x:v>R1, R4, R7</x:v>
       </x:c>
       <x:c r="C22" s="3" t="str">
-        <x:v>RheoBoard:AO3400A</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D22" s="3" t="str">
-        <x:v>C20917</x:v>
+        <x:v>C25803</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
       <x:c r="A23" s="3" t="str">
-        <x:v>100K/0603/1%</x:v>
+        <x:v>4K7/0603/1%</x:v>
       </x:c>
       <x:c r="B23" s="3" t="str">
-        <x:v>R1,R4,R7</x:v>
+        <x:v>R15, R20, R82, R83</x:v>
       </x:c>
       <x:c r="C23" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D23" s="3" t="str">
-        <x:v>C25803</x:v>
+        <x:v>C23162</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
       <x:c r="A24" s="3" t="str">
-        <x:v>2K2/0603/1%</x:v>
+        <x:v>10K/0603/1%</x:v>
       </x:c>
       <x:c r="B24" s="3" t="str">
-        <x:v>R10</x:v>
+        <x:v>R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84, R85</x:v>
       </x:c>
       <x:c r="C24" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D24" s="3" t="str">
-        <x:v>C4190</x:v>
+        <x:v>C25804</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
       <x:c r="A25" s="3" t="str">
-        <x:v>4K7/0603/1%</x:v>
+        <x:v>1k/0603/1%</x:v>
       </x:c>
       <x:c r="B25" s="3" t="str">
-        <x:v>R11, R15, R20, R82, R83</x:v>
+        <x:v>R24, R25, R26, R39, R40, R54, R59, R75</x:v>
       </x:c>
       <x:c r="C25" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D25" s="3" t="str">
-        <x:v>C23162</x:v>
+        <x:v>C21190</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="48" customHeight="1">
       <x:c r="A26" s="3" t="str">
-        <x:v>10K/0603/1%</x:v>
+        <x:v>100R/0603/1%</x:v>
       </x:c>
       <x:c r="B26" s="3" t="str">
-        <x:v>R13, R14, R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84, R85</x:v>
+        <x:v>R35, R36, R42, R55</x:v>
       </x:c>
       <x:c r="C26" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D26" s="3" t="str">
-        <x:v>C25804</x:v>
+        <x:v>C22775</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
       <x:c r="A27" s="3" t="str">
-        <x:v>1k/0603/1%</x:v>
+        <x:v>330/0603/1%</x:v>
       </x:c>
       <x:c r="B27" s="3" t="str">
-        <x:v>R24,R25,R26,R39,R40,R54,R59,R75</x:v>
+        <x:v>R44, R77</x:v>
       </x:c>
       <x:c r="C27" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D27" s="3" t="str">
-        <x:v>C21190</x:v>
+        <x:v>C23138</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="48" customHeight="1">
       <x:c r="A28" s="3" t="str">
-        <x:v>100R/0603/1%</x:v>
+        <x:v>196k ±1%</x:v>
       </x:c>
       <x:c r="B28" s="3" t="str">
-        <x:v>R35,R36,R42,R55</x:v>
+        <x:v>R45</x:v>
       </x:c>
       <x:c r="C28" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D28" s="3" t="str">
-        <x:v>C22775</x:v>
+        <x:v>C4203218</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="48" customHeight="1">
       <x:c r="A29" s="3" t="str">
-        <x:v>330/0603/1%</x:v>
+        <x:v>30K/0603/1%</x:v>
       </x:c>
       <x:c r="B29" s="3" t="str">
-        <x:v>R44,R77</x:v>
+        <x:v>R46, R74, R76</x:v>
       </x:c>
       <x:c r="C29" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D29" s="3" t="str">
-        <x:v>C23138</x:v>
+        <x:v>C22984</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="48" customHeight="1">
       <x:c r="A30" s="3" t="str">
-        <x:v>196k ±1%</x:v>
+        <x:v>270K/0603/1%</x:v>
       </x:c>
       <x:c r="B30" s="3" t="str">
-        <x:v>R45</x:v>
+        <x:v>R60</x:v>
       </x:c>
       <x:c r="C30" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D30" s="3" t="str">
-        <x:v>C4203218</x:v>
+        <x:v>C22965</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="48" customHeight="1">
       <x:c r="A31" s="3" t="str">
-        <x:v>30K/0603/1%</x:v>
+        <x:v>135k ±0.1%</x:v>
       </x:c>
       <x:c r="B31" s="3" t="str">
-        <x:v>R46,R74,R76</x:v>
+        <x:v>R61</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D31" s="3" t="str">
-        <x:v>C22984</x:v>
+        <x:v>C861113</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="48" customHeight="1">
       <x:c r="A32" s="3" t="str">
-        <x:v>270K/0603/1%</x:v>
+        <x:v>549R ±1%</x:v>
       </x:c>
       <x:c r="B32" s="3" t="str">
-        <x:v>R60</x:v>
+        <x:v>R73</x:v>
       </x:c>
       <x:c r="C32" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D32" s="3" t="str">
-        <x:v>C22965</x:v>
+        <x:v>C23079</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="48" customHeight="1">
       <x:c r="A33" s="3" t="str">
-        <x:v>135k ±0.1%</x:v>
+        <x:v>680k ±1%</x:v>
       </x:c>
       <x:c r="B33" s="3" t="str">
-        <x:v>R61</x:v>
+        <x:v>R78</x:v>
       </x:c>
       <x:c r="C33" s="3" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D33" s="3" t="str">
-        <x:v>C861113</x:v>
+        <x:v>C25822</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="48" customHeight="1">
       <x:c r="A34" s="3" t="str">
-        <x:v>549R ±1%</x:v>
+        <x:v>100K/0603/1%</x:v>
       </x:c>
       <x:c r="B34" s="3" t="str">
-        <x:v>R73</x:v>
+        <x:v>R79</x:v>
       </x:c>
       <x:c r="C34" s="3" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D34" s="3" t="str">
-        <x:v>C23079</x:v>
+        <x:v>C25803</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="48" customHeight="1">
       <x:c r="A35" s="3" t="str">
-        <x:v>680k ±1%</x:v>
+        <x:v>390k ±1%</x:v>
       </x:c>
       <x:c r="B35" s="3" t="str">
-        <x:v>R78</x:v>
+        <x:v>R80</x:v>
       </x:c>
       <x:c r="C35" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D35" s="3" t="str">
-        <x:v>C25822</x:v>
+        <x:v>C2759410</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="48" customHeight="1">
       <x:c r="A36" s="3" t="str">
-        <x:v>100K/0603/1%</x:v>
+        <x:v>1.65k ±1%</x:v>
       </x:c>
       <x:c r="B36" s="3" t="str">
-        <x:v>R79</x:v>
+        <x:v>R81</x:v>
       </x:c>
       <x:c r="C36" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D36" s="3" t="str">
-        <x:v>C25803</x:v>
+        <x:v>C22845</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="48" customHeight="1">
       <x:c r="A37" s="3" t="str">
-        <x:v>390k ±1%</x:v>
+        <x:v>TL3301NF160QG/P010515</x:v>
       </x:c>
       <x:c r="B37" s="3" t="str">
-        <x:v>R80</x:v>
+        <x:v>SW1, SW2, SW3, SW4</x:v>
       </x:c>
       <x:c r="C37" s="3" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
+        <x:v>RheoBoard:Tactile_Switch_4pad</x:v>
       </x:c>
       <x:c r="D37" s="3" t="str">
-        <x:v>C2759410</x:v>
+        <x:v>C273527</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="48" customHeight="1">
       <x:c r="A38" s="3" t="str">
-        <x:v>1.65k ±1%</x:v>
+        <x:v>TPS563203DRLR</x:v>
       </x:c>
       <x:c r="B38" s="3" t="str">
-        <x:v>R81</x:v>
+        <x:v>U1, U2, U3</x:v>
       </x:c>
       <x:c r="C38" s="3" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
+        <x:v>RheoBoard:TPS563203DRLR</x:v>
       </x:c>
       <x:c r="D38" s="3" t="str">
-        <x:v>C22845</x:v>
+        <x:v>C22445512</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="48" customHeight="1">
       <x:c r="A39" s="3" t="str">
-        <x:v>TL3301NF160QG/P010515</x:v>
+        <x:v>MPRLS0025PA00001A</x:v>
       </x:c>
       <x:c r="B39" s="3" t="str">
-        <x:v>SW1,SW2,SW3,SW4</x:v>
+        <x:v>U5</x:v>
       </x:c>
       <x:c r="C39" s="3" t="str">
-        <x:v>RheoBoard:Tactile_Switch_4pad</x:v>
+        <x:v>RheoBoard:MPRLS0025PA00001A</x:v>
       </x:c>
       <x:c r="D39" s="3" t="str">
-        <x:v>C273527</x:v>
+        <x:v>C3257154</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="48" customHeight="1">
       <x:c r="A40" s="3" t="str">
-        <x:v>TPS563203DRLR</x:v>
+        <x:v>PCA9685PW,118</x:v>
       </x:c>
       <x:c r="B40" s="3" t="str">
-        <x:v>U1,U2,U3</x:v>
+        <x:v>U7</x:v>
       </x:c>
       <x:c r="C40" s="3" t="str">
-        <x:v>RheoBoard:TPS563203DRLR</x:v>
+        <x:v>RheoBoard:PCA9685</x:v>
       </x:c>
       <x:c r="D40" s="3" t="str">
-        <x:v>C22445512</x:v>
+        <x:v>C2678753</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" s="3" t="str">
-        <x:v>TCA9534APWR</x:v>
+        <x:v>TPS259472ARPWR</x:v>
       </x:c>
       <x:c r="B41" s="3" t="str">
-        <x:v>U4</x:v>
+        <x:v>U12</x:v>
       </x:c>
       <x:c r="C41" s="3" t="str">
-        <x:v>RheoBoard:TCA9534APWR</x:v>
+        <x:v>RheoBoard:TI_RPW0010A_VQFN-HR_2x2mm</x:v>
       </x:c>
       <x:c r="D41" s="3" t="str">
-        <x:v>C206010</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="48" customHeight="1">
+        <x:v>C3662789</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="70" customHeight="1">
       <x:c r="A42" s="3" t="str">
-        <x:v>MPRLS0025PA00001A</x:v>
+        <x:v>TCA9517ADGKR</x:v>
       </x:c>
       <x:c r="B42" s="3" t="str">
-        <x:v>U5</x:v>
+        <x:v>U13</x:v>
       </x:c>
       <x:c r="C42" s="3" t="str">
-        <x:v>RheoBoard:MPRLS0025PA00001A</x:v>
+        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
       </x:c>
       <x:c r="D42" s="3" t="str">
-        <x:v>C3257154</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="48" customHeight="1">
+        <x:v>C201698</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="70" customHeight="1">
       <x:c r="A43" s="3" t="str">
-        <x:v>PCA9685PW,118</x:v>
+        <x:v>BZT52C10-7-F</x:v>
       </x:c>
       <x:c r="B43" s="3" t="str">
-        <x:v>U7</x:v>
+        <x:v>D37</x:v>
       </x:c>
       <x:c r="C43" s="3" t="str">
-        <x:v>RheoBoard:PCA9685</x:v>
+        <x:v>Diode_SMD:D_SOD-123</x:v>
       </x:c>
       <x:c r="D43" s="3" t="str">
-        <x:v>C2678753</x:v>
+        <x:v>C155227</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
-      <x:c r="A44" s="3" t="str">
-        <x:v>TPS259472ARPWR</x:v>
-      </x:c>
-      <x:c r="B44" s="3" t="str">
-        <x:v>U12</x:v>
-      </x:c>
-      <x:c r="C44" s="3" t="str">
-        <x:v>RheoBoard:TI_RPW0010A_VQFN-HR_2x2mm</x:v>
-      </x:c>
-      <x:c r="D44" s="3" t="str">
-        <x:v>C3662789</x:v>
-      </x:c>
+      <x:c r="A44"/>
+      <x:c r="B44"/>
+      <x:c r="C44"/>
+      <x:c r="D44"/>
     </x:row>
     <x:row r="45" ht="70" customHeight="1">
-      <x:c r="A45" s="3" t="str">
-        <x:v>TCA9517ADGKR</x:v>
-      </x:c>
-      <x:c r="B45" s="3" t="str">
-        <x:v>U13</x:v>
-      </x:c>
-      <x:c r="C45" s="3" t="str">
-        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
-      </x:c>
-      <x:c r="D45" s="3" t="str">
-        <x:v>C201698</x:v>
-      </x:c>
+      <x:c r="A45"/>
+      <x:c r="B45"/>
+      <x:c r="C45"/>
+      <x:c r="D45"/>
     </x:row>
     <x:row r="46" ht="70" customHeight="1">
-      <x:c r="A46" s="3" t="str">
-        <x:v>BZT52C10-7-F</x:v>
-      </x:c>
-      <x:c r="B46" s="3" t="str">
-        <x:v>D37</x:v>
-      </x:c>
-      <x:c r="C46" s="3" t="str">
-        <x:v>Diode_SMD:D_SOD-123</x:v>
-      </x:c>
-      <x:c r="D46" s="3" t="str">
-        <x:v>C155227</x:v>
-      </x:c>
+      <x:c r="A46"/>
+      <x:c r="B46"/>
+      <x:c r="C46"/>
+      <x:c r="D46"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4025bb32a59f468d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6898bcc561c7446a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update RheoBoard v1.05 manufacturing files and documentation. Refreshed BOM, Gerber, and assembly drawings with updated creation timestamps. Enhanced component descriptions and assembly notes for clarity and accuracy. Adjusted designators and added new properties for improved organization and documentation consistency.
</commit_message>
<xml_diff>
--- a/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
+++ b/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc49d70a3a61b4d8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="R990a9440e7d0479d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="R2af93f5fe7ed4dbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2616e66ae2134703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="R159c1004ebdb49dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="R5c92f4b4ed4f4c40"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1076,7 +1076,7 @@
         <x:v>https://www.lcsc.com/product-detail/C151252.html</x:v>
       </x:c>
       <x:c r="I17" s="7" t="str">
-        <x:v>https://m.littelfuse.com/~/media/electronics/datasheets/tvs_diodes/littelfuse_tvs_diode_smbj_datasheet.pdf.pdf</x:v>
+        <x:v>https://www.littelfuse.com/assetdocs/tvs-diodes-smbj-series-datasheet?assetguid=ba555e99-a12d-4f72-a0b6-86b06c67171e</x:v>
       </x:c>
       <x:c r="J17" s="7" t="str">
         <x:v>SMBJ13A</x:v>
@@ -1088,7 +1088,7 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M17" s="7" t="str">
-        <x:v>Catalog attribute table incorrectly lists 14V/23.2V while selected manufacturer MPN is SMBJ13A. Require exact MPN SMBJ13A, 13V standoff, 21.5V clamp at 28A per manufacturer table; inspect supplier approval. Not a substitute for eFuse.</x:v>
+        <x:v>Exact Littelfuse SMBJ13A. 13 V standoff, 21.5 V clamp at 28 A. Marking LG; cathode band at pad 1 / VIN_RAW. Do not substitute SMBJ13CA or SMBJ14A.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="53" customHeight="1">
@@ -2283,18 +2283,20 @@
       <x:c r="H48" s="11" t="str">
         <x:v>https://www.adafruit.com/product/392</x:v>
       </x:c>
-      <x:c r="I48" s="11"/>
+      <x:c r="I48" s="11" t="str">
+        <x:v>https://www.adafruit.com/product/392</x:v>
+      </x:c>
       <x:c r="J48" s="11" t="str">
         <x:v>392, cut to 5 positions</x:v>
       </x:c>
       <x:c r="K48" s="11" t="str">
-        <x:v>Adafruit or equivalent</x:v>
+        <x:v>Adafruit Industries LLC</x:v>
       </x:c>
       <x:c r="L48" s="11" t="str">
         <x:v>Manual</x:v>
       </x:c>
       <x:c r="M48" s="11" t="str">
-        <x:v>Straight 2.54mm male header. Pin1 GND,2 SW1,3 SW2,4 SW3,5 SW4. Buttons need separate GPIO cable and host power through J9.</x:v>
+        <x:v>Cut one 5-position segment from a 36-pin strip. Pin 1 GND, 2 VALVE1_IN, 3 VALVE2_IN, 4 PUMP1_IN, 5 PUMP2_IN. Manual assembly; host power through J9.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="53" customHeight="1">
@@ -2430,7 +2432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R440eec40d6a74330"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f11a450511c4742"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2621,7 +2623,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a7d9bc7a0b947ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red1f681413f44669"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3271,7 +3273,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R318198dae4ab4027"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24517812b014401d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BOM and schematic properties for RheoBoard v1.05. Adjusted component values, LCSC part numbers, and descriptions for capacitors and resistors. Enhanced clarity and accuracy in documentation, including updated creation timestamps for manufacturing files.
</commit_message>
<xml_diff>
--- a/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
+++ b/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2616e66ae2134703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="R159c1004ebdb49dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="R5c92f4b4ed4f4c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb4aff1c3d8994bd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="R72a9e9467a424203"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="Reac696242ad74b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts cost" sheetId="4" r:id="R84eca56fb32b48f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,12 +16,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="$0.0000"/>
     <x:numFmt numFmtId="202" formatCode="$0.00"/>
+    <x:numFmt numFmtId="203" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -40,8 +42,34 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Times New Roman"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -78,6 +106,31 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF24476A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -91,7 +144,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="55">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -147,6 +200,78 @@
     <x:xf numFmtId="201" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -155,21 +280,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="13">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:Q51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="17">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
     <x:tableColumn id="3" name="Footprint"/>
     <x:tableColumn id="4" name="LCSC / JLCPCB part"/>
     <x:tableColumn id="5" name="Qty"/>
-    <x:tableColumn id="6" name="Legacy unit estimate (USD)"/>
-    <x:tableColumn id="7" name="Priced subtotal (USD)"/>
+    <x:tableColumn id="6" name="JLC unit USD (5 boards)"/>
+    <x:tableColumn id="7" name="SMT parts / board USD"/>
     <x:tableColumn id="8" name="Selected part source"/>
     <x:tableColumn id="9" name="Datasheet / specification"/>
     <x:tableColumn id="10" name="Manufacturer part number"/>
     <x:tableColumn id="11" name="Manufacturer"/>
     <x:tableColumn id="12" name="Assembly"/>
     <x:tableColumn id="13" name="Revision notes"/>
+    <x:tableColumn id="14" name="Maximum allowed tolerance"/>
+    <x:tableColumn id="15" name="Substitution requirements"/>
+    <x:tableColumn id="16" name="JLCPCB category"/>
+    <x:tableColumn id="17" name="Available order quantity"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -191,7 +320,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="RheoBoard105SMT" displayName="RheoBoard105SMT" ref="A1:D44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="RheoBoard105SMT" displayName="RheoBoard105SMT" ref="A1:D46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
@@ -410,9 +539,13 @@
     <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="55" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="110" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="36" customHeight="1">
+    <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="18" t="str">
         <x:v>Comment</x:v>
       </x:c>
@@ -429,10 +562,10 @@
         <x:v>Qty</x:v>
       </x:c>
       <x:c r="F1" s="18" t="str">
-        <x:v>Legacy unit estimate (USD)</x:v>
+        <x:v>Unit USD (5-board order)</x:v>
       </x:c>
       <x:c r="G1" s="18" t="str">
-        <x:v>Priced subtotal (USD)</x:v>
+        <x:v>Fitted parts / board USD</x:v>
       </x:c>
       <x:c r="H1" s="18" t="str">
         <x:v>Selected part source</x:v>
@@ -452,8 +585,20 @@
       <x:c r="M1" s="18" t="str">
         <x:v>Revision notes</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="53" customHeight="1">
+      <x:c r="N1" s="23" t="str">
+        <x:v>Maximum allowed tolerance</x:v>
+      </x:c>
+      <x:c r="O1" s="23" t="str">
+        <x:v>Substitution requirements</x:v>
+      </x:c>
+      <x:c r="P1" s="27" t="str">
+        <x:v>JLCPCB category</x:v>
+      </x:c>
+      <x:c r="Q1" s="27" t="str">
+        <x:v>Available order quantity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="72" customHeight="1">
       <x:c r="A2" s="7" t="str">
         <x:v>10uF 25V X5R ±10%</x:v>
       </x:c>
@@ -470,14 +615,14 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="F2" s="9" t="n">
-        <x:v>0.256</x:v>
+        <x:v>0.0379</x:v>
       </x:c>
       <x:c r="G2" s="9" t="n">
         <x:f>IF(ISNUMBER(F2),E2*F2,"")</x:f>
-        <x:v>1.536</x:v>
+        <x:v>0.22740000000000002</x:v>
       </x:c>
       <x:c r="H2" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C5448891.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C5448891</x:v>
       </x:c>
       <x:c r="I2" s="7"/>
       <x:c r="J2" s="7" t="str">
@@ -490,8 +635,20 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M2" s="7"/>
-    </x:row>
-    <x:row r="3" ht="126" customHeight="1">
+      <x:c r="N2" s="31" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="O2" s="32" t="str">
+        <x:v>Same capacitance, footprint, voltage and dielectric. Preserve effective capacitance under DC bias; electrolytics also require matching ESR/ripple/life.</x:v>
+      </x:c>
+      <x:c r="P2" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q2" s="32" t="n">
+        <x:v>149131</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="72" customHeight="1">
       <x:c r="A3" s="7" t="str">
         <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
@@ -508,14 +665,14 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="F3" s="9" t="n">
-        <x:v>0.073</x:v>
+        <x:v>0.0087</x:v>
       </x:c>
       <x:c r="G3" s="9" t="n">
         <x:f>IF(ISNUMBER(F3),E3*F3,"")</x:f>
-        <x:v>1.3139999999999998</x:v>
+        <x:v>0.1566</x:v>
       </x:c>
       <x:c r="H3" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C14663.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C14663</x:v>
       </x:c>
       <x:c r="I3" s="7"/>
       <x:c r="J3" s="7" t="str">
@@ -530,8 +687,20 @@
       <x:c r="M3" s="7" t="str">
         <x:v>C68/C69 added as local/host U13 supply bypass.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="53" customHeight="1">
+      <x:c r="N3" s="31" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="O3" s="32" t="str">
+        <x:v>Same capacitance, footprint, voltage and dielectric. Preserve effective capacitance under DC bias; electrolytics also require matching ESR/ripple/life.</x:v>
+      </x:c>
+      <x:c r="P3" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q3" s="32" t="n">
+        <x:v>30393077</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="72" customHeight="1">
       <x:c r="A4" s="7" t="str">
         <x:v>1nF 50V X7R ±5%</x:v>
       </x:c>
@@ -548,14 +717,14 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>0.052</x:v>
+        <x:v>0.0051</x:v>
       </x:c>
       <x:c r="G4" s="9" t="n">
         <x:f>IF(ISNUMBER(F4),E4*F4,"")</x:f>
-        <x:v>0.052</x:v>
+        <x:v>0.0051</x:v>
       </x:c>
       <x:c r="H4" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C5360811.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C5360811</x:v>
       </x:c>
       <x:c r="I4" s="7"/>
       <x:c r="J4" s="7" t="str">
@@ -568,8 +737,20 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M4" s="7"/>
-    </x:row>
-    <x:row r="5" ht="53" customHeight="1">
+      <x:c r="N4" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O4" s="32" t="str">
+        <x:v>Same capacitance, footprint, voltage and dielectric. Preserve effective capacitance under DC bias; electrolytics also require matching ESR/ripple/life.</x:v>
+      </x:c>
+      <x:c r="P4" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q4" s="32" t="n">
+        <x:v>71799</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="72" customHeight="1">
       <x:c r="A5" s="7" t="str">
         <x:v>10uF 25V X5R ±10%</x:v>
       </x:c>
@@ -586,14 +767,14 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>0.165</x:v>
+        <x:v>0.0356</x:v>
       </x:c>
       <x:c r="G5" s="9" t="n">
         <x:f>IF(ISNUMBER(F5),E5*F5,"")</x:f>
-        <x:v>0.33</x:v>
+        <x:v>0.0712</x:v>
       </x:c>
       <x:c r="H5" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C7393892.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C7393892</x:v>
       </x:c>
       <x:c r="I5" s="7"/>
       <x:c r="J5" s="7" t="str">
@@ -606,8 +787,20 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M5" s="7"/>
-    </x:row>
-    <x:row r="6" ht="53" customHeight="1">
+      <x:c r="N5" s="31" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="O5" s="32" t="str">
+        <x:v>Same capacitance, footprint, voltage and dielectric. Preserve effective capacitance under DC bias; electrolytics also require matching ESR/ripple/life.</x:v>
+      </x:c>
+      <x:c r="P5" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q5" s="32" t="n">
+        <x:v>402730</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="72" customHeight="1">
       <x:c r="A6" s="7" t="str">
         <x:v>22uF 50V ±20%</x:v>
       </x:c>
@@ -623,12 +816,15 @@
       <x:c r="E6" s="8" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="F6" s="10"/>
-      <x:c r="G6" s="9" t="str">
+      <x:c r="F6" s="10" t="n">
+        <x:v>0.1789</x:v>
+      </x:c>
+      <x:c r="G6" s="9" t="n">
         <x:f>IF(ISNUMBER(F6),E6*F6,"")</x:f>
+        <x:v>0.7156</x:v>
       </x:c>
       <x:c r="H6" s="7" t="str">
-        <x:v>https://industrial.panasonic.com/ww/products/pt/aluminum-cap-smd/models/EEEFK1H220P</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C128458</x:v>
       </x:c>
       <x:c r="I6" s="7" t="str">
         <x:v>https://industrial.panasonic.com/cdbs/www-data/pdf/RDE0000/ABA0000C776.pdf</x:v>
@@ -645,8 +841,20 @@
       <x:c r="M6" s="7" t="str">
         <x:v>Reduced from 100uF to 22uF; each pump/valve rail is approximately 88.3uF nominal. Bench transient validation remains required.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="53" customHeight="1">
+      <x:c r="N6" s="31" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="O6" s="32" t="str">
+        <x:v>Same capacitance, footprint, voltage and dielectric. Preserve effective capacitance under DC bias; electrolytics also require matching ESR/ripple/life.</x:v>
+      </x:c>
+      <x:c r="P6" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q6" s="32" t="n">
+        <x:v>5494</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="72" customHeight="1">
       <x:c r="A7" s="7" t="str">
         <x:v>22uF 25V X5R ±20%</x:v>
       </x:c>
@@ -663,14 +871,14 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>0.216</x:v>
+        <x:v>0.1333</x:v>
       </x:c>
       <x:c r="G7" s="9" t="n">
         <x:f>IF(ISNUMBER(F7),E7*F7,"")</x:f>
-        <x:v>1.296</x:v>
+        <x:v>0.7998000000000001</x:v>
       </x:c>
       <x:c r="H7" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C20416420.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C20416420</x:v>
       </x:c>
       <x:c r="I7" s="7"/>
       <x:c r="J7" s="7" t="str">
@@ -683,71 +891,100 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M7" s="7"/>
-    </x:row>
-    <x:row r="8" ht="53" customHeight="1">
+      <x:c r="N7" s="31" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="O7" s="32" t="str">
+        <x:v>Same capacitance, footprint, voltage and dielectric. Preserve effective capacitance under DC bias; electrolytics also require matching ESR/ripple/life.</x:v>
+      </x:c>
+      <x:c r="P7" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q7" s="32" t="n">
+        <x:v>87761</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="72" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>18pF 50V C0G ±2%</x:v>
+        <x:v>18pF 50V C0G ±5%</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>C55, C58, C62</x:v>
+        <x:v>C55, C58</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D8" s="7" t="str">
-        <x:v>C2169079</x:v>
+        <x:v>C107040</x:v>
       </x:c>
       <x:c r="E8" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>0.043</x:v>
+        <x:v>0.0067</x:v>
       </x:c>
       <x:c r="G8" s="9" t="n">
         <x:f>IF(ISNUMBER(F8),E8*F8,"")</x:f>
-        <x:v>0.129</x:v>
+        <x:v>0.0134</x:v>
       </x:c>
       <x:c r="H8" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C2169079.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C107040</x:v>
       </x:c>
       <x:c r="I8" s="7"/>
       <x:c r="J8" s="7" t="str">
-        <x:v>VJ0603A180GXACW1BC</x:v>
+        <x:v>CC0603JRNPO9BN180</x:v>
       </x:c>
       <x:c r="K8" s="7" t="str">
-        <x:v>VISHAY</x:v>
+        <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="L8" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M8" s="7"/>
-    </x:row>
-    <x:row r="9" ht="53" customHeight="1">
+      <x:c r="M8" s="7" t="str">
+        <x:v>18 pF C0G 5%; same nominal value.</x:v>
+      </x:c>
+      <x:c r="N8" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O8" s="32" t="str">
+        <x:v>5% or better, 18 pF C0G/NP0, &gt;=50 V, 0603. Do not use X7R/X5R here.</x:v>
+      </x:c>
+      <x:c r="P8" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q8" s="32" t="n">
+        <x:v>697605</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="72" customHeight="1">
       <x:c r="A9" s="7" t="str">
-        <x:v>3.3nF 50V X7R ±10%</x:v>
+        <x:v>24pF 50V C0G ±5%</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>C64</x:v>
+        <x:v>C62</x:v>
       </x:c>
       <x:c r="C9" s="7" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D9" s="7" t="str">
-        <x:v>C107088</x:v>
+        <x:v>C107044</x:v>
       </x:c>
       <x:c r="E9" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F9" s="10"/>
-      <x:c r="G9" s="9" t="str">
+      <x:c r="F9" s="10" t="n">
+        <x:v>0.0109</x:v>
+      </x:c>
+      <x:c r="G9" s="9" t="n">
         <x:f>IF(ISNUMBER(F9),E9*F9,"")</x:f>
+        <x:v>0.0109</x:v>
       </x:c>
       <x:c r="H9" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C107088.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C107044</x:v>
       </x:c>
       <x:c r="I9" s="7"/>
       <x:c r="J9" s="7" t="str">
-        <x:v>CC0603KRX7R9BB332</x:v>
+        <x:v>CC0603JRNPO9BN240</x:v>
       </x:c>
       <x:c r="K9" s="7" t="str">
         <x:v>YAGEO</x:v>
@@ -756,37 +993,50 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M9" s="7" t="str">
-        <x:v>New controlled-startup timing capacitor for U12.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="53" customHeight="1">
+        <x:v>24 pF C0G 5%; scales feed-forward timing for R61 100k. Bench transient check required.</x:v>
+      </x:c>
+      <x:c r="N9" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O9" s="32" t="str">
+        <x:v>5% or better, 24 pF C0G/NP0, &gt;=50 V, 0603.</x:v>
+      </x:c>
+      <x:c r="P9" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q9" s="32" t="n">
+        <x:v>23936</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="72" customHeight="1">
       <x:c r="A10" s="7" t="str">
-        <x:v>1uF 50V X7R ±10%</x:v>
+        <x:v>3.3nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>C65</x:v>
+        <x:v>C64</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
-        <x:v>Capacitor_SMD:C_0805_2012Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D10" s="7" t="str">
-        <x:v>C91185</x:v>
+        <x:v>C107088</x:v>
       </x:c>
       <x:c r="E10" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F10" s="10"/>
-      <x:c r="G10" s="9" t="str">
+      <x:c r="F10" s="10" t="n">
+        <x:v>0.0055</x:v>
+      </x:c>
+      <x:c r="G10" s="9" t="n">
         <x:f>IF(ISNUMBER(F10),E10*F10,"")</x:f>
+        <x:v>0.0055</x:v>
       </x:c>
       <x:c r="H10" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C91185.html</x:v>
-      </x:c>
-      <x:c r="I10" s="7" t="str">
-        <x:v>https://www.yageogroup.com/download/specsheet/CC0805KKX7R9BB105</x:v>
-      </x:c>
+        <x:v>https://jlcpcb.com/partdetail/component/C107088</x:v>
+      </x:c>
+      <x:c r="I10" s="7"/>
       <x:c r="J10" s="7" t="str">
-        <x:v>CC0805KKX7R9BB105</x:v>
+        <x:v>CC0603KRX7R9BB332</x:v>
       </x:c>
       <x:c r="K10" s="7" t="str">
         <x:v>YAGEO</x:v>
@@ -795,38 +1045,52 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M10" s="7" t="str">
-        <x:v>New local input bypass for U12; place beside IN/GND.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="53" customHeight="1">
+        <x:v>New controlled-startup timing capacitor for U12.</x:v>
+      </x:c>
+      <x:c r="N10" s="31" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="O10" s="32" t="str">
+        <x:v>Same capacitance, footprint, voltage and dielectric. Preserve effective capacitance under DC bias; electrolytics also require matching ESR/ripple/life.</x:v>
+      </x:c>
+      <x:c r="P10" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q10" s="32" t="n">
+        <x:v>506819</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="72" customHeight="1">
       <x:c r="A11" s="7" t="str">
-        <x:v>100nF 50V X7R ±10%</x:v>
+        <x:v>1uF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>C66</x:v>
+        <x:v>C65</x:v>
       </x:c>
       <x:c r="C11" s="7" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:C_0805_2012Metric</x:v>
       </x:c>
       <x:c r="D11" s="7" t="str">
-        <x:v>C14663</x:v>
+        <x:v>C91185</x:v>
       </x:c>
       <x:c r="E11" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F11" s="9" t="n">
-        <x:v>0.073</x:v>
+        <x:v>0.0348</x:v>
       </x:c>
       <x:c r="G11" s="9" t="n">
         <x:f>IF(ISNUMBER(F11),E11*F11,"")</x:f>
-        <x:v>0.073</x:v>
+        <x:v>0.0348</x:v>
       </x:c>
       <x:c r="H11" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C14663.html</x:v>
-      </x:c>
-      <x:c r="I11" s="7"/>
+        <x:v>https://jlcpcb.com/partdetail/component/C91185</x:v>
+      </x:c>
+      <x:c r="I11" s="7" t="str">
+        <x:v>https://www.yageogroup.com/download/specsheet/CC0805KKX7R9BB105</x:v>
+      </x:c>
       <x:c r="J11" s="7" t="str">
-        <x:v>CC0603KRX7R9BB104</x:v>
+        <x:v>CC0805KKX7R9BB105</x:v>
       </x:c>
       <x:c r="K11" s="7" t="str">
         <x:v>YAGEO</x:v>
@@ -835,37 +1099,50 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M11" s="7" t="str">
-        <x:v>New local input high-frequency bypass for U12.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="53" customHeight="1">
+        <x:v>New local input bypass for U12; place beside IN/GND.</x:v>
+      </x:c>
+      <x:c r="N11" s="31" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="O11" s="32" t="str">
+        <x:v>Same capacitance, footprint, voltage and dielectric. Preserve effective capacitance under DC bias; electrolytics also require matching ESR/ripple/life.</x:v>
+      </x:c>
+      <x:c r="P11" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q11" s="32" t="n">
+        <x:v>317889</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="72" customHeight="1">
       <x:c r="A12" s="7" t="str">
-        <x:v>4.7uF 50V X7R ±10%</x:v>
+        <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>C67</x:v>
+        <x:v>C66</x:v>
       </x:c>
       <x:c r="C12" s="7" t="str">
-        <x:v>Capacitor_SMD:C_1206_3216Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D12" s="7" t="str">
-        <x:v>C132170</x:v>
+        <x:v>C14663</x:v>
       </x:c>
       <x:c r="E12" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F12" s="10"/>
-      <x:c r="G12" s="9" t="str">
+      <x:c r="F12" s="10" t="n">
+        <x:v>0.0087</x:v>
+      </x:c>
+      <x:c r="G12" s="9" t="n">
         <x:f>IF(ISNUMBER(F12),E12*F12,"")</x:f>
+        <x:v>0.0087</x:v>
       </x:c>
       <x:c r="H12" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C132170.html</x:v>
-      </x:c>
-      <x:c r="I12" s="7" t="str">
-        <x:v>https://www.yageogroup.com/download/specsheet/CC1206KKX7R9BB475</x:v>
-      </x:c>
+        <x:v>https://jlcpcb.com/partdetail/component/C14663</x:v>
+      </x:c>
+      <x:c r="I12" s="7"/>
       <x:c r="J12" s="7" t="str">
-        <x:v>CC1206KKX7R9BB475</x:v>
+        <x:v>CC0603KRX7R9BB104</x:v>
       </x:c>
       <x:c r="K12" s="7" t="str">
         <x:v>YAGEO</x:v>
@@ -874,538 +1151,646 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M12" s="7" t="str">
-        <x:v>New local output bypass for U12; place beside OUT/GND.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="53" customHeight="1">
+        <x:v>New local input high-frequency bypass for U12.</x:v>
+      </x:c>
+      <x:c r="N12" s="31" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="O12" s="32" t="str">
+        <x:v>Same capacitance, footprint, voltage and dielectric. Preserve effective capacitance under DC bias; electrolytics also require matching ESR/ripple/life.</x:v>
+      </x:c>
+      <x:c r="P12" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q12" s="32" t="n">
+        <x:v>30393077</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="72" customHeight="1">
       <x:c r="A13" s="7" t="str">
-        <x:v>DMP6023LE-13</x:v>
+        <x:v>4.7uF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B13" s="7" t="str">
-        <x:v>Q11</x:v>
+        <x:v>C67</x:v>
       </x:c>
       <x:c r="C13" s="7" t="str">
-        <x:v>RheoBoard:SOT-223-3_TabPin2_DFM</x:v>
+        <x:v>Capacitor_SMD:C_1206_3216Metric</x:v>
       </x:c>
       <x:c r="D13" s="7" t="str">
-        <x:v>C154901</x:v>
+        <x:v>C132170</x:v>
       </x:c>
       <x:c r="E13" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F13" s="10"/>
-      <x:c r="G13" s="9" t="str">
+      <x:c r="F13" s="10" t="n">
+        <x:v>0.1189</x:v>
+      </x:c>
+      <x:c r="G13" s="9" t="n">
         <x:f>IF(ISNUMBER(F13),E13*F13,"")</x:f>
+        <x:v>0.1189</x:v>
       </x:c>
       <x:c r="H13" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C154901.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C132170</x:v>
       </x:c>
       <x:c r="I13" s="7" t="str">
-        <x:v>https://www.diodes.com/datasheet/download/DMP6023LE.pdf</x:v>
+        <x:v>https://www.yageogroup.com/download/specsheet/CC1206KKX7R9BB475</x:v>
       </x:c>
       <x:c r="J13" s="7" t="str">
-        <x:v>DMP6023LE-13</x:v>
+        <x:v>CC1206KKX7R9BB475</x:v>
       </x:c>
       <x:c r="K13" s="7" t="str">
-        <x:v>Diodes Incorporated</x:v>
+        <x:v>YAGEO</x:v>
       </x:c>
       <x:c r="L13" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M13" s="7" t="str">
-        <x:v>Replaces D1 with lower-loss reverse-polarity protection. 1 gate, 2 drain/tab to fused input, 3 source to VIN_RAW.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="53" customHeight="1">
+        <x:v>New local output bypass for U12; place beside OUT/GND.</x:v>
+      </x:c>
+      <x:c r="N13" s="31" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="O13" s="32" t="str">
+        <x:v>Same capacitance, footprint, voltage and dielectric. Preserve effective capacitance under DC bias; electrolytics also require matching ESR/ripple/life.</x:v>
+      </x:c>
+      <x:c r="P13" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q13" s="32" t="n">
+        <x:v>16653</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="72" customHeight="1">
       <x:c r="A14" s="7" t="str">
-        <x:v>LED_Red</x:v>
+        <x:v>DMP6023LE-13</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>D6, D7, D8, D13, D14, D15, D17, D19</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RheoBoard:LED_SZYY0603R_A1_K2_HandSolder</x:t>
-        </x:is>
+        <x:v>Q11</x:v>
+      </x:c>
+      <x:c r="C14" s="7" t="str">
+        <x:v>RheoBoard:SOT-223-3_TabPin2_DFM</x:v>
       </x:c>
       <x:c r="D14" s="7" t="str">
-        <x:v>C434419</x:v>
+        <x:v>C154901</x:v>
       </x:c>
       <x:c r="E14" s="8" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F14" s="9" t="n">
-        <x:v>0.098</x:v>
+        <x:v>0.6237</x:v>
       </x:c>
       <x:c r="G14" s="9" t="n">
         <x:f>IF(ISNUMBER(F14),E14*F14,"")</x:f>
-        <x:v>0.784</x:v>
+        <x:v>0.6237</x:v>
       </x:c>
       <x:c r="H14" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C434419.html</x:v>
-      </x:c>
-      <x:c r="I14" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://datasheet.lcsc.com/datasheet/pdf/7948f9a4498910c84f6e992ff3fa9e63.pdf</x:t>
-        </x:is>
+        <x:v>https://jlcpcb.com/partdetail/component/C154901</x:v>
+      </x:c>
+      <x:c r="I14" s="7" t="str">
+        <x:v>https://www.diodes.com/datasheet/download/DMP6023LE.pdf</x:v>
       </x:c>
       <x:c r="J14" s="7" t="str">
-        <x:v>SZYY0603R</x:v>
+        <x:v>DMP6023LE-13</x:v>
       </x:c>
       <x:c r="K14" s="7" t="str">
-        <x:v>Yongyu Photoelectric</x:v>
+        <x:v>Diodes Incorporated</x:v>
       </x:c>
       <x:c r="L14" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M14" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manufacturer numbering: 1=A(+), 2=K(-). Cathode bar marks pad 2. See LED assembly guide.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="53" customHeight="1">
+      <x:c r="M14" s="7" t="str">
+        <x:v>Replaces D1 with lower-loss reverse-polarity protection. 1 gate, 2 drain/tab to fused input, 3 source to VIN_RAW.</x:v>
+      </x:c>
+      <x:c r="N14" s="31"/>
+      <x:c r="O14" s="32"/>
+      <x:c r="P14" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q14" s="32" t="n">
+        <x:v>476</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="72" customHeight="1">
       <x:c r="A15" s="7" t="str">
-        <x:v>SS34</x:v>
+        <x:v>LED_Red</x:v>
       </x:c>
       <x:c r="B15" s="7" t="str">
-        <x:v>D11, D12, D16, D18</x:v>
+        <x:v>D6, D7, D8, D13, D14, D15, D17, D19</x:v>
       </x:c>
       <x:c r="C15" s="7" t="str">
-        <x:v>Diode_SMD:D_SMA</x:v>
+        <x:v>RheoBoard:LED_SZYY0603R_A1_K2_HandSolder</x:v>
       </x:c>
       <x:c r="D15" s="7" t="str">
-        <x:v>C115205</x:v>
+        <x:v>C434419</x:v>
       </x:c>
       <x:c r="E15" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F15" s="9" t="n">
-        <x:v>0.467</x:v>
+        <x:v>0.0137</x:v>
       </x:c>
       <x:c r="G15" s="9" t="n">
         <x:f>IF(ISNUMBER(F15),E15*F15,"")</x:f>
-        <x:v>1.868</x:v>
+        <x:v>0.1096</x:v>
       </x:c>
       <x:c r="H15" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C115205.html</x:v>
-      </x:c>
-      <x:c r="I15" s="7"/>
+        <x:v>https://jlcpcb.com/partdetail/component/C434419</x:v>
+      </x:c>
+      <x:c r="I15" s="7" t="str">
+        <x:v>https://datasheet.lcsc.com/datasheet/pdf/7948f9a4498910c84f6e992ff3fa9e63.pdf</x:v>
+      </x:c>
       <x:c r="J15" s="7" t="str">
-        <x:v>SS34</x:v>
+        <x:v>SZYY0603R</x:v>
       </x:c>
       <x:c r="K15" s="7" t="str">
-        <x:v>Jingdao Microelectronics</x:v>
+        <x:v>Yongyu Photoelectric</x:v>
       </x:c>
       <x:c r="L15" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M15" s="7" t="str">
-        <x:v>SMA footprint and polarity mark match selected Jingdao SS34.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="53" customHeight="1">
+        <x:v>Manufacturer numbering: 1=A(+), 2=K(-). Cathode bar marks pad 2. See LED assembly guide.</x:v>
+      </x:c>
+      <x:c r="N15" s="31"/>
+      <x:c r="O15" s="32"/>
+      <x:c r="P15" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q15" s="32" t="n">
+        <x:v>830337</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="72" customHeight="1">
       <x:c r="A16" s="7" t="str">
-        <x:v>LED_Red</x:v>
+        <x:v>SS34</x:v>
       </x:c>
       <x:c r="B16" s="7" t="str">
-        <x:v>D33, D34, D35</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RheoBoard:LED_SZYY0603R_A1_K2_Nominal</x:t>
-        </x:is>
+        <x:v>D11, D12, D16, D18</x:v>
+      </x:c>
+      <x:c r="C16" s="7" t="str">
+        <x:v>Diode_SMD:D_SMA</x:v>
       </x:c>
       <x:c r="D16" s="7" t="str">
-        <x:v>C434419</x:v>
+        <x:v>C115205</x:v>
       </x:c>
       <x:c r="E16" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F16" s="9" t="n">
-        <x:v>0.098</x:v>
+        <x:v>0.0377</x:v>
       </x:c>
       <x:c r="G16" s="9" t="n">
         <x:f>IF(ISNUMBER(F16),E16*F16,"")</x:f>
-        <x:v>0.29400000000000004</x:v>
+        <x:v>0.1508</x:v>
       </x:c>
       <x:c r="H16" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C434419.html</x:v>
-      </x:c>
-      <x:c r="I16" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://datasheet.lcsc.com/datasheet/pdf/7948f9a4498910c84f6e992ff3fa9e63.pdf</x:t>
-        </x:is>
-      </x:c>
+        <x:v>https://jlcpcb.com/partdetail/component/C115205</x:v>
+      </x:c>
+      <x:c r="I16" s="7"/>
       <x:c r="J16" s="7" t="str">
-        <x:v>SZYY0603R</x:v>
+        <x:v>SS34</x:v>
       </x:c>
       <x:c r="K16" s="7" t="str">
-        <x:v>Yongyu Photoelectric</x:v>
+        <x:v>Jingdao Microelectronics</x:v>
       </x:c>
       <x:c r="L16" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M16" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manufacturer numbering: 1=A(+), 2=K(-). Cathode bar marks pad 2. See LED assembly guide.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="83" customHeight="1">
+      <x:c r="M16" s="7" t="str">
+        <x:v>SMA footprint and polarity mark match selected Jingdao SS34.</x:v>
+      </x:c>
+      <x:c r="N16" s="31"/>
+      <x:c r="O16" s="32"/>
+      <x:c r="P16" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q16" s="32" t="n">
+        <x:v>61565</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="72" customHeight="1">
       <x:c r="A17" s="7" t="str">
-        <x:v>SMBJ13A</x:v>
+        <x:v>LED_Red</x:v>
       </x:c>
       <x:c r="B17" s="7" t="str">
-        <x:v>D36</x:v>
+        <x:v>D33, D34, D35</x:v>
       </x:c>
       <x:c r="C17" s="7" t="str">
-        <x:v>Diode_SMD:D_SMB</x:v>
+        <x:v>RheoBoard:LED_SZYY0603R_A1_K2_Nominal</x:v>
       </x:c>
       <x:c r="D17" s="7" t="str">
-        <x:v>C151252</x:v>
+        <x:v>C434419</x:v>
       </x:c>
       <x:c r="E17" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F17" s="10"/>
-      <x:c r="G17" s="9" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F17" s="10" t="n">
+        <x:v>0.0137</x:v>
+      </x:c>
+      <x:c r="G17" s="9" t="n">
         <x:f>IF(ISNUMBER(F17),E17*F17,"")</x:f>
+        <x:v>0.0411</x:v>
       </x:c>
       <x:c r="H17" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C151252.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C434419</x:v>
       </x:c>
       <x:c r="I17" s="7" t="str">
-        <x:v>https://www.littelfuse.com/assetdocs/tvs-diodes-smbj-series-datasheet?assetguid=ba555e99-a12d-4f72-a0b6-86b06c67171e</x:v>
+        <x:v>https://datasheet.lcsc.com/datasheet/pdf/7948f9a4498910c84f6e992ff3fa9e63.pdf</x:v>
       </x:c>
       <x:c r="J17" s="7" t="str">
-        <x:v>SMBJ13A</x:v>
+        <x:v>SZYY0603R</x:v>
       </x:c>
       <x:c r="K17" s="7" t="str">
-        <x:v>Littelfuse</x:v>
+        <x:v>Yongyu Photoelectric</x:v>
       </x:c>
       <x:c r="L17" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M17" s="7" t="str">
-        <x:v>Exact Littelfuse SMBJ13A. 13 V standoff, 21.5 V clamp at 28 A. Marking LG; cathode band at pad 1 / VIN_RAW. Do not substitute SMBJ13CA or SMBJ14A.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="53" customHeight="1">
+        <x:v>Manufacturer numbering: 1=A(+), 2=K(-). Cathode bar marks pad 2. See LED assembly guide.</x:v>
+      </x:c>
+      <x:c r="N17" s="31"/>
+      <x:c r="O17" s="32"/>
+      <x:c r="P17" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q17" s="32" t="n">
+        <x:v>830337</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="72" customHeight="1">
       <x:c r="A18" s="7" t="str">
-        <x:v>2A time-delay JFC1032-1200TS</x:v>
+        <x:v>SMBJ13A</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>F1</x:v>
+        <x:v>D36</x:v>
       </x:c>
       <x:c r="C18" s="7" t="str">
-        <x:v>RheoBoard:Fuse_JDT_JFC1032TS_10.25x3.2mm</x:v>
+        <x:v>Diode_SMD:D_SMB</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
-        <x:v>C53035082</x:v>
+        <x:v>C151252</x:v>
       </x:c>
       <x:c r="E18" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F18" s="9" t="n">
-        <x:v>1.45</x:v>
+        <x:v>0.1425</x:v>
       </x:c>
       <x:c r="G18" s="9" t="n">
         <x:f>IF(ISNUMBER(F18),E18*F18,"")</x:f>
-        <x:v>1.45</x:v>
+        <x:v>0.1425</x:v>
       </x:c>
       <x:c r="H18" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C53035082.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C151252</x:v>
       </x:c>
       <x:c r="I18" s="7" t="str">
-        <x:v>https://www.jdtfuse.com/upload/PDF/JFC1032TS.pdf</x:v>
+        <x:v>https://www.littelfuse.com/assetdocs/tvs-diodes-smbj-series-datasheet?assetguid=ba555e99-a12d-4f72-a0b6-86b06c67171e</x:v>
       </x:c>
       <x:c r="J18" s="7" t="str">
-        <x:v>JFC1032-1200TS</x:v>
+        <x:v>SMBJ13A</x:v>
       </x:c>
       <x:c r="K18" s="7" t="str">
-        <x:v>JDTfuse</x:v>
+        <x:v>Littelfuse</x:v>
       </x:c>
       <x:c r="L18" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M18" s="7" t="str">
-        <x:v>Corrected centered origin and JDT land pattern. Check the new placement preview.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="53" customHeight="1">
+        <x:v>Exact Littelfuse SMBJ13A. 13 V standoff, 21.5 V clamp at 28 A. Marking LG; cathode band at pad 1 / VIN_RAW. Do not substitute SMBJ13CA or SMBJ14A.</x:v>
+      </x:c>
+      <x:c r="N18" s="31"/>
+      <x:c r="O18" s="32"/>
+      <x:c r="P18" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q18" s="32" t="n">
+        <x:v>1226</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="7" t="str">
-        <x:v>JST SH 4-pin 1.00mm</x:v>
+        <x:v>2A time-delay JFC1032-1200TS</x:v>
       </x:c>
       <x:c r="B19" s="7" t="str">
-        <x:v>J1, J9, J12, J17</x:v>
+        <x:v>F1</x:v>
       </x:c>
       <x:c r="C19" s="7" t="str">
-        <x:v>Connector_JST:JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</x:v>
+        <x:v>RheoBoard:Fuse_JDT_JFC1032TS_10.25x3.2mm</x:v>
       </x:c>
       <x:c r="D19" s="7" t="str">
-        <x:v>C160404</x:v>
+        <x:v>C53035082</x:v>
       </x:c>
       <x:c r="E19" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F19" s="9" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.2937</x:v>
       </x:c>
       <x:c r="G19" s="9" t="n">
         <x:f>IF(ISNUMBER(F19),E19*F19,"")</x:f>
-        <x:v>2.4</x:v>
+        <x:v>0.2937</x:v>
       </x:c>
       <x:c r="H19" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C160404.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C53035082</x:v>
       </x:c>
       <x:c r="I19" s="7" t="str">
-        <x:v>https://www.jst-mfg.com/product/pdf/eng/eSH.pdf</x:v>
+        <x:v>https://www.jdtfuse.com/upload/PDF/JFC1032TS.pdf</x:v>
       </x:c>
       <x:c r="J19" s="7" t="str">
-        <x:v>SM04B-SRSS-TB(LF)(SN)</x:v>
+        <x:v>JFC1032-1200TS</x:v>
       </x:c>
       <x:c r="K19" s="7" t="str">
-        <x:v>JST</x:v>
+        <x:v>JDTfuse</x:v>
       </x:c>
       <x:c r="L19" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M19" s="7" t="str">
-        <x:v>Standard Qwiic pin order: 1 GND, 2 3.3 V, 3 SDA, 4 SCL. J9 is the dedicated MASTER port; J1/J12/J17 power local SENSOR modules. J9 power/signal nets are separated by U13.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="53" customHeight="1">
+        <x:v>Corrected centered origin and JDT land pattern. Check the new placement preview.</x:v>
+      </x:c>
+      <x:c r="N19" s="31"/>
+      <x:c r="O19" s="32"/>
+      <x:c r="P19" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q19" s="32" t="n">
+        <x:v>1504</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="72" customHeight="1">
       <x:c r="A20" s="11" t="str">
-        <x:v>PJ-082BH</x:v>
+        <x:v>JST SH 4-pin 1.00mm</x:v>
       </x:c>
       <x:c r="B20" s="11" t="str">
-        <x:v>J2</x:v>
+        <x:v>J1, J9, J12, J17</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
-        <x:v>RheoBoard:PJ-082BH</x:v>
+        <x:v>Connector_JST:JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</x:v>
       </x:c>
       <x:c r="D20" s="11" t="str">
-        <x:v>C3094233</x:v>
+        <x:v>C160404</x:v>
       </x:c>
       <x:c r="E20" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F20" s="13" t="n">
-        <x:v>1.58</x:v>
+        <x:v>0.2148</x:v>
       </x:c>
       <x:c r="G20" s="13" t="n">
         <x:f>IF(ISNUMBER(F20),E20*F20,"")</x:f>
-        <x:v>1.58</x:v>
+        <x:v>0.8592</x:v>
       </x:c>
       <x:c r="H20" s="11" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C3094233.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C160404</x:v>
       </x:c>
       <x:c r="I20" s="11" t="str">
-        <x:v>https://www.sameskydevices.com/product/resource/pj-082bh.pdf</x:v>
+        <x:v>https://www.jst-mfg.com/product/pdf/eng/eSH.pdf</x:v>
       </x:c>
       <x:c r="J20" s="11" t="str">
+        <x:v>SM04B-SRSS-TB(LF)(SN)</x:v>
+      </x:c>
+      <x:c r="K20" s="11" t="str">
+        <x:v>JST</x:v>
+      </x:c>
+      <x:c r="L20" s="11" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M20" s="11" t="str">
+        <x:v>Standard Qwiic pin order: 1 GND, 2 3.3 V, 3 SDA, 4 SCL. J9 is the dedicated MASTER port; J1/J12/J17 power local SENSOR modules. J9 power/signal nets are separated by U13.</x:v>
+      </x:c>
+      <x:c r="N20" s="31"/>
+      <x:c r="O20" s="32"/>
+      <x:c r="P20" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q20" s="32" t="n">
+        <x:v>65620</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="72" customHeight="1">
+      <x:c r="A21" s="11" t="str">
         <x:v>PJ-082BH</x:v>
       </x:c>
-      <x:c r="K20" s="11" t="str">
-        <x:v>CUI</x:v>
-      </x:c>
-      <x:c r="L20" s="11" t="str">
-        <x:v>Manual THT</x:v>
-      </x:c>
-      <x:c r="M20" s="11" t="str">
-        <x:v>Manual through-hole assembly. Center-positive 12 V, 5.5 x 2.5 mm mating plug.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="53" customHeight="1">
-      <x:c r="A21" s="11" t="str">
-        <x:v>JST EH 4-pin 2.50mm</x:v>
-      </x:c>
       <x:c r="B21" s="11" t="str">
-        <x:v>J3</x:v>
+        <x:v>J2</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
-        <x:v>RheoBoard:JST_EH_B4B-EH-A_1x04_P2.50mm_Vertical_DFM</x:v>
+        <x:v>RheoBoard:PJ-082BH</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
-        <x:v>C160258</x:v>
+        <x:v>C3094233</x:v>
       </x:c>
       <x:c r="E21" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F21" s="13" t="n">
-        <x:v>0.139</x:v>
+        <x:f>'Parts cost'!G18/'Parts cost'!E18</x:f>
+        <x:v>2.608</x:v>
       </x:c>
       <x:c r="G21" s="13" t="n">
         <x:f>IF(ISNUMBER(F21),E21*F21,"")</x:f>
-        <x:v>0.139</x:v>
+        <x:v>2.608</x:v>
       </x:c>
       <x:c r="H21" s="11" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C160258.html</x:v>
+        <x:v>https://www.lcsc.com/product-detail/C3094233.html</x:v>
       </x:c>
       <x:c r="I21" s="11" t="str">
-        <x:v>https://www.jst-mfg.com/product/pdf/eng/eEH.pdf</x:v>
+        <x:v>https://www.sameskydevices.com/product/resource/pj-082bh.pdf</x:v>
       </x:c>
       <x:c r="J21" s="11" t="str">
-        <x:v>B4B-EH-A(LF)(SN)</x:v>
+        <x:v>PJ-082BH</x:v>
       </x:c>
       <x:c r="K21" s="11" t="str">
-        <x:v>JST</x:v>
+        <x:v>CUI</x:v>
       </x:c>
       <x:c r="L21" s="11" t="str">
         <x:v>Manual THT</x:v>
       </x:c>
       <x:c r="M21" s="11" t="str">
-        <x:v>Manual through-hole assembly. Pin 2 supplies local 3.3 V to peripherals.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="53" customHeight="1">
+        <x:v>Manual through-hole assembly. Center-positive 12 V, 5.5 x 2.5 mm mating plug.</x:v>
+      </x:c>
+      <x:c r="N21" s="31"/>
+      <x:c r="O21" s="32"/>
+      <x:c r="P21" s="32"/>
+      <x:c r="Q21" s="32"/>
+    </x:row>
+    <x:row r="22" ht="72" customHeight="1">
       <x:c r="A22" s="7" t="str">
-        <x:v>4.7uH FXL0530-4R7-M</x:v>
+        <x:v>JST EH 4-pin 2.50mm</x:v>
       </x:c>
       <x:c r="B22" s="7" t="str">
-        <x:v>L1, L2, L5</x:v>
+        <x:v>J3</x:v>
       </x:c>
       <x:c r="C22" s="7" t="str">
-        <x:v>Inductor_SMD:L_Changjiang_FXL0530</x:v>
+        <x:v>RheoBoard:JST_EH_B4B-EH-A_1x04_P2.50mm_Vertical_DFM</x:v>
       </x:c>
       <x:c r="D22" s="7" t="str">
-        <x:v>C177246</x:v>
+        <x:v>C160258</x:v>
       </x:c>
       <x:c r="E22" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F22" s="9" t="n">
-        <x:v>0.904</x:v>
+        <x:f>'Parts cost'!G19/'Parts cost'!E19</x:f>
+        <x:v>0.0613</x:v>
       </x:c>
       <x:c r="G22" s="9" t="n">
         <x:f>IF(ISNUMBER(F22),E22*F22,"")</x:f>
-        <x:v>2.712</x:v>
+        <x:v>0.0613</x:v>
       </x:c>
       <x:c r="H22" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C177246.html</x:v>
-      </x:c>
-      <x:c r="I22" s="7"/>
+        <x:v>https://www.lcsc.com/product-detail/C160258.html</x:v>
+      </x:c>
+      <x:c r="I22" s="7" t="str">
+        <x:v>https://www.jst-mfg.com/product/pdf/eng/eEH.pdf</x:v>
+      </x:c>
       <x:c r="J22" s="7" t="str">
-        <x:v>FXL0530-4R7-M</x:v>
+        <x:v>B4B-EH-A(LF)(SN)</x:v>
       </x:c>
       <x:c r="K22" s="7" t="str">
-        <x:v>cjiang</x:v>
+        <x:v>JST</x:v>
       </x:c>
       <x:c r="L22" s="7" t="str">
-        <x:v>SMT</x:v>
+        <x:v>Manual THT</x:v>
       </x:c>
       <x:c r="M22" s="7" t="str">
-        <x:v>FXL0530 pads match the selected inductor; old Bourns purchasing link removed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="53" customHeight="1">
+        <x:v>Manual through-hole assembly. Pin 2 supplies local 3.3 V to peripherals.</x:v>
+      </x:c>
+      <x:c r="N22" s="31"/>
+      <x:c r="O22" s="32"/>
+      <x:c r="P22" s="32"/>
+      <x:c r="Q22" s="32"/>
+    </x:row>
+    <x:row r="23" ht="72" customHeight="1">
       <x:c r="A23" s="7" t="str">
-        <x:v>AO3400A</x:v>
+        <x:v>4.7uH FXL0530-4R7-M</x:v>
       </x:c>
       <x:c r="B23" s="7" t="str">
-        <x:v>Q4, Q8, Q10</x:v>
+        <x:v>L1, L2, L5</x:v>
       </x:c>
       <x:c r="C23" s="7" t="str">
-        <x:v>RheoBoard:AO3400A</x:v>
+        <x:v>Inductor_SMD:L_Changjiang_FXL0530</x:v>
       </x:c>
       <x:c r="D23" s="7" t="str">
-        <x:v>C20917</x:v>
+        <x:v>C177246</x:v>
       </x:c>
       <x:c r="E23" s="8" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F23" s="9" t="n">
-        <x:v>0.322</x:v>
+        <x:v>0.1244</x:v>
       </x:c>
       <x:c r="G23" s="9" t="n">
         <x:f>IF(ISNUMBER(F23),E23*F23,"")</x:f>
-        <x:v>0.966</x:v>
+        <x:v>0.3732</x:v>
       </x:c>
       <x:c r="H23" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C20917.html</x:v>
-      </x:c>
-      <x:c r="I23" s="7" t="str">
-        <x:v>https://www.aosmd.com/sites/default/files/res/data_sheets/AO3400A.pdf</x:v>
-      </x:c>
+        <x:v>https://jlcpcb.com/partdetail/component/C177246</x:v>
+      </x:c>
+      <x:c r="I23" s="7"/>
       <x:c r="J23" s="7" t="str">
-        <x:v>AO3400A</x:v>
+        <x:v>FXL0530-4R7-M</x:v>
       </x:c>
       <x:c r="K23" s="7" t="str">
-        <x:v>AOS</x:v>
+        <x:v>cjiang</x:v>
       </x:c>
       <x:c r="L23" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M23" s="7"/>
-    </x:row>
-    <x:row r="24" ht="53" customHeight="1">
+      <x:c r="M23" s="7" t="str">
+        <x:v>FXL0530 pads match the selected inductor; old Bourns purchasing link removed.</x:v>
+      </x:c>
+      <x:c r="N23" s="31" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="O23" s="32" t="str">
+        <x:v>Retain FXL0530-4R7-M. Any substitute needs current, saturation, DCR, height and pad-fit review; inductance tolerance alone is insufficient.</x:v>
+      </x:c>
+      <x:c r="P23" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q23" s="32" t="n">
+        <x:v>51637</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="72" customHeight="1">
       <x:c r="A24" s="7" t="str">
-        <x:v>100K/0603/1%</x:v>
+        <x:v>AO3400A</x:v>
       </x:c>
       <x:c r="B24" s="7" t="str">
-        <x:v>R1, R4, R7</x:v>
+        <x:v>Q4, Q8, Q10</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
+        <x:v>RheoBoard:AO3400A</x:v>
       </x:c>
       <x:c r="D24" s="7" t="str">
-        <x:v>C25803</x:v>
+        <x:v>C20917</x:v>
       </x:c>
       <x:c r="E24" s="8" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F24" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.0889</x:v>
       </x:c>
       <x:c r="G24" s="9" t="n">
         <x:f>IF(ISNUMBER(F24),E24*F24,"")</x:f>
-        <x:v>0.042</x:v>
+        <x:v>0.26670000000000005</x:v>
       </x:c>
       <x:c r="H24" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25803.html</x:v>
-      </x:c>
-      <x:c r="I24" s="7"/>
+        <x:v>https://jlcpcb.com/partdetail/component/C20917</x:v>
+      </x:c>
+      <x:c r="I24" s="7" t="str">
+        <x:v>https://www.aosmd.com/sites/default/files/res/data_sheets/AO3400A.pdf</x:v>
+      </x:c>
       <x:c r="J24" s="7" t="str">
-        <x:v>0603WAF1003T5E</x:v>
+        <x:v>AO3400A</x:v>
       </x:c>
       <x:c r="K24" s="7" t="str">
-        <x:v>UNI-ROYAL</x:v>
+        <x:v>AOS</x:v>
       </x:c>
       <x:c r="L24" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M24" s="7"/>
-    </x:row>
-    <x:row r="25" ht="53" customHeight="1">
+      <x:c r="N24" s="31"/>
+      <x:c r="O24" s="32"/>
+      <x:c r="P24" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q24" s="32" t="n">
+        <x:v>994885</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="72" customHeight="1">
       <x:c r="A25" s="7" t="str">
-        <x:v>4K7/0603/1%</x:v>
+        <x:v>100K/0603/1%</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
-        <x:v>R15, R20, R82, R83</x:v>
+        <x:v>R1, R4, R7</x:v>
       </x:c>
       <x:c r="C25" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D25" s="7" t="str">
-        <x:v>C23162</x:v>
+        <x:v>C25803</x:v>
       </x:c>
       <x:c r="E25" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F25" s="9" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.0031</x:v>
       </x:c>
       <x:c r="G25" s="9" t="n">
         <x:f>IF(ISNUMBER(F25),E25*F25,"")</x:f>
-        <x:v>0.004</x:v>
+        <x:v>0.0093</x:v>
       </x:c>
       <x:c r="H25" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C23162.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C25803</x:v>
       </x:c>
       <x:c r="I25" s="7"/>
       <x:c r="J25" s="7" t="str">
-        <x:v>0603WAF4701T5E</x:v>
+        <x:v>0603WAF1003T5E</x:v>
       </x:c>
       <x:c r="K25" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1413,39 +1798,49 @@
       <x:c r="L25" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M25" s="7" t="str">
-        <x:v>R82/R83 added as 4.7 kohm host SDA/SCL pullups; local R15/R20 retained.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="126" customHeight="1">
+      <x:c r="M25" s="7"/>
+      <x:c r="N25" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O25" s="32" t="str">
+        <x:v>5% or better. Same value and 0603 package; &gt;=0.1 W and original voltage rating. Retain cheaper selected 1% part when available.</x:v>
+      </x:c>
+      <x:c r="P25" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q25" s="32" t="n">
+        <x:v>15325462</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="72" customHeight="1">
       <x:c r="A26" s="7" t="str">
-        <x:v>10K/0603/1%</x:v>
+        <x:v>4K7/0603/1%</x:v>
       </x:c>
       <x:c r="B26" s="7" t="str">
-        <x:v>R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84, R85</x:v>
+        <x:v>R15, R20, R82, R83</x:v>
       </x:c>
       <x:c r="C26" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D26" s="7" t="str">
-        <x:v>C25804</x:v>
+        <x:v>C23162</x:v>
       </x:c>
       <x:c r="E26" s="8" t="n">
-        <x:v>18</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F26" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.0028</x:v>
       </x:c>
       <x:c r="G26" s="9" t="n">
         <x:f>IF(ISNUMBER(F26),E26*F26,"")</x:f>
-        <x:v>0.252</x:v>
+        <x:v>0.0112</x:v>
       </x:c>
       <x:c r="H26" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25804.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C23162</x:v>
       </x:c>
       <x:c r="I26" s="7"/>
       <x:c r="J26" s="7" t="str">
-        <x:v>0603WAF1002T5E</x:v>
+        <x:v>0603WAF4701T5E</x:v>
       </x:c>
       <x:c r="K26" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1454,38 +1849,50 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M26" s="7" t="str">
-        <x:v>R16–R19 pull the button signals to HOST_3V3 from J9. R84 discharges HOST_3V3. R85 pulls Q11 gate to GND.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="53" customHeight="1">
+        <x:v>R82/R83 added as 4.7 kohm host SDA/SCL pullups; local R15/R20 retained.</x:v>
+      </x:c>
+      <x:c r="N26" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O26" s="32" t="str">
+        <x:v>5% or better. Same value and 0603 package; &gt;=0.1 W and original voltage rating. Retain cheaper selected 1% part when available.</x:v>
+      </x:c>
+      <x:c r="P26" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q26" s="32" t="n">
+        <x:v>13375910</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="170" customHeight="1">
       <x:c r="A27" s="7" t="str">
-        <x:v>1k/0603/1%</x:v>
+        <x:v>10K/0603/1%</x:v>
       </x:c>
       <x:c r="B27" s="7" t="str">
-        <x:v>R24, R25, R26, R39, R40, R54, R59, R75</x:v>
+        <x:v>R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84, R85</x:v>
       </x:c>
       <x:c r="C27" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D27" s="7" t="str">
-        <x:v>C21190</x:v>
+        <x:v>C25804</x:v>
       </x:c>
       <x:c r="E27" s="8" t="n">
-        <x:v>8</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F27" s="9" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.0018</x:v>
       </x:c>
       <x:c r="G27" s="9" t="n">
         <x:f>IF(ISNUMBER(F27),E27*F27,"")</x:f>
-        <x:v>0.008</x:v>
+        <x:v>0.0324</x:v>
       </x:c>
       <x:c r="H27" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C21190.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C25804</x:v>
       </x:c>
       <x:c r="I27" s="7"/>
       <x:c r="J27" s="7" t="str">
-        <x:v>0603WAF1001T5E</x:v>
+        <x:v>0603WAF1002T5E</x:v>
       </x:c>
       <x:c r="K27" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1493,37 +1900,51 @@
       <x:c r="L27" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M27" s="7"/>
-    </x:row>
-    <x:row r="28" ht="53" customHeight="1">
+      <x:c r="M27" s="7" t="str">
+        <x:v>R16–R19 pull the button signals to HOST_3V3 from J9. R84 discharges HOST_3V3. R85 pulls Q11 gate to GND.</x:v>
+      </x:c>
+      <x:c r="N27" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O27" s="32" t="str">
+        <x:v>5% or better. Same value and 0603 package; &gt;=0.1 W and original voltage rating. Retain cheaper selected 1% part when available.</x:v>
+      </x:c>
+      <x:c r="P27" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q27" s="32" t="n">
+        <x:v>28532408</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="72" customHeight="1">
       <x:c r="A28" s="7" t="str">
-        <x:v>100R/0603/1%</x:v>
+        <x:v>1k/0603/1%</x:v>
       </x:c>
       <x:c r="B28" s="7" t="str">
-        <x:v>R35, R36, R42, R55</x:v>
+        <x:v>R24, R25, R26, R39, R40, R54, R59, R75</x:v>
       </x:c>
       <x:c r="C28" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D28" s="7" t="str">
-        <x:v>C22775</x:v>
+        <x:v>C21190</x:v>
       </x:c>
       <x:c r="E28" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F28" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.0017</x:v>
       </x:c>
       <x:c r="G28" s="9" t="n">
         <x:f>IF(ISNUMBER(F28),E28*F28,"")</x:f>
-        <x:v>0.056</x:v>
+        <x:v>0.0136</x:v>
       </x:c>
       <x:c r="H28" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22775.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C21190</x:v>
       </x:c>
       <x:c r="I28" s="7"/>
       <x:c r="J28" s="7" t="str">
-        <x:v>0603WAF1000T5E</x:v>
+        <x:v>0603WAF1001T5E</x:v>
       </x:c>
       <x:c r="K28" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1532,36 +1953,48 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M28" s="7"/>
-    </x:row>
-    <x:row r="29" ht="53" customHeight="1">
+      <x:c r="N28" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O28" s="32" t="str">
+        <x:v>5% or better. Same value and 0603 package; &gt;=0.1 W and original voltage rating. Retain cheaper selected 1% part when available.</x:v>
+      </x:c>
+      <x:c r="P28" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q28" s="32" t="n">
+        <x:v>26905773</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="72" customHeight="1">
       <x:c r="A29" s="7" t="str">
-        <x:v>330/0603/1%</x:v>
+        <x:v>100R/0603/1%</x:v>
       </x:c>
       <x:c r="B29" s="7" t="str">
-        <x:v>R44, R77</x:v>
+        <x:v>R35, R36, R42, R55</x:v>
       </x:c>
       <x:c r="C29" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D29" s="7" t="str">
-        <x:v>C23138</x:v>
+        <x:v>C22775</x:v>
       </x:c>
       <x:c r="E29" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F29" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.0023</x:v>
       </x:c>
       <x:c r="G29" s="9" t="n">
         <x:f>IF(ISNUMBER(F29),E29*F29,"")</x:f>
-        <x:v>0.028</x:v>
+        <x:v>0.0092</x:v>
       </x:c>
       <x:c r="H29" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C23138.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C22775</x:v>
       </x:c>
       <x:c r="I29" s="7"/>
       <x:c r="J29" s="7" t="str">
-        <x:v>0603WAF3300T5E</x:v>
+        <x:v>0603WAF1000T5E</x:v>
       </x:c>
       <x:c r="K29" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1570,114 +2003,150 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M29" s="7"/>
-    </x:row>
-    <x:row r="30" ht="53" customHeight="1">
+      <x:c r="N29" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O29" s="32" t="str">
+        <x:v>5% or better. Same value and 0603 package; &gt;=0.1 W and original voltage rating. Retain cheaper selected 1% part when available.</x:v>
+      </x:c>
+      <x:c r="P29" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q29" s="32" t="n">
+        <x:v>8109445</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="72" customHeight="1">
       <x:c r="A30" s="7" t="str">
-        <x:v>196k ±1%</x:v>
+        <x:v>330/0603/1%</x:v>
       </x:c>
       <x:c r="B30" s="7" t="str">
-        <x:v>R45</x:v>
+        <x:v>R44, R77</x:v>
       </x:c>
       <x:c r="C30" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D30" s="7" t="str">
-        <x:v>C4203218</x:v>
+        <x:v>C23138</x:v>
       </x:c>
       <x:c r="E30" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F30" s="9" t="n">
-        <x:v>0.02</x:v>
+        <x:v>0.002</x:v>
       </x:c>
       <x:c r="G30" s="9" t="n">
         <x:f>IF(ISNUMBER(F30),E30*F30,"")</x:f>
-        <x:v>0.02</x:v>
+        <x:v>0.004</x:v>
       </x:c>
       <x:c r="H30" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C4203218.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C23138</x:v>
       </x:c>
       <x:c r="I30" s="7"/>
       <x:c r="J30" s="7" t="str">
-        <x:v>CRCW0603196KFKEA</x:v>
+        <x:v>0603WAF3300T5E</x:v>
       </x:c>
       <x:c r="K30" s="7" t="str">
-        <x:v>VISHAY</x:v>
+        <x:v>UNI-ROYAL</x:v>
       </x:c>
       <x:c r="L30" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M30" s="7" t="str">
-        <x:v>Schematic corrected to the assembled 196k value; pump rail approximately 4.52 V.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="53" customHeight="1">
+      <x:c r="M30" s="7"/>
+      <x:c r="N30" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O30" s="32" t="str">
+        <x:v>5% or better. Same value and 0603 package; &gt;=0.1 W and original voltage rating. Retain cheaper selected 1% part when available.</x:v>
+      </x:c>
+      <x:c r="P30" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q30" s="32" t="n">
+        <x:v>3123833</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="72" customHeight="1">
       <x:c r="A31" s="7" t="str">
-        <x:v>30K/0603/1%</x:v>
+        <x:v>196k ±1%</x:v>
       </x:c>
       <x:c r="B31" s="7" t="str">
-        <x:v>R46, R74, R76</x:v>
+        <x:v>R45</x:v>
       </x:c>
       <x:c r="C31" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D31" s="7" t="str">
-        <x:v>C22984</x:v>
+        <x:v>C4203218</x:v>
       </x:c>
       <x:c r="E31" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F31" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.0149</x:v>
       </x:c>
       <x:c r="G31" s="9" t="n">
         <x:f>IF(ISNUMBER(F31),E31*F31,"")</x:f>
-        <x:v>0.042</x:v>
+        <x:v>0.0149</x:v>
       </x:c>
       <x:c r="H31" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22984.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C4203218</x:v>
       </x:c>
       <x:c r="I31" s="7"/>
       <x:c r="J31" s="7" t="str">
-        <x:v>0603WAF3002T5E</x:v>
+        <x:v>CRCW0603196KFKEA</x:v>
       </x:c>
       <x:c r="K31" s="7" t="str">
-        <x:v>UNI-ROYAL</x:v>
+        <x:v>VISHAY</x:v>
       </x:c>
       <x:c r="L31" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M31" s="7"/>
-    </x:row>
-    <x:row r="32" ht="53" customHeight="1">
+      <x:c r="M31" s="7" t="str">
+        <x:v>Schematic corrected to the assembled 196k value; pump rail approximately 4.52 V.</x:v>
+      </x:c>
+      <x:c r="N31" s="31" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="O31" s="32" t="str">
+        <x:v>Feedback/protection: 1% or better. Same value, package, ratings and TCR.</x:v>
+      </x:c>
+      <x:c r="P31" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q31" s="32" t="n">
+        <x:v>1482</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="72" customHeight="1">
       <x:c r="A32" s="7" t="str">
-        <x:v>270K/0603/1%</x:v>
+        <x:v>30K/0603/1%</x:v>
       </x:c>
       <x:c r="B32" s="7" t="str">
-        <x:v>R60</x:v>
+        <x:v>R46, R74</x:v>
       </x:c>
       <x:c r="C32" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D32" s="7" t="str">
-        <x:v>C22965</x:v>
+        <x:v>C22984</x:v>
       </x:c>
       <x:c r="E32" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F32" s="9" t="n">
-        <x:v>0.001</x:v>
+        <x:v>0.0047</x:v>
       </x:c>
       <x:c r="G32" s="9" t="n">
         <x:f>IF(ISNUMBER(F32),E32*F32,"")</x:f>
-        <x:v>0.001</x:v>
+        <x:v>0.0094</x:v>
       </x:c>
       <x:c r="H32" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22965.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C22984</x:v>
       </x:c>
       <x:c r="I32" s="7"/>
       <x:c r="J32" s="7" t="str">
-        <x:v>0603WAF2703T5E</x:v>
+        <x:v>0603WAF3002T5E</x:v>
       </x:c>
       <x:c r="K32" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1686,74 +2155,100 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M32" s="7"/>
-    </x:row>
-    <x:row r="33" ht="53" customHeight="1">
+      <x:c r="N32" s="31" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="O32" s="32" t="str">
+        <x:v>Feedback/protection: 1% or better. Same value, package, ratings and TCR.</x:v>
+      </x:c>
+      <x:c r="P32" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q32" s="32" t="n">
+        <x:v>1902045</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="72" customHeight="1">
       <x:c r="A33" s="7" t="str">
-        <x:v>135k ±0.1%</x:v>
+        <x:v>22k ±1%</x:v>
       </x:c>
       <x:c r="B33" s="7" t="str">
-        <x:v>R61</x:v>
+        <x:v>R76</x:v>
       </x:c>
       <x:c r="C33" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D33" s="7" t="str">
-        <x:v>C861113</x:v>
+        <x:v>C31850</x:v>
       </x:c>
       <x:c r="E33" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F33" s="9" t="n">
-        <x:v>0.06</x:v>
+        <x:v>0.0042</x:v>
       </x:c>
       <x:c r="G33" s="9" t="n">
         <x:f>IF(ISNUMBER(F33),E33*F33,"")</x:f>
-        <x:v>0.06</x:v>
+        <x:v>0.0042</x:v>
       </x:c>
       <x:c r="H33" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C861113.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C31850</x:v>
       </x:c>
       <x:c r="I33" s="7"/>
       <x:c r="J33" s="7" t="str">
-        <x:v>RT0603BRD07135KL</x:v>
+        <x:v>0603WAF2202T5E</x:v>
       </x:c>
       <x:c r="K33" s="7" t="str">
-        <x:v>YAGEO</x:v>
+        <x:v>UNI-ROYAL</x:v>
       </x:c>
       <x:c r="L33" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M33" s="7"/>
-    </x:row>
-    <x:row r="34" ht="53" customHeight="1">
+      <x:c r="M33" s="7" t="str">
+        <x:v>U3 lower feedback resistor; paired with R61 100k.</x:v>
+      </x:c>
+      <x:c r="N33" s="31" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="O33" s="32" t="str">
+        <x:v>Feedback/protection: 1% or better. Same value, package, ratings and TCR.</x:v>
+      </x:c>
+      <x:c r="P33" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q33" s="32" t="n">
+        <x:v>2766862</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="72" customHeight="1">
       <x:c r="A34" s="7" t="str">
-        <x:v>549R ±1%</x:v>
+        <x:v>270K/0603/1%</x:v>
       </x:c>
       <x:c r="B34" s="7" t="str">
-        <x:v>R73</x:v>
+        <x:v>R60</x:v>
       </x:c>
       <x:c r="C34" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D34" s="7" t="str">
-        <x:v>C23079</x:v>
+        <x:v>C22965</x:v>
       </x:c>
       <x:c r="E34" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F34" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.0018</x:v>
       </x:c>
       <x:c r="G34" s="9" t="n">
         <x:f>IF(ISNUMBER(F34),E34*F34,"")</x:f>
-        <x:v>0.014</x:v>
+        <x:v>0.0018</x:v>
       </x:c>
       <x:c r="H34" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C23079.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C22965</x:v>
       </x:c>
       <x:c r="I34" s="7"/>
       <x:c r="J34" s="7" t="str">
-        <x:v>0603WAF5490T5E</x:v>
+        <x:v>0603WAF2703T5E</x:v>
       </x:c>
       <x:c r="K34" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1761,36 +2256,49 @@
       <x:c r="L34" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M34" s="7" t="str">
-        <x:v>Schematic corrected to the assembled 549 ohm value.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="53" customHeight="1">
+      <x:c r="M34" s="7"/>
+      <x:c r="N34" s="31" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="O34" s="32" t="str">
+        <x:v>Feedback/protection: 1% or better. Same value, package, ratings and TCR.</x:v>
+      </x:c>
+      <x:c r="P34" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q34" s="32" t="n">
+        <x:v>220840</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="72" customHeight="1">
       <x:c r="A35" s="7" t="str">
-        <x:v>680k ±1%</x:v>
+        <x:v>100k ±1%</x:v>
       </x:c>
       <x:c r="B35" s="7" t="str">
-        <x:v>R78</x:v>
+        <x:v>R61</x:v>
       </x:c>
       <x:c r="C35" s="7" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D35" s="7" t="str">
-        <x:v>C25822</x:v>
+        <x:v>C25803</x:v>
       </x:c>
       <x:c r="E35" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F35" s="10"/>
-      <x:c r="G35" s="9" t="str">
+      <x:c r="F35" s="10" t="n">
+        <x:v>0.0031</x:v>
+      </x:c>
+      <x:c r="G35" s="9" t="n">
         <x:f>IF(ISNUMBER(F35),E35*F35,"")</x:f>
+        <x:v>0.0031</x:v>
       </x:c>
       <x:c r="H35" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25822.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C25803</x:v>
       </x:c>
       <x:c r="I35" s="7"/>
       <x:c r="J35" s="7" t="str">
-        <x:v>0603WAF6803T5E</x:v>
+        <x:v>0603WAF1003T5E</x:v>
       </x:c>
       <x:c r="K35" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1798,37 +2306,51 @@
       <x:c r="L35" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M35" s="7"/>
-    </x:row>
-    <x:row r="36" ht="53" customHeight="1">
+      <x:c r="M35" s="7" t="str">
+        <x:v>U3 3.3 V feedback: 100k/22k gives 3.327 V nominal. Use 1% resistors.</x:v>
+      </x:c>
+      <x:c r="N35" s="31" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="O35" s="32" t="str">
+        <x:v>Feedback/protection: 1% or better. Same value, package, ratings and TCR.</x:v>
+      </x:c>
+      <x:c r="P35" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q35" s="32" t="n">
+        <x:v>15325462</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="72" customHeight="1">
       <x:c r="A36" s="7" t="str">
-        <x:v>100K/0603/1%</x:v>
+        <x:v>560R ±1%</x:v>
       </x:c>
       <x:c r="B36" s="7" t="str">
-        <x:v>R79</x:v>
+        <x:v>R73</x:v>
       </x:c>
       <x:c r="C36" s="7" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D36" s="7" t="str">
-        <x:v>C25803</x:v>
+        <x:v>C23204</x:v>
       </x:c>
       <x:c r="E36" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F36" s="9" t="n">
-        <x:v>0.014</x:v>
+        <x:v>0.0034</x:v>
       </x:c>
       <x:c r="G36" s="9" t="n">
         <x:f>IF(ISNUMBER(F36),E36*F36,"")</x:f>
-        <x:v>0.014</x:v>
+        <x:v>0.0034</x:v>
       </x:c>
       <x:c r="H36" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C25803.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C23204</x:v>
       </x:c>
       <x:c r="I36" s="7"/>
       <x:c r="J36" s="7" t="str">
-        <x:v>0603WAF1003T5E</x:v>
+        <x:v>0603WAF5600T5E</x:v>
       </x:c>
       <x:c r="K36" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1836,34 +2358,51 @@
       <x:c r="L36" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M36" s="7"/>
-    </x:row>
-    <x:row r="37" ht="53" customHeight="1">
+      <x:c r="M36" s="7" t="str">
+        <x:v>560 ohm standard value replaces 549 ohm. LED current falls approximately 2%.</x:v>
+      </x:c>
+      <x:c r="N36" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O36" s="32" t="str">
+        <x:v>5% or better. Same value and 0603 package; &gt;=0.1 W and original voltage rating. Retain cheaper selected 1% part when available.</x:v>
+      </x:c>
+      <x:c r="P36" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q36" s="32" t="n">
+        <x:v>2541355</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="72" customHeight="1">
       <x:c r="A37" s="7" t="str">
-        <x:v>390k ±1%</x:v>
+        <x:v>680k ±1%</x:v>
       </x:c>
       <x:c r="B37" s="7" t="str">
-        <x:v>R80</x:v>
+        <x:v>R78</x:v>
       </x:c>
       <x:c r="C37" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D37" s="7" t="str">
-        <x:v>C2759410</x:v>
+        <x:v>C25822</x:v>
       </x:c>
       <x:c r="E37" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F37" s="10"/>
-      <x:c r="G37" s="9" t="str">
+      <x:c r="F37" s="10" t="n">
+        <x:v>0.0015</x:v>
+      </x:c>
+      <x:c r="G37" s="9" t="n">
         <x:f>IF(ISNUMBER(F37),E37*F37,"")</x:f>
+        <x:v>0.0015</x:v>
       </x:c>
       <x:c r="H37" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C2759410.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C25822</x:v>
       </x:c>
       <x:c r="I37" s="7"/>
       <x:c r="J37" s="7" t="str">
-        <x:v>HP03W5F3903T5E</x:v>
+        <x:v>0603WAF6803T5E</x:v>
       </x:c>
       <x:c r="K37" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1872,33 +2411,48 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M37" s="7"/>
-    </x:row>
-    <x:row r="38" ht="53" customHeight="1">
+      <x:c r="N37" s="31" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="O37" s="32" t="str">
+        <x:v>Feedback/protection: 1% or better. Same value, package, ratings and TCR.</x:v>
+      </x:c>
+      <x:c r="P37" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q37" s="32" t="n">
+        <x:v>1045292</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="72" customHeight="1">
       <x:c r="A38" s="7" t="str">
-        <x:v>1.65k ±1%</x:v>
+        <x:v>100K/0603/1%</x:v>
       </x:c>
       <x:c r="B38" s="7" t="str">
-        <x:v>R81</x:v>
+        <x:v>R79</x:v>
       </x:c>
       <x:c r="C38" s="7" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D38" s="7" t="str">
-        <x:v>C22845</x:v>
+        <x:v>C25803</x:v>
       </x:c>
       <x:c r="E38" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F38" s="10"/>
-      <x:c r="G38" s="9" t="str">
+      <x:c r="F38" s="10" t="n">
+        <x:v>0.0031</x:v>
+      </x:c>
+      <x:c r="G38" s="9" t="n">
         <x:f>IF(ISNUMBER(F38),E38*F38,"")</x:f>
+        <x:v>0.0031</x:v>
       </x:c>
       <x:c r="H38" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22845.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C25803</x:v>
       </x:c>
       <x:c r="I38" s="7"/>
       <x:c r="J38" s="7" t="str">
-        <x:v>0603WAF1651T5E</x:v>
+        <x:v>0603WAF1003T5E</x:v>
       </x:c>
       <x:c r="K38" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -1907,532 +2461,725 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M38" s="7"/>
-    </x:row>
-    <x:row r="39" ht="53" customHeight="1">
+      <x:c r="N38" s="31" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="O38" s="32" t="str">
+        <x:v>Feedback/protection: 1% or better. Same value, package, ratings and TCR.</x:v>
+      </x:c>
+      <x:c r="P38" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q38" s="32" t="n">
+        <x:v>15325462</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="72" customHeight="1">
       <x:c r="A39" s="7" t="str">
-        <x:v>TL3301NF160QG/P010515</x:v>
+        <x:v>390k ±1%</x:v>
       </x:c>
       <x:c r="B39" s="7" t="str">
-        <x:v>SW1, SW2, SW3, SW4</x:v>
+        <x:v>R80</x:v>
       </x:c>
       <x:c r="C39" s="7" t="str">
-        <x:v>RheoBoard:Tactile_Switch_4pad</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D39" s="7" t="str">
-        <x:v>C273527</x:v>
+        <x:v>C2759410</x:v>
       </x:c>
       <x:c r="E39" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F39" s="9" t="n">
-        <x:v>0.183</x:v>
+        <x:v>0.0022</x:v>
       </x:c>
       <x:c r="G39" s="9" t="n">
         <x:f>IF(ISNUMBER(F39),E39*F39,"")</x:f>
-        <x:v>0.732</x:v>
+        <x:v>0.0022</x:v>
       </x:c>
       <x:c r="H39" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C273527.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C2759410</x:v>
       </x:c>
       <x:c r="I39" s="7"/>
       <x:c r="J39" s="7" t="str">
-        <x:v>TL3301NF160QG/P010515</x:v>
+        <x:v>HP03W5F3903T5E</x:v>
       </x:c>
       <x:c r="K39" s="7" t="str">
-        <x:v>E-Switch</x:v>
+        <x:v>UNI-ROYAL</x:v>
       </x:c>
       <x:c r="L39" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M39" s="7"/>
-    </x:row>
-    <x:row r="40" ht="53" customHeight="1">
+      <x:c r="N39" s="31" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="O39" s="32" t="str">
+        <x:v>Feedback/protection: 1% or better. Same value, package, ratings and TCR.</x:v>
+      </x:c>
+      <x:c r="P39" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q39" s="32" t="n">
+        <x:v>4541</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="72" customHeight="1">
       <x:c r="A40" s="7" t="str">
-        <x:v>TPS563203DRLR</x:v>
+        <x:v>1.65k ±1%</x:v>
       </x:c>
       <x:c r="B40" s="7" t="str">
-        <x:v>U1, U2, U3</x:v>
+        <x:v>R81</x:v>
       </x:c>
       <x:c r="C40" s="7" t="str">
-        <x:v>RheoBoard:TPS563203DRLR</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D40" s="7" t="str">
-        <x:v>C22445512</x:v>
+        <x:v>C22845</x:v>
       </x:c>
       <x:c r="E40" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F40" s="9" t="n">
-        <x:v>0.225</x:v>
+        <x:v>0.0018</x:v>
       </x:c>
       <x:c r="G40" s="9" t="n">
         <x:f>IF(ISNUMBER(F40),E40*F40,"")</x:f>
-        <x:v>0.675</x:v>
+        <x:v>0.0018</x:v>
       </x:c>
       <x:c r="H40" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C22445512.html</x:v>
-      </x:c>
-      <x:c r="I40" s="7" t="str">
-        <x:v>https://www.ti.com/lit/gpn/tps563203</x:v>
-      </x:c>
+        <x:v>https://jlcpcb.com/partdetail/component/C22845</x:v>
+      </x:c>
+      <x:c r="I40" s="7"/>
       <x:c r="J40" s="7" t="str">
-        <x:v>TPS563203DRLR</x:v>
+        <x:v>0603WAF1651T5E</x:v>
       </x:c>
       <x:c r="K40" s="7" t="str">
-        <x:v>TI</x:v>
+        <x:v>UNI-ROYAL</x:v>
       </x:c>
       <x:c r="L40" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M40" s="7"/>
-    </x:row>
-    <x:row r="41" ht="68" customHeight="1">
+      <x:c r="N40" s="31" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="O40" s="32" t="str">
+        <x:v>Feedback/protection: 1% or better. Same value, package, ratings and TCR.</x:v>
+      </x:c>
+      <x:c r="P40" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q40" s="32" t="n">
+        <x:v>13058</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="72" customHeight="1">
       <x:c r="A41" s="7" t="str">
-        <x:v>MPRLS0025PA00001A</x:v>
+        <x:v>TL3301NF160QG/P010515</x:v>
       </x:c>
       <x:c r="B41" s="7" t="str">
-        <x:v>U5</x:v>
+        <x:v>SW1, SW2, SW3, SW4</x:v>
       </x:c>
       <x:c r="C41" s="7" t="str">
-        <x:v>RheoBoard:MPRLS0025PA00001A</x:v>
+        <x:v>RheoBoard:Tactile_Switch_4pad</x:v>
       </x:c>
       <x:c r="D41" s="7" t="str">
-        <x:v>C3257154</x:v>
+        <x:v>C273527</x:v>
       </x:c>
       <x:c r="E41" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F41" s="9" t="n">
-        <x:v>15.93</x:v>
+        <x:v>0.2657</x:v>
       </x:c>
       <x:c r="G41" s="9" t="n">
         <x:f>IF(ISNUMBER(F41),E41*F41,"")</x:f>
-        <x:v>15.93</x:v>
+        <x:v>1.0628</x:v>
       </x:c>
       <x:c r="H41" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C3257154.html</x:v>
-      </x:c>
-      <x:c r="I41" s="7" t="str">
-        <x:v>https://automation.honeywell.com/content/dam/honeywell-edam/sps/ast/en-us/campaigns/pressure-sensors/documents/sps-siot-mpr-series-datasheet-32332628-ciid-172626.pdf</x:v>
-      </x:c>
+        <x:v>https://jlcpcb.com/partdetail/component/C273527</x:v>
+      </x:c>
+      <x:c r="I41" s="7"/>
       <x:c r="J41" s="7" t="str">
-        <x:v>MPRLS0025PA00001A</x:v>
+        <x:v>TL3301NF160QG/P010515</x:v>
       </x:c>
       <x:c r="K41" s="7" t="str">
-        <x:v>Honeywell</x:v>
+        <x:v>E-Switch</x:v>
       </x:c>
       <x:c r="L41" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M41" s="7"/>
-    </x:row>
-    <x:row r="42" ht="53" customHeight="1">
+      <x:c r="N41" s="31"/>
+      <x:c r="O41" s="32"/>
+      <x:c r="P41" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q41" s="32" t="n">
+        <x:v>467</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="72" customHeight="1">
       <x:c r="A42" s="7" t="str">
-        <x:v>PCA9685PW,118</x:v>
+        <x:v>TPS563203DRLR</x:v>
       </x:c>
       <x:c r="B42" s="7" t="str">
-        <x:v>U7</x:v>
+        <x:v>U1, U2, U3</x:v>
       </x:c>
       <x:c r="C42" s="7" t="str">
-        <x:v>RheoBoard:PCA9685</x:v>
+        <x:v>RheoBoard:TPS563203DRLR</x:v>
       </x:c>
       <x:c r="D42" s="7" t="str">
-        <x:v>C2678753</x:v>
+        <x:v>C22445512</x:v>
       </x:c>
       <x:c r="E42" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F42" s="9" t="n">
-        <x:v>3.445</x:v>
+        <x:v>0.1197</x:v>
       </x:c>
       <x:c r="G42" s="9" t="n">
         <x:f>IF(ISNUMBER(F42),E42*F42,"")</x:f>
-        <x:v>3.445</x:v>
+        <x:v>0.3591</x:v>
       </x:c>
       <x:c r="H42" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C2678753.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C22445512</x:v>
       </x:c>
       <x:c r="I42" s="7" t="str">
-        <x:v>https://www.nxp.com/docs/en/data-sheet/PCA9685.pdf</x:v>
+        <x:v>https://www.ti.com/lit/gpn/tps563203</x:v>
       </x:c>
       <x:c r="J42" s="7" t="str">
-        <x:v>PCA9685PW,118</x:v>
+        <x:v>TPS563203DRLR</x:v>
       </x:c>
       <x:c r="K42" s="7" t="str">
-        <x:v>NXP</x:v>
+        <x:v>TI</x:v>
       </x:c>
       <x:c r="L42" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M42" s="7" t="str">
-        <x:v>Pumps LED0/1, indicators LED2–4, valves LED5/6 using FULL ON/OFF. TCA9534 removed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="53" customHeight="1">
+      <x:c r="M42" s="7"/>
+      <x:c r="N42" s="31"/>
+      <x:c r="O42" s="32"/>
+      <x:c r="P42" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q42" s="32" t="n">
+        <x:v>14064</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="72" customHeight="1">
       <x:c r="A43" s="11" t="str">
-        <x:v>ZR370-02PM / 4.5V / 2.5 LPM / ~500 mA</x:v>
+        <x:v>MPRLS0025PA00001A</x:v>
       </x:c>
       <x:c r="B43" s="11" t="str">
-        <x:v>U8, U11</x:v>
+        <x:v>U5</x:v>
       </x:c>
       <x:c r="C43" s="11" t="str">
-        <x:v>RheoBoard:PUMP</x:v>
-      </x:c>
-      <x:c r="D43" s="11"/>
+        <x:v>RheoBoard:MPRLS0025PA00001A</x:v>
+      </x:c>
+      <x:c r="D43" s="11" t="str">
+        <x:v>C3257154</x:v>
+      </x:c>
       <x:c r="E43" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F43" s="13" t="n">
-        <x:v>7.16</x:v>
+        <x:v>10.4036</x:v>
       </x:c>
       <x:c r="G43" s="13" t="n">
         <x:f>IF(ISNUMBER(F43),E43*F43,"")</x:f>
+        <x:v>10.4036</x:v>
+      </x:c>
+      <x:c r="H43" s="11" t="str">
+        <x:v>https://jlcpcb.com/partdetail/component/C3257154</x:v>
+      </x:c>
+      <x:c r="I43" s="11" t="str">
+        <x:v>https://automation.honeywell.com/content/dam/honeywell-edam/sps/ast/en-us/campaigns/pressure-sensors/documents/sps-siot-mpr-series-datasheet-32332628-ciid-172626.pdf</x:v>
+      </x:c>
+      <x:c r="J43" s="11" t="str">
+        <x:v>MPRLS0025PA00001A</x:v>
+      </x:c>
+      <x:c r="K43" s="11" t="str">
+        <x:v>Honeywell</x:v>
+      </x:c>
+      <x:c r="L43" s="11" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M43" s="11"/>
+      <x:c r="N43" s="31"/>
+      <x:c r="O43" s="32"/>
+      <x:c r="P43" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q43" s="32" t="n">
+        <x:v>497</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="72" customHeight="1">
+      <x:c r="A44" s="11" t="str">
+        <x:v>PCA9685PW,118</x:v>
+      </x:c>
+      <x:c r="B44" s="11" t="str">
+        <x:v>U7</x:v>
+      </x:c>
+      <x:c r="C44" s="11" t="str">
+        <x:v>RheoBoard:PCA9685</x:v>
+      </x:c>
+      <x:c r="D44" s="11" t="str">
+        <x:v>C2678753</x:v>
+      </x:c>
+      <x:c r="E44" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F44" s="10" t="n">
+        <x:v>3.3359</x:v>
+      </x:c>
+      <x:c r="G44" s="13" t="n">
+        <x:f>IF(ISNUMBER(F44),E44*F44,"")</x:f>
+        <x:v>3.3359</x:v>
+      </x:c>
+      <x:c r="H44" s="11" t="str">
+        <x:v>https://jlcpcb.com/partdetail/component/C2678753</x:v>
+      </x:c>
+      <x:c r="I44" s="11" t="str">
+        <x:v>https://www.nxp.com/docs/en/data-sheet/PCA9685.pdf</x:v>
+      </x:c>
+      <x:c r="J44" s="11" t="str">
+        <x:v>PCA9685PW,118</x:v>
+      </x:c>
+      <x:c r="K44" s="11" t="str">
+        <x:v>NXP</x:v>
+      </x:c>
+      <x:c r="L44" s="11" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M44" s="11" t="str">
+        <x:v>Pumps LED0/1, indicators LED2–4, valves LED5/6 using FULL ON/OFF. TCA9534 removed.</x:v>
+      </x:c>
+      <x:c r="N44" s="31"/>
+      <x:c r="O44" s="32"/>
+      <x:c r="P44" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q44" s="32" t="n">
+        <x:v>4871</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="72" customHeight="1">
+      <x:c r="A45" s="7" t="str">
+        <x:v>ZR370-02PM / 4.5V / 2.5 LPM / ~500 mA</x:v>
+      </x:c>
+      <x:c r="B45" s="7" t="str">
+        <x:v>U8, U11</x:v>
+      </x:c>
+      <x:c r="C45" s="7" t="str">
+        <x:v>RheoBoard:PUMP</x:v>
+      </x:c>
+      <x:c r="D45" s="7"/>
+      <x:c r="E45" s="8" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F45" s="10" t="n">
+        <x:f>'Parts cost'!G21/'Parts cost'!E21</x:f>
+        <x:v>7.16</x:v>
+      </x:c>
+      <x:c r="G45" s="9" t="n">
+        <x:f>IF(ISNUMBER(F45),E45*F45,"")</x:f>
         <x:v>14.32</x:v>
       </x:c>
-      <x:c r="H43" s="11" t="str">
+      <x:c r="H45" s="7" t="str">
         <x:v>https://www.adafruit.com/product/4699</x:v>
       </x:c>
-      <x:c r="I43" s="11"/>
-      <x:c r="J43" s="11" t="str">
+      <x:c r="I45" s="7"/>
+      <x:c r="J45" s="7" t="str">
         <x:v>ZR370-02PM</x:v>
       </x:c>
-      <x:c r="K43" s="11" t="str">
+      <x:c r="K45" s="7" t="str">
         <x:v>Supplier-specified</x:v>
       </x:c>
-      <x:c r="L43" s="11" t="str">
+      <x:c r="L45" s="7" t="str">
         <x:v>Manual pump fitting</x:v>
       </x:c>
-      <x:c r="M43" s="11" t="str">
+      <x:c r="M45" s="7" t="str">
         <x:v>Existing pump retained for intermittent use. Manual fitting; provide mechanical support.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="44" ht="53" customHeight="1">
-      <x:c r="A44" s="11" t="str">
+      <x:c r="N45" s="31"/>
+      <x:c r="O45" s="32"/>
+      <x:c r="P45" s="32"/>
+      <x:c r="Q45" s="32"/>
+    </x:row>
+    <x:row r="46" ht="72" customHeight="1">
+      <x:c r="A46" s="7" t="str">
         <x:v>JST XH 2-pin 2.50mm</x:v>
       </x:c>
-      <x:c r="B44" s="11" t="str">
+      <x:c r="B46" s="7" t="str">
         <x:v>U9, U10</x:v>
       </x:c>
-      <x:c r="C44" s="11" t="str">
+      <x:c r="C46" s="7" t="str">
         <x:v>RheoBoard:VALVE_v105</x:v>
       </x:c>
-      <x:c r="D44" s="11" t="str">
+      <x:c r="D46" s="7" t="str">
         <x:v>C158012</x:v>
       </x:c>
-      <x:c r="E44" s="12" t="n">
+      <x:c r="E46" s="8" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F44" s="10"/>
-      <x:c r="G44" s="13" t="str">
-        <x:f>IF(ISNUMBER(F44),E44*F44,"")</x:f>
-      </x:c>
-      <x:c r="H44" s="11" t="str">
+      <x:c r="F46" s="10" t="n">
+        <x:f>'Parts cost'!G22/'Parts cost'!E22</x:f>
+        <x:v>0.041</x:v>
+      </x:c>
+      <x:c r="G46" s="9" t="n">
+        <x:f>IF(ISNUMBER(F46),E46*F46,"")</x:f>
+        <x:v>0.082</x:v>
+      </x:c>
+      <x:c r="H46" s="7" t="str">
         <x:v>https://www.lcsc.com/product-detail/C158012.html</x:v>
       </x:c>
-      <x:c r="I44" s="11" t="str">
+      <x:c r="I46" s="7" t="str">
         <x:v>https://www.jst-mfg.com/product/pdf/eng/eXH.pdf</x:v>
       </x:c>
-      <x:c r="J44" s="11" t="str">
+      <x:c r="J46" s="7" t="str">
         <x:v>B2B-XH-A(LF)(SN)</x:v>
       </x:c>
-      <x:c r="K44" s="11" t="str">
+      <x:c r="K46" s="7" t="str">
         <x:v>JST</x:v>
       </x:c>
-      <x:c r="L44" s="11" t="str">
+      <x:c r="L46" s="7" t="str">
         <x:v>Manual THT</x:v>
       </x:c>
-      <x:c r="M44" s="11" t="str">
+      <x:c r="M46" s="7" t="str">
         <x:v>Fitted JST XH header only. External valve is listed on Manual accessories. Manual through-hole assembly.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="45" ht="53" customHeight="1">
-      <x:c r="A45" s="7" t="str">
+      <x:c r="N46" s="31"/>
+      <x:c r="O46" s="32"/>
+      <x:c r="P46" s="32"/>
+      <x:c r="Q46" s="32"/>
+    </x:row>
+    <x:row r="47" ht="72" customHeight="1">
+      <x:c r="A47" s="7" t="str">
         <x:v>TPS259472ARPWR</x:v>
       </x:c>
-      <x:c r="B45" s="7" t="str">
+      <x:c r="B47" s="7" t="str">
         <x:v>U12</x:v>
       </x:c>
-      <x:c r="C45" s="7" t="str">
+      <x:c r="C47" s="7" t="str">
         <x:v>RheoBoard:TI_RPW0010A_VQFN-HR_2x2mm</x:v>
       </x:c>
-      <x:c r="D45" s="7" t="str">
+      <x:c r="D47" s="7" t="str">
         <x:v>C3662789</x:v>
-      </x:c>
-      <x:c r="E45" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F45" s="10"/>
-      <x:c r="G45" s="9" t="str">
-        <x:f>IF(ISNUMBER(F45),E45*F45,"")</x:f>
-      </x:c>
-      <x:c r="H45" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C3662789.html</x:v>
-      </x:c>
-      <x:c r="I45" s="7" t="str">
-        <x:v>https://www.ti.com/lit/ds/symlink/tps25947.pdf</x:v>
-      </x:c>
-      <x:c r="J45" s="7" t="str">
-        <x:v>TPS259472ARPWR</x:v>
-      </x:c>
-      <x:c r="K45" s="7" t="str">
-        <x:v>Texas Instruments</x:v>
-      </x:c>
-      <x:c r="L45" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M45" s="7" t="str">
-        <x:v>New auto-retry input eFuse; TI RPW0010A HotRod footprint, approximately 2 A limit / 13.8 V clamp.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="112" customHeight="1">
-      <x:c r="A46" s="7" t="str">
-        <x:v>TCA9517ADGKR</x:v>
-      </x:c>
-      <x:c r="B46" s="7" t="str">
-        <x:v>U13</x:v>
-      </x:c>
-      <x:c r="C46" s="7" t="str">
-        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
-      </x:c>
-      <x:c r="D46" s="7" t="str">
-        <x:v>C201698</x:v>
-      </x:c>
-      <x:c r="E46" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F46" s="10"/>
-      <x:c r="G46" s="9" t="str">
-        <x:f>IF(ISNUMBER(F46),E46*F46,"")</x:f>
-      </x:c>
-      <x:c r="H46" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C201698.html</x:v>
-      </x:c>
-      <x:c r="I46" s="7" t="str">
-        <x:v>https://www.ti.com/lit/ds/symlink/tca9517a.pdf</x:v>
-      </x:c>
-      <x:c r="J46" s="7" t="str">
-        <x:v>TCA9517ADGKR</x:v>
-      </x:c>
-      <x:c r="K46" s="7" t="str">
-        <x:v>Texas Instruments</x:v>
-      </x:c>
-      <x:c r="L46" s="7" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="M46" s="7" t="str">
-        <x:v>Qwiic master interface: local bus on A, host on B. EN and VCCB use HOST_3V3; separate supplies, common GND. TI DGK land pattern: 1.4 x 0.45 mm pads, 0.65 mm pitch, 4.4 mm row-center span.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="83" customHeight="1">
-      <x:c r="A47" s="7" t="str">
-        <x:v>BZT52C10-7-F</x:v>
-      </x:c>
-      <x:c r="B47" s="7" t="str">
-        <x:v>D37</x:v>
-      </x:c>
-      <x:c r="C47" s="7" t="str">
-        <x:v>Diode_SMD:D_SOD-123</x:v>
-      </x:c>
-      <x:c r="D47" s="7" t="str">
-        <x:v>C155227</x:v>
       </x:c>
       <x:c r="E47" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F47" s="10"/>
-      <x:c r="G47" s="9" t="str">
+      <x:c r="F47" s="10" t="n">
+        <x:v>1.0754</x:v>
+      </x:c>
+      <x:c r="G47" s="9" t="n">
         <x:f>IF(ISNUMBER(F47),E47*F47,"")</x:f>
+        <x:v>1.0754</x:v>
       </x:c>
       <x:c r="H47" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C155227.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C3662789</x:v>
       </x:c>
       <x:c r="I47" s="7" t="str">
-        <x:v>https://www.diodes.com/datasheet/download/BZT52Cxx.pdf</x:v>
+        <x:v>https://www.ti.com/lit/ds/symlink/tps25947.pdf</x:v>
       </x:c>
       <x:c r="J47" s="7" t="str">
-        <x:v>BZT52C10-7-F</x:v>
+        <x:v>TPS259472ARPWR</x:v>
       </x:c>
       <x:c r="K47" s="7" t="str">
-        <x:v>Diodes Incorporated</x:v>
+        <x:v>Texas Instruments</x:v>
       </x:c>
       <x:c r="L47" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M47" s="7" t="str">
-        <x:v>Q11 gate-source clamp. Cathode to VIN_RAW/source; anode to gate.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="53" customHeight="1">
+        <x:v>New auto-retry input eFuse; TI RPW0010A HotRod footprint, approximately 2 A limit / 13.8 V clamp.</x:v>
+      </x:c>
+      <x:c r="N47" s="31"/>
+      <x:c r="O47" s="32"/>
+      <x:c r="P47" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q47" s="32" t="n">
+        <x:v>1856</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="72" customHeight="1">
       <x:c r="A48" s="11" t="str">
-        <x:v>Button GPIO 1x05 2.54mm</x:v>
+        <x:v>TCA9517ADGKR</x:v>
       </x:c>
       <x:c r="B48" s="11" t="str">
-        <x:v>J19</x:v>
+        <x:v>U13</x:v>
       </x:c>
       <x:c r="C48" s="11" t="str">
-        <x:v>Connector_PinHeader_2.54mm:PinHeader_1x05_P2.54mm_Vertical</x:v>
-      </x:c>
-      <x:c r="D48" s="11"/>
+        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
+      </x:c>
+      <x:c r="D48" s="11" t="str">
+        <x:v>C201698</x:v>
+      </x:c>
       <x:c r="E48" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F48" s="20"/>
-      <x:c r="G48" s="13" t="str">
+      <x:c r="F48" s="10" t="n">
+        <x:v>0.4878</x:v>
+      </x:c>
+      <x:c r="G48" s="13" t="n">
         <x:f>IF(ISNUMBER(F48),E48*F48,"")</x:f>
+        <x:v>0.4878</x:v>
       </x:c>
       <x:c r="H48" s="11" t="str">
-        <x:v>https://www.adafruit.com/product/392</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C201698</x:v>
       </x:c>
       <x:c r="I48" s="11" t="str">
-        <x:v>https://www.adafruit.com/product/392</x:v>
+        <x:v>https://www.ti.com/lit/ds/symlink/tca9517a.pdf</x:v>
       </x:c>
       <x:c r="J48" s="11" t="str">
-        <x:v>392, cut to 5 positions</x:v>
+        <x:v>TCA9517ADGKR</x:v>
       </x:c>
       <x:c r="K48" s="11" t="str">
-        <x:v>Adafruit Industries LLC</x:v>
+        <x:v>Texas Instruments</x:v>
       </x:c>
       <x:c r="L48" s="11" t="str">
-        <x:v>Manual</x:v>
+        <x:v>SMT</x:v>
       </x:c>
       <x:c r="M48" s="11" t="str">
-        <x:v>Cut one 5-position segment from a 36-pin strip. Pin 1 GND, 2 VALVE1_IN, 3 VALVE2_IN, 4 PUMP1_IN, 5 PUMP2_IN. Manual assembly; host power through J9.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="53" customHeight="1">
+        <x:v>Qwiic master interface: local bus on A, host on B. EN and VCCB use HOST_3V3; separate supplies, common GND. TI DGK land pattern: 1.4 x 0.45 mm pads, 0.65 mm pitch, 4.4 mm row-center span.</x:v>
+      </x:c>
+      <x:c r="N48" s="31"/>
+      <x:c r="O48" s="32"/>
+      <x:c r="P48" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q48" s="32" t="n">
+        <x:v>17568</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="72" customHeight="1">
       <x:c r="A49" s="7" t="str">
-        <x:v>AO3400A</x:v>
+        <x:v>BZT52C10-7-F</x:v>
       </x:c>
       <x:c r="B49" s="7" t="str">
-        <x:v>Q3</x:v>
+        <x:v>D37</x:v>
       </x:c>
       <x:c r="C49" s="7" t="str">
-        <x:v>RheoBoard:AO3400A_Pin1Offset</x:v>
+        <x:v>Diode_SMD:D_SOD-123</x:v>
       </x:c>
       <x:c r="D49" s="7" t="str">
-        <x:v>C20917</x:v>
+        <x:v>C155227</x:v>
       </x:c>
       <x:c r="E49" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F49" s="9" t="n">
-        <x:v>0.322</x:v>
+        <x:v>0.0542</x:v>
       </x:c>
       <x:c r="G49" s="9" t="n">
         <x:f>IF(ISNUMBER(F49),E49*F49,"")</x:f>
-        <x:v>0.322</x:v>
+        <x:v>0.0542</x:v>
       </x:c>
       <x:c r="H49" s="7" t="str">
-        <x:v>https://www.lcsc.com/product-detail/C20917.html</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C155227</x:v>
       </x:c>
       <x:c r="I49" s="7" t="str">
-        <x:v>https://www.aosmd.com/sites/default/files/res/data_sheets/AO3400A.pdf</x:v>
+        <x:v>https://www.diodes.com/datasheet/download/BZT52Cxx.pdf</x:v>
       </x:c>
       <x:c r="J49" s="7" t="str">
-        <x:v>AO3400A</x:v>
+        <x:v>BZT52C10-7-F</x:v>
       </x:c>
       <x:c r="K49" s="7" t="str">
-        <x:v>AOS</x:v>
+        <x:v>Diodes Incorporated</x:v>
       </x:c>
       <x:c r="L49" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M49" s="7"/>
-    </x:row>
-    <x:row r="50" ht="30" customHeight="1">
-      <x:c r="A50" s="14" t="str">
-        <x:v>Total fitted parts / incomplete priced subtotal</x:v>
-      </x:c>
-      <x:c r="B50" s="14"/>
-      <x:c r="C50" s="14"/>
-      <x:c r="D50" s="14"/>
-      <x:c r="E50" s="14" t="n">
-        <x:f>SUM(E2:E49)</x:f>
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="F50" s="14" t="str">
-        <x:v>Incomplete estimate</x:v>
-      </x:c>
-      <x:c r="G50" s="15" t="n">
-        <x:f>SUM(G2:G49)</x:f>
-        <x:v>52.888000000000005</x:v>
-      </x:c>
-      <x:c r="H50"/>
-      <x:c r="I50"/>
-      <x:c r="J50"/>
-      <x:c r="K50"/>
-      <x:c r="L50"/>
-      <x:c r="M50"/>
-    </x:row>
-    <x:row r="51" ht="30" customHeight="1">
-      <x:c r="A51"/>
-      <x:c r="B51"/>
-      <x:c r="C51"/>
-      <x:c r="D51"/>
-      <x:c r="E51"/>
-      <x:c r="F51"/>
-      <x:c r="G51"/>
-      <x:c r="H51"/>
-      <x:c r="I51"/>
-      <x:c r="J51"/>
-      <x:c r="K51"/>
-      <x:c r="L51"/>
-      <x:c r="M51"/>
-    </x:row>
-    <x:row r="52" ht="36" customHeight="1">
+      <x:c r="M49" s="7" t="str">
+        <x:v>Q11 gate-source clamp. Cathode to VIN_RAW/source; anode to gate.</x:v>
+      </x:c>
+      <x:c r="N49" s="31"/>
+      <x:c r="O49" s="32"/>
+      <x:c r="P49" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q49" s="32" t="n">
+        <x:v>138717</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="72" customHeight="1">
+      <x:c r="A50" s="4" t="str">
+        <x:v>Button GPIO 1x05 2.54mm</x:v>
+      </x:c>
+      <x:c r="B50" s="4" t="str">
+        <x:v>J19</x:v>
+      </x:c>
+      <x:c r="C50" s="4" t="str">
+        <x:v>Connector_PinHeader_2.54mm:PinHeader_1x05_P2.54mm_Vertical</x:v>
+      </x:c>
+      <x:c r="D50" s="4" t="str">
+        <x:v>C124379</x:v>
+      </x:c>
+      <x:c r="E50" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F50" s="35" t="n">
+        <x:f>'Parts cost'!G20/'Parts cost'!E20</x:f>
+        <x:v>0.0561</x:v>
+      </x:c>
+      <x:c r="G50" s="35" t="n">
+        <x:f>IF(ISNUMBER(F50),E50*F50,"")</x:f>
+        <x:v>0.0561</x:v>
+      </x:c>
+      <x:c r="H50" s="33" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C124379.html</x:v>
+      </x:c>
+      <x:c r="I50" s="33" t="str">
+        <x:v>https://datasheet.lcsc.com/datasheet/pdf/219f7e7eb5f34457895b2c164313179f.pdf?productCode=C124379</x:v>
+      </x:c>
+      <x:c r="J50" s="33" t="str">
+        <x:v>B-2100S05P-A110</x:v>
+      </x:c>
+      <x:c r="K50" s="33" t="str">
+        <x:v>Ckmtw</x:v>
+      </x:c>
+      <x:c r="L50" s="33" t="str">
+        <x:v>Manual</x:v>
+      </x:c>
+      <x:c r="M50" s="33" t="str">
+        <x:v>Ready-made 5-pin vertical male header; manual through-hole assembly. 2.54 mm pitch, 0.60 ±0.02 mm square pins, 3 mm tails, 6 mm mating pins. Fits current J19 1.0 mm drills; footprint and pinout unchanged. Pin 1 GND, 2 VALVE1_IN, 3 VALVE2_IN, 4 PUMP1_IN, 5 PUMP2_IN.</x:v>
+      </x:c>
+      <x:c r="N50" s="31"/>
+      <x:c r="O50" s="32"/>
+      <x:c r="P50" s="32"/>
+      <x:c r="Q50" s="32" t="n">
+        <x:v>18170</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="72" customHeight="1">
+      <x:c r="A51" s="33" t="str">
+        <x:v>AO3400A</x:v>
+      </x:c>
+      <x:c r="B51" s="33" t="str">
+        <x:v>Q3</x:v>
+      </x:c>
+      <x:c r="C51" s="33" t="str">
+        <x:v>RheoBoard:AO3400A_Pin1Offset</x:v>
+      </x:c>
+      <x:c r="D51" s="33" t="str">
+        <x:v>C20917</x:v>
+      </x:c>
+      <x:c r="E51" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F51" s="36" t="n">
+        <x:v>0.0889</x:v>
+      </x:c>
+      <x:c r="G51" s="36" t="n">
+        <x:f>IF(ISNUMBER(F51),E51*F51,"")</x:f>
+        <x:v>0.0889</x:v>
+      </x:c>
+      <x:c r="H51" s="33" t="str">
+        <x:v>https://jlcpcb.com/partdetail/component/C20917</x:v>
+      </x:c>
+      <x:c r="I51" s="33" t="str">
+        <x:v>https://www.aosmd.com/sites/default/files/res/data_sheets/AO3400A.pdf</x:v>
+      </x:c>
+      <x:c r="J51" s="33" t="str">
+        <x:v>AO3400A</x:v>
+      </x:c>
+      <x:c r="K51" s="33" t="str">
+        <x:v>AOS</x:v>
+      </x:c>
+      <x:c r="L51" s="33" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M51" s="33"/>
+      <x:c r="N51" s="31"/>
+      <x:c r="O51" s="32"/>
+      <x:c r="P51" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q51" s="32" t="n">
+        <x:v>994885</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" s="16" t="str">
-        <x:v>Prices are retained from the original workbook only where the selected part is unchanged. New parts have blank prices. This subtotal is incomplete and is not a JLCPCB quotation; obtain a fresh quote for v1.05.</x:v>
+        <x:v>Total fitted parts / cost (valves extra)</x:v>
       </x:c>
       <x:c r="B52" s="16"/>
       <x:c r="C52" s="16"/>
       <x:c r="D52" s="16"/>
-      <x:c r="E52" s="16"/>
-      <x:c r="F52" s="16"/>
-      <x:c r="G52" s="16"/>
+      <x:c r="E52" s="16" t="n">
+        <x:f>SUM(E2:E51)</x:f>
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="F52" s="37"/>
+      <x:c r="G52" s="37" t="n">
+        <x:f>SUM(G2:G51)</x:f>
+        <x:v>39.1486</x:v>
+      </x:c>
       <x:c r="H52" s="16"/>
       <x:c r="I52" s="16"/>
       <x:c r="J52" s="16"/>
       <x:c r="K52" s="16"/>
       <x:c r="L52" s="16"/>
       <x:c r="M52" s="16"/>
-    </x:row>
-    <x:row r="53" ht="34" customHeight="1">
-      <x:c r="A53"/>
-      <x:c r="B53"/>
-      <x:c r="C53"/>
-      <x:c r="D53"/>
-      <x:c r="E53"/>
+      <x:c r="N52" s="26"/>
+      <x:c r="O52" s="27"/>
+    </x:row>
+    <x:row r="53" ht="48" customHeight="1">
+      <x:c r="A53" s="16" t="str">
+        <x:v>Fitted parts for 5 boards (valves extra)</x:v>
+      </x:c>
+      <x:c r="B53" s="16"/>
+      <x:c r="C53" s="16"/>
+      <x:c r="D53" s="16"/>
+      <x:c r="E53" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="F53"/>
-      <x:c r="G53"/>
+      <x:c r="G53" s="28" t="n">
+        <x:f>G52*E53</x:f>
+        <x:v>195.743</x:v>
+      </x:c>
       <x:c r="H53"/>
       <x:c r="I53"/>
       <x:c r="J53"/>
       <x:c r="K53"/>
       <x:c r="L53"/>
       <x:c r="M53"/>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54"/>
-      <x:c r="B54"/>
-      <x:c r="C54"/>
-      <x:c r="D54"/>
-      <x:c r="E54"/>
-      <x:c r="F54"/>
-      <x:c r="G54"/>
-      <x:c r="H54"/>
-      <x:c r="I54"/>
-      <x:c r="J54"/>
-      <x:c r="K54"/>
-      <x:c r="L54"/>
-      <x:c r="M54"/>
+      <x:c r="N53" s="26"/>
+      <x:c r="O53" s="27"/>
+    </x:row>
+    <x:row r="54" ht="40" customHeight="1">
+      <x:c r="A54" s="16" t="str">
+        <x:v>See Parts cost for the FULL board parts total: fitted parts plus external valves, and minimum-pack purchase budget. Prices checked 2026-10-27. Excludes PCB, assembly, SMT attrition, shipping, tax and system accessories.</x:v>
+      </x:c>
+      <x:c r="B54" s="16"/>
+      <x:c r="C54" s="16"/>
+      <x:c r="D54" s="16"/>
+      <x:c r="E54" s="16"/>
+      <x:c r="F54" s="16"/>
+      <x:c r="G54" s="16"/>
+      <x:c r="H54" s="16"/>
+      <x:c r="I54" s="16"/>
+      <x:c r="J54" s="16"/>
+      <x:c r="K54" s="16"/>
+      <x:c r="L54" s="16"/>
+      <x:c r="M54" s="16"/>
+      <x:c r="N54" s="26"/>
+      <x:c r="O54" s="27"/>
+      <x:c r="P54" s="16"/>
+      <x:c r="Q54" s="16"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A52:M52"/>
+    <x:mergeCell ref="A54:Q54"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f11a450511c4742"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05cc8c22dba84215"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2493,7 +3240,7 @@
         <x:v>https://www.adafruit.com/product/4663</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>Existing specified valve retained. JST XH mating cable; verify supplied cable polarity. Header parts appear on main BOM separately.</x:v>
+        <x:v>Included in Parts cost, two per board. JST XH mating cable supplied; verify cable polarity. U9/U10 header parts counted separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="154" customHeight="1">
@@ -2623,7 +3370,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red1f681413f44669"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R377052dac96a4745"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2636,6 +3383,7 @@
     <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="70" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2651,6 +3399,7 @@
       <x:c r="D1" s="18" t="str">
         <x:v>LCSC Part #</x:v>
       </x:c>
+      <x:c r="E1" s="23"/>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="3" t="str">
@@ -2665,6 +3414,7 @@
       <x:c r="D2" s="3" t="str">
         <x:v>C5448891</x:v>
       </x:c>
+      <x:c r="E2" s="24"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="3" t="str">
@@ -2679,6 +3429,7 @@
       <x:c r="D3" s="3" t="str">
         <x:v>C14663</x:v>
       </x:c>
+      <x:c r="E3" s="24"/>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="3" t="str">
@@ -2693,6 +3444,7 @@
       <x:c r="D4" s="3" t="str">
         <x:v>C5360811</x:v>
       </x:c>
+      <x:c r="E4" s="24"/>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="3" t="str">
@@ -2707,6 +3459,7 @@
       <x:c r="D5" s="3" t="str">
         <x:v>C7393892</x:v>
       </x:c>
+      <x:c r="E5" s="24"/>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="3" t="str">
@@ -2721,6 +3474,7 @@
       <x:c r="D6" s="3" t="str">
         <x:v>C128458</x:v>
       </x:c>
+      <x:c r="E6" s="24"/>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="3" t="str">
@@ -2735,545 +3489,1213 @@
       <x:c r="D7" s="3" t="str">
         <x:v>C20416420</x:v>
       </x:c>
+      <x:c r="E7" s="24"/>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="3" t="str">
-        <x:v>18pF 50V C0G ±2%</x:v>
+        <x:v>18pF 50V C0G ±5%</x:v>
       </x:c>
       <x:c r="B8" s="3" t="str">
-        <x:v>C55, C58, C62</x:v>
+        <x:v>C55, C58</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D8" s="3" t="str">
-        <x:v>C2169079</x:v>
-      </x:c>
+        <x:v>C107040</x:v>
+      </x:c>
+      <x:c r="E8" s="24"/>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="3" t="str">
-        <x:v>3.3nF 50V X7R ±10%</x:v>
+        <x:v>24pF 50V C0G ±5%</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
-        <x:v>C64</x:v>
+        <x:v>C62</x:v>
       </x:c>
       <x:c r="C9" s="3" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D9" s="3" t="str">
-        <x:v>C107088</x:v>
-      </x:c>
+        <x:v>C107044</x:v>
+      </x:c>
+      <x:c r="E9" s="24"/>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="3" t="str">
-        <x:v>1uF 50V X7R ±10%</x:v>
+        <x:v>3.3nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>C65</x:v>
+        <x:v>C64</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
-        <x:v>Capacitor_SMD:C_0805_2012Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D10" s="3" t="str">
-        <x:v>C91185</x:v>
-      </x:c>
+        <x:v>C107088</x:v>
+      </x:c>
+      <x:c r="E10" s="24"/>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="3" t="str">
-        <x:v>100nF 50V X7R ±10%</x:v>
+        <x:v>1uF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
-        <x:v>C66</x:v>
+        <x:v>C65</x:v>
       </x:c>
       <x:c r="C11" s="3" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:C_0805_2012Metric</x:v>
       </x:c>
       <x:c r="D11" s="3" t="str">
-        <x:v>C14663</x:v>
-      </x:c>
+        <x:v>C91185</x:v>
+      </x:c>
+      <x:c r="E11" s="24"/>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="3" t="str">
-        <x:v>4.7uF 50V X7R ±10%</x:v>
+        <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
-        <x:v>C67</x:v>
+        <x:v>C66</x:v>
       </x:c>
       <x:c r="C12" s="3" t="str">
-        <x:v>Capacitor_SMD:C_1206_3216Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D12" s="3" t="str">
-        <x:v>C132170</x:v>
-      </x:c>
+        <x:v>C14663</x:v>
+      </x:c>
+      <x:c r="E12" s="24"/>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="3" t="str">
-        <x:v>DMP6023LE-13</x:v>
+        <x:v>4.7uF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B13" s="3" t="str">
-        <x:v>Q11</x:v>
+        <x:v>C67</x:v>
       </x:c>
       <x:c r="C13" s="3" t="str">
-        <x:v>RheoBoard:SOT-223-3_TabPin2_DFM</x:v>
+        <x:v>Capacitor_SMD:C_1206_3216Metric</x:v>
       </x:c>
       <x:c r="D13" s="3" t="str">
-        <x:v>C154901</x:v>
-      </x:c>
+        <x:v>C132170</x:v>
+      </x:c>
+      <x:c r="E13" s="24"/>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="3" t="str">
-        <x:v>LED_Red</x:v>
+        <x:v>DMP6023LE-13</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
-        <x:v>D6, D7, D8, D13, D14, D15, D17, D19</x:v>
-      </x:c>
-      <x:c r="C14" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RheoBoard:LED_SZYY0603R_A1_K2_HandSolder</x:t>
-        </x:is>
+        <x:v>Q11</x:v>
+      </x:c>
+      <x:c r="C14" s="3" t="str">
+        <x:v>RheoBoard:SOT-223-3_TabPin2_DFM</x:v>
       </x:c>
       <x:c r="D14" s="3" t="str">
-        <x:v>C434419</x:v>
-      </x:c>
+        <x:v>C154901</x:v>
+      </x:c>
+      <x:c r="E14" s="24"/>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="3" t="str">
-        <x:v>SS34</x:v>
+        <x:v>LED_Red</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
-        <x:v>D11, D12, D16, D18</x:v>
+        <x:v>D6, D7, D8, D13, D14, D15, D17, D19</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
-        <x:v>Diode_SMD:D_SMA</x:v>
+        <x:v>RheoBoard:LED_SZYY0603R_A1_K2_HandSolder</x:v>
       </x:c>
       <x:c r="D15" s="3" t="str">
-        <x:v>C115205</x:v>
-      </x:c>
+        <x:v>C434419</x:v>
+      </x:c>
+      <x:c r="E15" s="24"/>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="3" t="str">
-        <x:v>LED_Red</x:v>
+        <x:v>SS34</x:v>
       </x:c>
       <x:c r="B16" s="3" t="str">
-        <x:v>D33, D34, D35</x:v>
-      </x:c>
-      <x:c r="C16" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RheoBoard:LED_SZYY0603R_A1_K2_Nominal</x:t>
-        </x:is>
+        <x:v>D11, D12, D16, D18</x:v>
+      </x:c>
+      <x:c r="C16" s="3" t="str">
+        <x:v>Diode_SMD:D_SMA</x:v>
       </x:c>
       <x:c r="D16" s="3" t="str">
-        <x:v>C434419</x:v>
-      </x:c>
+        <x:v>C115205</x:v>
+      </x:c>
+      <x:c r="E16" s="24"/>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="3" t="str">
-        <x:v>SMBJ13A</x:v>
+        <x:v>LED_Red</x:v>
       </x:c>
       <x:c r="B17" s="3" t="str">
-        <x:v>D36</x:v>
+        <x:v>D33, D34, D35</x:v>
       </x:c>
       <x:c r="C17" s="3" t="str">
-        <x:v>Diode_SMD:D_SMB</x:v>
+        <x:v>RheoBoard:LED_SZYY0603R_A1_K2_Nominal</x:v>
       </x:c>
       <x:c r="D17" s="3" t="str">
-        <x:v>C151252</x:v>
-      </x:c>
+        <x:v>C434419</x:v>
+      </x:c>
+      <x:c r="E17" s="24"/>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="3" t="str">
-        <x:v>2A time-delay JFC1032-1200TS</x:v>
+        <x:v>SMBJ13A</x:v>
       </x:c>
       <x:c r="B18" s="3" t="str">
-        <x:v>F1</x:v>
+        <x:v>D36</x:v>
       </x:c>
       <x:c r="C18" s="3" t="str">
-        <x:v>RheoBoard:Fuse_JDT_JFC1032TS_10.25x3.2mm</x:v>
+        <x:v>Diode_SMD:D_SMB</x:v>
       </x:c>
       <x:c r="D18" s="3" t="str">
-        <x:v>C53035082</x:v>
-      </x:c>
+        <x:v>C151252</x:v>
+      </x:c>
+      <x:c r="E18" s="24"/>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" s="3" t="str">
-        <x:v>JST SH 4-pin 1.00mm</x:v>
+        <x:v>2A time-delay JFC1032-1200TS</x:v>
       </x:c>
       <x:c r="B19" s="3" t="str">
-        <x:v>J1, J9, J12, J17</x:v>
+        <x:v>F1</x:v>
       </x:c>
       <x:c r="C19" s="3" t="str">
-        <x:v>Connector_JST:JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</x:v>
+        <x:v>RheoBoard:Fuse_JDT_JFC1032TS_10.25x3.2mm</x:v>
       </x:c>
       <x:c r="D19" s="3" t="str">
-        <x:v>C160404</x:v>
-      </x:c>
+        <x:v>C53035082</x:v>
+      </x:c>
+      <x:c r="E19" s="24"/>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
       <x:c r="A20" s="3" t="str">
-        <x:v>4.7uH FXL0530-4R7-M</x:v>
+        <x:v>JST SH 4-pin 1.00mm</x:v>
       </x:c>
       <x:c r="B20" s="3" t="str">
-        <x:v>L1, L2, L5</x:v>
+        <x:v>J1, J9, J12, J17</x:v>
       </x:c>
       <x:c r="C20" s="3" t="str">
-        <x:v>Inductor_SMD:L_Changjiang_FXL0530</x:v>
+        <x:v>Connector_JST:JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</x:v>
       </x:c>
       <x:c r="D20" s="3" t="str">
-        <x:v>C177246</x:v>
-      </x:c>
+        <x:v>C160404</x:v>
+      </x:c>
+      <x:c r="E20" s="24"/>
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
       <x:c r="A21" s="3" t="str">
-        <x:v>AO3400A</x:v>
+        <x:v>4.7uH FXL0530-4R7-M</x:v>
       </x:c>
       <x:c r="B21" s="3" t="str">
-        <x:v>Q4, Q8, Q10</x:v>
+        <x:v>L1, L2, L5</x:v>
       </x:c>
       <x:c r="C21" s="3" t="str">
-        <x:v>RheoBoard:AO3400A</x:v>
+        <x:v>Inductor_SMD:L_Changjiang_FXL0530</x:v>
       </x:c>
       <x:c r="D21" s="3" t="str">
-        <x:v>C20917</x:v>
-      </x:c>
+        <x:v>C177246</x:v>
+      </x:c>
+      <x:c r="E21" s="24"/>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" s="3" t="str">
-        <x:v>100K/0603/1%</x:v>
+        <x:v>AO3400A</x:v>
       </x:c>
       <x:c r="B22" s="3" t="str">
-        <x:v>R1, R4, R7</x:v>
+        <x:v>Q4, Q8, Q10</x:v>
       </x:c>
       <x:c r="C22" s="3" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
+        <x:v>RheoBoard:AO3400A</x:v>
       </x:c>
       <x:c r="D22" s="3" t="str">
-        <x:v>C25803</x:v>
-      </x:c>
+        <x:v>C20917</x:v>
+      </x:c>
+      <x:c r="E22" s="24"/>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
       <x:c r="A23" s="3" t="str">
-        <x:v>4K7/0603/1%</x:v>
+        <x:v>100K/0603/1%</x:v>
       </x:c>
       <x:c r="B23" s="3" t="str">
-        <x:v>R15, R20, R82, R83</x:v>
+        <x:v>R1, R4, R7</x:v>
       </x:c>
       <x:c r="C23" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D23" s="3" t="str">
-        <x:v>C23162</x:v>
-      </x:c>
+        <x:v>C25803</x:v>
+      </x:c>
+      <x:c r="E23" s="24"/>
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
       <x:c r="A24" s="3" t="str">
-        <x:v>10K/0603/1%</x:v>
+        <x:v>4K7/0603/1%</x:v>
       </x:c>
       <x:c r="B24" s="3" t="str">
-        <x:v>R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84, R85</x:v>
+        <x:v>R15, R20, R82, R83</x:v>
       </x:c>
       <x:c r="C24" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D24" s="3" t="str">
-        <x:v>C25804</x:v>
-      </x:c>
+        <x:v>C23162</x:v>
+      </x:c>
+      <x:c r="E24" s="24"/>
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
       <x:c r="A25" s="3" t="str">
-        <x:v>1k/0603/1%</x:v>
+        <x:v>10K/0603/1%</x:v>
       </x:c>
       <x:c r="B25" s="3" t="str">
-        <x:v>R24, R25, R26, R39, R40, R54, R59, R75</x:v>
+        <x:v>R16, R17, R18, R19, R22, R23, R29, R30, R31, R32, R33, R34, R37, R38, R51, R56, R84, R85</x:v>
       </x:c>
       <x:c r="C25" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D25" s="3" t="str">
-        <x:v>C21190</x:v>
-      </x:c>
+        <x:v>C25804</x:v>
+      </x:c>
+      <x:c r="E25" s="24"/>
     </x:row>
     <x:row r="26" ht="48" customHeight="1">
       <x:c r="A26" s="3" t="str">
-        <x:v>100R/0603/1%</x:v>
+        <x:v>1k/0603/1%</x:v>
       </x:c>
       <x:c r="B26" s="3" t="str">
-        <x:v>R35, R36, R42, R55</x:v>
+        <x:v>R24, R25, R26, R39, R40, R54, R59, R75</x:v>
       </x:c>
       <x:c r="C26" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D26" s="3" t="str">
-        <x:v>C22775</x:v>
-      </x:c>
+        <x:v>C21190</x:v>
+      </x:c>
+      <x:c r="E26" s="24"/>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
       <x:c r="A27" s="3" t="str">
-        <x:v>330/0603/1%</x:v>
+        <x:v>100R/0603/1%</x:v>
       </x:c>
       <x:c r="B27" s="3" t="str">
-        <x:v>R44, R77</x:v>
+        <x:v>R35, R36, R42, R55</x:v>
       </x:c>
       <x:c r="C27" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D27" s="3" t="str">
-        <x:v>C23138</x:v>
-      </x:c>
+        <x:v>C22775</x:v>
+      </x:c>
+      <x:c r="E27" s="24"/>
     </x:row>
     <x:row r="28" ht="48" customHeight="1">
       <x:c r="A28" s="3" t="str">
-        <x:v>196k ±1%</x:v>
+        <x:v>330/0603/1%</x:v>
       </x:c>
       <x:c r="B28" s="3" t="str">
-        <x:v>R45</x:v>
+        <x:v>R44, R77</x:v>
       </x:c>
       <x:c r="C28" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D28" s="3" t="str">
-        <x:v>C4203218</x:v>
-      </x:c>
+        <x:v>C23138</x:v>
+      </x:c>
+      <x:c r="E28" s="24"/>
     </x:row>
     <x:row r="29" ht="48" customHeight="1">
       <x:c r="A29" s="3" t="str">
-        <x:v>30K/0603/1%</x:v>
+        <x:v>196k ±1%</x:v>
       </x:c>
       <x:c r="B29" s="3" t="str">
-        <x:v>R46, R74, R76</x:v>
+        <x:v>R45</x:v>
       </x:c>
       <x:c r="C29" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D29" s="3" t="str">
-        <x:v>C22984</x:v>
-      </x:c>
+        <x:v>C4203218</x:v>
+      </x:c>
+      <x:c r="E29" s="24"/>
     </x:row>
     <x:row r="30" ht="48" customHeight="1">
       <x:c r="A30" s="3" t="str">
-        <x:v>270K/0603/1%</x:v>
+        <x:v>30K/0603/1%</x:v>
       </x:c>
       <x:c r="B30" s="3" t="str">
-        <x:v>R60</x:v>
+        <x:v>R46, R74</x:v>
       </x:c>
       <x:c r="C30" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D30" s="3" t="str">
-        <x:v>C22965</x:v>
-      </x:c>
+        <x:v>C22984</x:v>
+      </x:c>
+      <x:c r="E30" s="24"/>
     </x:row>
     <x:row r="31" ht="48" customHeight="1">
       <x:c r="A31" s="3" t="str">
-        <x:v>135k ±0.1%</x:v>
+        <x:v>22k ±1%</x:v>
       </x:c>
       <x:c r="B31" s="3" t="str">
-        <x:v>R61</x:v>
+        <x:v>R76</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D31" s="3" t="str">
-        <x:v>C861113</x:v>
-      </x:c>
+        <x:v>C31850</x:v>
+      </x:c>
+      <x:c r="E31" s="24"/>
     </x:row>
     <x:row r="32" ht="48" customHeight="1">
       <x:c r="A32" s="3" t="str">
-        <x:v>549R ±1%</x:v>
+        <x:v>270K/0603/1%</x:v>
       </x:c>
       <x:c r="B32" s="3" t="str">
-        <x:v>R73</x:v>
+        <x:v>R60</x:v>
       </x:c>
       <x:c r="C32" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D32" s="3" t="str">
-        <x:v>C23079</x:v>
-      </x:c>
+        <x:v>C22965</x:v>
+      </x:c>
+      <x:c r="E32" s="24"/>
     </x:row>
     <x:row r="33" ht="48" customHeight="1">
       <x:c r="A33" s="3" t="str">
-        <x:v>680k ±1%</x:v>
+        <x:v>100k ±1%</x:v>
       </x:c>
       <x:c r="B33" s="3" t="str">
-        <x:v>R78</x:v>
+        <x:v>R61</x:v>
       </x:c>
       <x:c r="C33" s="3" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D33" s="3" t="str">
-        <x:v>C25822</x:v>
-      </x:c>
+        <x:v>C25803</x:v>
+      </x:c>
+      <x:c r="E33" s="24"/>
     </x:row>
     <x:row r="34" ht="48" customHeight="1">
       <x:c r="A34" s="3" t="str">
-        <x:v>100K/0603/1%</x:v>
+        <x:v>560R ±1%</x:v>
       </x:c>
       <x:c r="B34" s="3" t="str">
-        <x:v>R79</x:v>
+        <x:v>R73</x:v>
       </x:c>
       <x:c r="C34" s="3" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D34" s="3" t="str">
-        <x:v>C25803</x:v>
-      </x:c>
+        <x:v>C23204</x:v>
+      </x:c>
+      <x:c r="E34" s="24"/>
     </x:row>
     <x:row r="35" ht="48" customHeight="1">
       <x:c r="A35" s="3" t="str">
-        <x:v>390k ±1%</x:v>
+        <x:v>680k ±1%</x:v>
       </x:c>
       <x:c r="B35" s="3" t="str">
-        <x:v>R80</x:v>
+        <x:v>R78</x:v>
       </x:c>
       <x:c r="C35" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D35" s="3" t="str">
-        <x:v>C2759410</x:v>
-      </x:c>
+        <x:v>C25822</x:v>
+      </x:c>
+      <x:c r="E35" s="24"/>
     </x:row>
     <x:row r="36" ht="48" customHeight="1">
       <x:c r="A36" s="3" t="str">
-        <x:v>1.65k ±1%</x:v>
+        <x:v>100K/0603/1%</x:v>
       </x:c>
       <x:c r="B36" s="3" t="str">
-        <x:v>R81</x:v>
+        <x:v>R79</x:v>
       </x:c>
       <x:c r="C36" s="3" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D36" s="3" t="str">
-        <x:v>C22845</x:v>
-      </x:c>
+        <x:v>C25803</x:v>
+      </x:c>
+      <x:c r="E36" s="24"/>
     </x:row>
     <x:row r="37" ht="48" customHeight="1">
       <x:c r="A37" s="3" t="str">
-        <x:v>TL3301NF160QG/P010515</x:v>
+        <x:v>390k ±1%</x:v>
       </x:c>
       <x:c r="B37" s="3" t="str">
-        <x:v>SW1, SW2, SW3, SW4</x:v>
+        <x:v>R80</x:v>
       </x:c>
       <x:c r="C37" s="3" t="str">
-        <x:v>RheoBoard:Tactile_Switch_4pad</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D37" s="3" t="str">
-        <x:v>C273527</x:v>
-      </x:c>
+        <x:v>C2759410</x:v>
+      </x:c>
+      <x:c r="E37" s="24"/>
     </x:row>
     <x:row r="38" ht="48" customHeight="1">
       <x:c r="A38" s="3" t="str">
-        <x:v>TPS563203DRLR</x:v>
+        <x:v>1.65k ±1%</x:v>
       </x:c>
       <x:c r="B38" s="3" t="str">
-        <x:v>U1, U2, U3</x:v>
+        <x:v>R81</x:v>
       </x:c>
       <x:c r="C38" s="3" t="str">
-        <x:v>RheoBoard:TPS563203DRLR</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D38" s="3" t="str">
-        <x:v>C22445512</x:v>
-      </x:c>
+        <x:v>C22845</x:v>
+      </x:c>
+      <x:c r="E38" s="24"/>
     </x:row>
     <x:row r="39" ht="48" customHeight="1">
       <x:c r="A39" s="3" t="str">
-        <x:v>MPRLS0025PA00001A</x:v>
+        <x:v>TL3301NF160QG/P010515</x:v>
       </x:c>
       <x:c r="B39" s="3" t="str">
-        <x:v>U5</x:v>
+        <x:v>SW1, SW2, SW3, SW4</x:v>
       </x:c>
       <x:c r="C39" s="3" t="str">
-        <x:v>RheoBoard:MPRLS0025PA00001A</x:v>
+        <x:v>RheoBoard:Tactile_Switch_4pad</x:v>
       </x:c>
       <x:c r="D39" s="3" t="str">
-        <x:v>C3257154</x:v>
-      </x:c>
+        <x:v>C273527</x:v>
+      </x:c>
+      <x:c r="E39" s="24"/>
     </x:row>
     <x:row r="40" ht="48" customHeight="1">
       <x:c r="A40" s="3" t="str">
-        <x:v>PCA9685PW,118</x:v>
+        <x:v>TPS563203DRLR</x:v>
       </x:c>
       <x:c r="B40" s="3" t="str">
-        <x:v>U7</x:v>
+        <x:v>U1, U2, U3</x:v>
       </x:c>
       <x:c r="C40" s="3" t="str">
-        <x:v>RheoBoard:PCA9685</x:v>
+        <x:v>RheoBoard:TPS563203DRLR</x:v>
       </x:c>
       <x:c r="D40" s="3" t="str">
-        <x:v>C2678753</x:v>
-      </x:c>
+        <x:v>C22445512</x:v>
+      </x:c>
+      <x:c r="E40" s="24"/>
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" s="3" t="str">
-        <x:v>TPS259472ARPWR</x:v>
+        <x:v>MPRLS0025PA00001A</x:v>
       </x:c>
       <x:c r="B41" s="3" t="str">
-        <x:v>U12</x:v>
+        <x:v>U5</x:v>
       </x:c>
       <x:c r="C41" s="3" t="str">
-        <x:v>RheoBoard:TI_RPW0010A_VQFN-HR_2x2mm</x:v>
+        <x:v>RheoBoard:MPRLS0025PA00001A</x:v>
       </x:c>
       <x:c r="D41" s="3" t="str">
-        <x:v>C3662789</x:v>
-      </x:c>
+        <x:v>C3257154</x:v>
+      </x:c>
+      <x:c r="E41" s="24"/>
     </x:row>
     <x:row r="42" ht="70" customHeight="1">
       <x:c r="A42" s="3" t="str">
-        <x:v>TCA9517ADGKR</x:v>
+        <x:v>PCA9685PW,118</x:v>
       </x:c>
       <x:c r="B42" s="3" t="str">
-        <x:v>U13</x:v>
+        <x:v>U7</x:v>
       </x:c>
       <x:c r="C42" s="3" t="str">
-        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
+        <x:v>RheoBoard:PCA9685</x:v>
       </x:c>
       <x:c r="D42" s="3" t="str">
-        <x:v>C201698</x:v>
-      </x:c>
+        <x:v>C2678753</x:v>
+      </x:c>
+      <x:c r="E42" s="24"/>
     </x:row>
     <x:row r="43" ht="70" customHeight="1">
       <x:c r="A43" s="3" t="str">
-        <x:v>BZT52C10-7-F</x:v>
+        <x:v>TPS259472ARPWR</x:v>
       </x:c>
       <x:c r="B43" s="3" t="str">
-        <x:v>D37</x:v>
+        <x:v>U12</x:v>
       </x:c>
       <x:c r="C43" s="3" t="str">
-        <x:v>Diode_SMD:D_SOD-123</x:v>
+        <x:v>RheoBoard:TI_RPW0010A_VQFN-HR_2x2mm</x:v>
       </x:c>
       <x:c r="D43" s="3" t="str">
-        <x:v>C155227</x:v>
-      </x:c>
+        <x:v>C3662789</x:v>
+      </x:c>
+      <x:c r="E43" s="24"/>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" s="3" t="str">
+        <x:v>TCA9517ADGKR</x:v>
+      </x:c>
+      <x:c r="B44" s="3" t="str">
+        <x:v>U13</x:v>
+      </x:c>
+      <x:c r="C44" s="3" t="str">
+        <x:v>RheoBoard:TI_DGK0008A_VSSOP_3x3mm_P0.65mm</x:v>
+      </x:c>
+      <x:c r="D44" s="3" t="str">
+        <x:v>C201698</x:v>
+      </x:c>
+      <x:c r="E44" s="24"/>
+    </x:row>
+    <x:row r="45" ht="70" customHeight="1">
+      <x:c r="A45" t="str">
+        <x:v>BZT52C10-7-F</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>D37</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>Diode_SMD:D_SOD-123</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>C155227</x:v>
+      </x:c>
+      <x:c r="E45" s="24"/>
+    </x:row>
+    <x:row r="46" ht="70" customHeight="1">
+      <x:c r="A46" t="str">
         <x:v>AO3400A</x:v>
       </x:c>
-      <x:c r="B44" s="3" t="str">
+      <x:c r="B46" t="str">
         <x:v>Q3</x:v>
       </x:c>
-      <x:c r="C44" s="3" t="str">
+      <x:c r="C46" t="str">
         <x:v>RheoBoard:AO3400A_Pin1Offset</x:v>
       </x:c>
-      <x:c r="D44" s="3" t="str">
+      <x:c r="D46" t="str">
         <x:v>C20917</x:v>
       </x:c>
-    </x:row>
-    <x:row r="45" ht="70" customHeight="1">
-      <x:c r="A45"/>
-      <x:c r="B45"/>
-      <x:c r="C45"/>
-      <x:c r="D45"/>
-    </x:row>
-    <x:row r="46" ht="70" customHeight="1">
-      <x:c r="A46"/>
-      <x:c r="B46"/>
-      <x:c r="C46"/>
-      <x:c r="D46"/>
+      <x:c r="E46" s="24"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24517812b014401d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R802152188f2640d4"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="76" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="39" t="str">
+        <x:v>RheoBoard v1.05 — full board parts cost</x:v>
+      </x:c>
+      <x:c r="B1" s="38"/>
+      <x:c r="C1" s="38"/>
+      <x:c r="D1" s="38"/>
+      <x:c r="E1" s="38"/>
+      <x:c r="F1" s="38"/>
+      <x:c r="G1" s="38"/>
+      <x:c r="H1" s="38"/>
+      <x:c r="I1" s="38"/>
+      <x:c r="J1" s="38"/>
+      <x:c r="K1" s="38"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="38" t="str">
+        <x:v>USD • prices checked 2026-10-27 • five-board purchasing basis</x:v>
+      </x:c>
+      <x:c r="B2" s="38"/>
+      <x:c r="C2" s="38"/>
+      <x:c r="D2" s="38"/>
+      <x:c r="E2" s="38"/>
+      <x:c r="F2" s="38"/>
+      <x:c r="G2" s="38"/>
+      <x:c r="H2" s="38"/>
+      <x:c r="I2" s="38"/>
+      <x:c r="J2" s="38"/>
+      <x:c r="K2" s="38"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="38"/>
+      <x:c r="B3" s="38"/>
+      <x:c r="C3" s="38"/>
+      <x:c r="D3" s="38"/>
+      <x:c r="E3" s="38"/>
+      <x:c r="F3" s="38"/>
+      <x:c r="G3" s="38"/>
+      <x:c r="H3" s="38"/>
+      <x:c r="I3" s="38"/>
+      <x:c r="J3" s="38"/>
+      <x:c r="K3" s="38"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="38" t="str">
+        <x:v>Boards in this estimate</x:v>
+      </x:c>
+      <x:c r="B4" s="49" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C4" s="38"/>
+      <x:c r="D4" s="38"/>
+      <x:c r="E4" s="38"/>
+      <x:c r="F4" s="38"/>
+      <x:c r="G4" s="38"/>
+      <x:c r="H4" s="38"/>
+      <x:c r="I4" s="38"/>
+      <x:c r="J4" s="38"/>
+      <x:c r="K4" s="38"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="38"/>
+      <x:c r="B5" s="38"/>
+      <x:c r="C5" s="38"/>
+      <x:c r="D5" s="38"/>
+      <x:c r="E5" s="38"/>
+      <x:c r="F5" s="38"/>
+      <x:c r="G5" s="38"/>
+      <x:c r="H5" s="38"/>
+      <x:c r="I5" s="38"/>
+      <x:c r="J5" s="38"/>
+      <x:c r="K5" s="38"/>
+    </x:row>
+    <x:row r="6" ht="32" customHeight="1">
+      <x:c r="A6" s="42" t="str">
+        <x:v>Cost category</x:v>
+      </x:c>
+      <x:c r="B6" s="42" t="str">
+        <x:v>Per board (USD)</x:v>
+      </x:c>
+      <x:c r="C6" s="42" t="str">
+        <x:v>Five boards (USD)</x:v>
+      </x:c>
+      <x:c r="D6" s="38"/>
+      <x:c r="E6" s="38"/>
+      <x:c r="F6" s="38"/>
+      <x:c r="G6" s="38"/>
+      <x:c r="H6" s="38"/>
+      <x:c r="I6" s="38"/>
+      <x:c r="J6" s="38"/>
+      <x:c r="K6" s="38"/>
+    </x:row>
+    <x:row r="7" ht="26" customHeight="1">
+      <x:c r="A7" s="38" t="str">
+        <x:v>JLCPCB SMT components</x:v>
+      </x:c>
+      <x:c r="B7" s="46" t="n">
+        <x:f>SUMIFS(Sheet1!G2:G51,Sheet1!L2:L51,"SMT")</x:f>
+        <x:v>22.021199999999997</x:v>
+      </x:c>
+      <x:c r="C7" s="46" t="n">
+        <x:f>B7*$B$4</x:f>
+        <x:v>110.10599999999998</x:v>
+      </x:c>
+      <x:c r="D7" s="38"/>
+      <x:c r="E7" s="38"/>
+      <x:c r="F7" s="38"/>
+      <x:c r="G7" s="38"/>
+      <x:c r="H7" s="38"/>
+      <x:c r="I7" s="38"/>
+      <x:c r="J7" s="38"/>
+      <x:c r="K7" s="38"/>
+    </x:row>
+    <x:row r="8" ht="26" customHeight="1">
+      <x:c r="A8" s="38" t="str">
+        <x:v>Manually fitted parts and valves</x:v>
+      </x:c>
+      <x:c r="B8" s="46" t="n">
+        <x:f>SUM(H18:H23)</x:f>
+        <x:v>22.447400000000002</x:v>
+      </x:c>
+      <x:c r="C8" s="46" t="n">
+        <x:f>B8*$B$4</x:f>
+        <x:v>112.23700000000001</x:v>
+      </x:c>
+      <x:c r="D8" s="38"/>
+      <x:c r="E8" s="38"/>
+      <x:c r="F8" s="38"/>
+      <x:c r="G8" s="38"/>
+      <x:c r="H8" s="38"/>
+      <x:c r="I8" s="38"/>
+      <x:c r="J8" s="38"/>
+      <x:c r="K8" s="38"/>
+    </x:row>
+    <x:row r="9" ht="26" customHeight="1">
+      <x:c r="A9" s="43" t="str">
+        <x:v>Total parts consumed</x:v>
+      </x:c>
+      <x:c r="B9" s="47" t="n">
+        <x:f>SUM(B7:B8)</x:f>
+        <x:v>44.468599999999995</x:v>
+      </x:c>
+      <x:c r="C9" s="47" t="n">
+        <x:f>SUM(C7:C8)</x:f>
+        <x:v>222.343</x:v>
+      </x:c>
+      <x:c r="D9" s="38"/>
+      <x:c r="E9" s="38"/>
+      <x:c r="F9" s="38"/>
+      <x:c r="G9" s="38"/>
+      <x:c r="H9" s="38"/>
+      <x:c r="I9" s="38"/>
+      <x:c r="J9" s="38"/>
+      <x:c r="K9" s="38"/>
+    </x:row>
+    <x:row r="10" ht="26" customHeight="1">
+      <x:c r="A10" s="38" t="str">
+        <x:v>Minimum-pack surplus</x:v>
+      </x:c>
+      <x:c r="B10" s="46" t="n">
+        <x:f>C10/$B$4</x:f>
+        <x:v>0.1993999999999943</x:v>
+      </x:c>
+      <x:c r="C10" s="46" t="n">
+        <x:f>SUM(J18:J23)-C8</x:f>
+        <x:v>0.9969999999999715</x:v>
+      </x:c>
+      <x:c r="D10" s="38"/>
+      <x:c r="E10" s="38"/>
+      <x:c r="F10" s="38"/>
+      <x:c r="G10" s="38"/>
+      <x:c r="H10" s="38"/>
+      <x:c r="I10" s="38"/>
+      <x:c r="J10" s="38"/>
+      <x:c r="K10" s="38"/>
+    </x:row>
+    <x:row r="11" ht="26" customHeight="1">
+      <x:c r="A11" s="45" t="str">
+        <x:v>Parts purchase budget</x:v>
+      </x:c>
+      <x:c r="B11" s="48" t="n">
+        <x:f>C11/$B$4</x:f>
+        <x:v>44.66799999999999</x:v>
+      </x:c>
+      <x:c r="C11" s="48" t="n">
+        <x:f>SUM(C9:C10)</x:f>
+        <x:v>223.33999999999997</x:v>
+      </x:c>
+      <x:c r="D11" s="38"/>
+      <x:c r="E11" s="38"/>
+      <x:c r="F11" s="38"/>
+      <x:c r="G11" s="38"/>
+      <x:c r="H11" s="38"/>
+      <x:c r="I11" s="38"/>
+      <x:c r="J11" s="38"/>
+      <x:c r="K11" s="38"/>
+    </x:row>
+    <x:row r="12" ht="40" customHeight="1">
+      <x:c r="A12" s="38" t="str">
+        <x:v>Header availability</x:v>
+      </x:c>
+      <x:c r="B12" s="54" t="str">
+        <x:v>C124379: 18,170 in stock on 2026-10-27; buy 10.</x:v>
+      </x:c>
+      <x:c r="C12" s="54"/>
+      <x:c r="D12" s="54"/>
+      <x:c r="E12" s="38"/>
+      <x:c r="F12" s="38"/>
+      <x:c r="G12" s="38"/>
+      <x:c r="H12" s="38"/>
+      <x:c r="I12" s="38"/>
+      <x:c r="J12" s="38"/>
+      <x:c r="K12" s="38"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="38"/>
+      <x:c r="B13" s="38"/>
+      <x:c r="C13" s="38"/>
+      <x:c r="D13" s="38"/>
+      <x:c r="E13" s="38"/>
+      <x:c r="F13" s="38"/>
+      <x:c r="G13" s="38"/>
+      <x:c r="H13" s="38"/>
+      <x:c r="I13" s="38"/>
+      <x:c r="J13" s="38"/>
+      <x:c r="K13" s="38"/>
+    </x:row>
+    <x:row r="14" ht="32" customHeight="1">
+      <x:c r="A14" s="27" t="str">
+        <x:v>Includes all 142 fitted BOM parts plus two external valves per board. Prices below use the five-board order tiers. Per-board costs are allocations of that batch, not a one-board shopping quote.</x:v>
+      </x:c>
+      <x:c r="B14" s="27"/>
+      <x:c r="C14" s="27"/>
+      <x:c r="D14" s="27"/>
+      <x:c r="E14" s="27"/>
+      <x:c r="F14" s="27"/>
+      <x:c r="G14" s="27"/>
+      <x:c r="H14" s="27"/>
+      <x:c r="I14" s="27"/>
+      <x:c r="J14" s="27"/>
+      <x:c r="K14" s="27"/>
+    </x:row>
+    <x:row r="15" ht="32" customHeight="1">
+      <x:c r="A15" s="27" t="str">
+        <x:v>Excludes PCB fabrication, assembly fees/labor, SMT attrition, shipping and tax. System controller, mux, power supply, cables, tubing and mounting materials remain separate; see Manual accessories.</x:v>
+      </x:c>
+      <x:c r="B15" s="27"/>
+      <x:c r="C15" s="27"/>
+      <x:c r="D15" s="27"/>
+      <x:c r="E15" s="27"/>
+      <x:c r="F15" s="27"/>
+      <x:c r="G15" s="27"/>
+      <x:c r="H15" s="27"/>
+      <x:c r="I15" s="27"/>
+      <x:c r="J15" s="27"/>
+      <x:c r="K15" s="27"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="38"/>
+      <x:c r="B16" s="38"/>
+      <x:c r="C16" s="38"/>
+      <x:c r="D16" s="38"/>
+      <x:c r="E16" s="38"/>
+      <x:c r="F16" s="38"/>
+      <x:c r="G16" s="38"/>
+      <x:c r="H16" s="38"/>
+      <x:c r="I16" s="38"/>
+      <x:c r="J16" s="38"/>
+      <x:c r="K16" s="38"/>
+    </x:row>
+    <x:row r="17" ht="44" customHeight="1">
+      <x:c r="A17" s="42" t="str">
+        <x:v>Manual part</x:v>
+      </x:c>
+      <x:c r="B17" s="42" t="str">
+        <x:v>Reference</x:v>
+      </x:c>
+      <x:c r="C17" s="42" t="str">
+        <x:v>Qty / board</x:v>
+      </x:c>
+      <x:c r="D17" s="42" t="str">
+        <x:v>Needed for batch</x:v>
+      </x:c>
+      <x:c r="E17" s="42" t="str">
+        <x:v>Usable parts / pack</x:v>
+      </x:c>
+      <x:c r="F17" s="42" t="str">
+        <x:v>Pack multiple</x:v>
+      </x:c>
+      <x:c r="G17" s="42" t="str">
+        <x:v>Price / pack USD</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="str">
+        <x:v>Used / board USD</x:v>
+      </x:c>
+      <x:c r="I17" s="42" t="str">
+        <x:v>Packs to buy</x:v>
+      </x:c>
+      <x:c r="J17" s="42" t="str">
+        <x:v>Batch purchase USD</x:v>
+      </x:c>
+      <x:c r="K17" s="42" t="str">
+        <x:v>Source and pricing basis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="72" customHeight="1">
+      <x:c r="A18" s="32" t="str">
+        <x:v>DC barrel jack</x:v>
+      </x:c>
+      <x:c r="B18" s="32" t="str">
+        <x:v>J2</x:v>
+      </x:c>
+      <x:c r="C18" s="53" t="n">
+        <x:f>Sheet1!E21</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D18" s="53" t="n">
+        <x:f>C18*$B$4</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E18" s="53" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F18" s="53" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G18" s="51" t="n">
+        <x:v>2.608</x:v>
+      </x:c>
+      <x:c r="H18" s="51" t="n">
+        <x:f>C18*G18/E18</x:f>
+        <x:v>2.608</x:v>
+      </x:c>
+      <x:c r="I18" s="53" t="n">
+        <x:f>ROUNDUP(D18/E18/F18,0)*F18</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J18" s="52" t="n">
+        <x:f>I18*G18</x:f>
+        <x:v>13.040000000000001</x:v>
+      </x:c>
+      <x:c r="K18" s="32" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C3094233.html — 1+ tier, minimum 1; 490 in stock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="72" customHeight="1">
+      <x:c r="A19" s="32" t="str">
+        <x:v>Four-pin debug header</x:v>
+      </x:c>
+      <x:c r="B19" s="32" t="str">
+        <x:v>J3</x:v>
+      </x:c>
+      <x:c r="C19" s="53" t="n">
+        <x:f>Sheet1!E22</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D19" s="53" t="n">
+        <x:f>C19*$B$4</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E19" s="53" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F19" s="53" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G19" s="51" t="n">
+        <x:v>0.0613</x:v>
+      </x:c>
+      <x:c r="H19" s="51" t="n">
+        <x:f>C19*G19/E19</x:f>
+        <x:v>0.0613</x:v>
+      </x:c>
+      <x:c r="I19" s="53" t="n">
+        <x:f>ROUNDUP(D19/E19/F19,0)*F19</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J19" s="52" t="n">
+        <x:f>I19*G19</x:f>
+        <x:v>0.613</x:v>
+      </x:c>
+      <x:c r="K19" s="32" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C160258.html — minimum / multiple 10; buy 10, fit 5.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="96" customHeight="1">
+      <x:c r="A20" s="32" t="str">
+        <x:v>Five-pin button header</x:v>
+      </x:c>
+      <x:c r="B20" s="32" t="str">
+        <x:v>J19</x:v>
+      </x:c>
+      <x:c r="C20" s="53" t="n">
+        <x:f>Sheet1!E50</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D20" s="53" t="n">
+        <x:f>C20*$B$4</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E20" s="53" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F20" s="53" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G20" s="51" t="n">
+        <x:v>0.0561</x:v>
+      </x:c>
+      <x:c r="H20" s="51" t="n">
+        <x:f>C20*G20/E20</x:f>
+        <x:v>0.0561</x:v>
+      </x:c>
+      <x:c r="I20" s="53" t="n">
+        <x:f>ROUNDUP(D20/E20/F20,0)*F20</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J20" s="52" t="n">
+        <x:f>I20*G20</x:f>
+        <x:v>0.5609999999999999</x:v>
+      </x:c>
+      <x:c r="K20" s="32" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C124379.html — Ckmtw B-2100S05P-A110; 18,170 in stock on 2026-10-27. $0.0561 each, minimum / multiple 10. Buy ten complete 5-pin headers, fit five.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="72" customHeight="1">
+      <x:c r="A21" s="32" t="str">
+        <x:v>Air pumps</x:v>
+      </x:c>
+      <x:c r="B21" s="32" t="str">
+        <x:v>U8, U11</x:v>
+      </x:c>
+      <x:c r="C21" s="53" t="n">
+        <x:f>Sheet1!E45</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D21" s="53" t="n">
+        <x:f>C21*$B$4</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E21" s="53" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F21" s="53" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G21" s="51" t="n">
+        <x:v>7.16</x:v>
+      </x:c>
+      <x:c r="H21" s="51" t="n">
+        <x:f>C21*G21/E21</x:f>
+        <x:v>14.32</x:v>
+      </x:c>
+      <x:c r="I21" s="53" t="n">
+        <x:f>ROUNDUP(D21/E21/F21,0)*F21</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J21" s="52" t="n">
+        <x:f>I21*G21</x:f>
+        <x:v>71.6</x:v>
+      </x:c>
+      <x:c r="K21" s="32" t="str">
+        <x:v>https://www.adafruit.com/product/4699 — 10–99 pumps: $7.16 each; below 10: $7.95.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="72" customHeight="1">
+      <x:c r="A22" s="32" t="str">
+        <x:v>Two-pin valve headers</x:v>
+      </x:c>
+      <x:c r="B22" s="32" t="str">
+        <x:v>U9, U10</x:v>
+      </x:c>
+      <x:c r="C22" s="53" t="n">
+        <x:f>Sheet1!E46</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D22" s="53" t="n">
+        <x:f>C22*$B$4</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E22" s="53" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F22" s="53" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G22" s="51" t="n">
+        <x:v>0.041</x:v>
+      </x:c>
+      <x:c r="H22" s="51" t="n">
+        <x:f>C22*G22/E22</x:f>
+        <x:v>0.082</x:v>
+      </x:c>
+      <x:c r="I22" s="53" t="n">
+        <x:f>ROUNDUP(D22/E22/F22,0)*F22</x:f>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J22" s="52" t="n">
+        <x:f>I22*G22</x:f>
+        <x:v>0.8200000000000001</x:v>
+      </x:c>
+      <x:c r="K22" s="32" t="str">
+        <x:v>https://www.lcsc.com/product-detail/C158012.html — minimum / multiple 20; buy 20, fit 10; 399,780 in stock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="72" customHeight="1">
+      <x:c r="A23" s="32" t="str">
+        <x:v>External air valves</x:v>
+      </x:c>
+      <x:c r="B23" s="32" t="str">
+        <x:v>External, U9/U10</x:v>
+      </x:c>
+      <x:c r="C23" s="53" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D23" s="53" t="n">
+        <x:f>C23*$B$4</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E23" s="53" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F23" s="53" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G23" s="51" t="n">
+        <x:v>2.66</x:v>
+      </x:c>
+      <x:c r="H23" s="51" t="n">
+        <x:f>C23*G23/E23</x:f>
+        <x:v>5.32</x:v>
+      </x:c>
+      <x:c r="I23" s="53" t="n">
+        <x:f>ROUNDUP(D23/E23/F23,0)*F23</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J23" s="52" t="n">
+        <x:f>I23*G23</x:f>
+        <x:v>26.6</x:v>
+      </x:c>
+      <x:c r="K23" s="32" t="str">
+        <x:v>https://www.adafruit.com/product/4663 — 10–99 valves: $2.66 each; below 10: $2.95.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="38"/>
+      <x:c r="B24" s="38"/>
+      <x:c r="C24" s="38"/>
+      <x:c r="D24" s="38"/>
+      <x:c r="E24" s="38"/>
+      <x:c r="F24" s="38"/>
+      <x:c r="G24" s="38"/>
+      <x:c r="H24" s="38"/>
+      <x:c r="I24" s="38"/>
+      <x:c r="J24" s="38"/>
+      <x:c r="K24" s="38"/>
+    </x:row>
+    <x:row r="25" ht="32" customHeight="1">
+      <x:c r="A25" s="27" t="str">
+        <x:v>Minimum-pack surplus is included in the purchase budget. Buy ten complete J19 headers and use five. No spares or JLCPCB attrition quantities have been added for SMT parts.</x:v>
+      </x:c>
+      <x:c r="B25" s="27"/>
+      <x:c r="C25" s="27"/>
+      <x:c r="D25" s="27"/>
+      <x:c r="E25" s="27"/>
+      <x:c r="F25" s="27"/>
+      <x:c r="G25" s="27"/>
+      <x:c r="H25" s="27"/>
+      <x:c r="I25" s="27"/>
+      <x:c r="J25" s="27"/>
+      <x:c r="K25" s="27"/>
+    </x:row>
+    <x:row r="26" ht="32" customHeight="1">
+      <x:c r="A26" s="27" t="str">
+        <x:v>Changing batch size updates quantities and pack rounding only. Refresh supplier price tiers before using a different batch size. Stock is not reserved.</x:v>
+      </x:c>
+      <x:c r="B26" s="27"/>
+      <x:c r="C26" s="27"/>
+      <x:c r="D26" s="27"/>
+      <x:c r="E26" s="27"/>
+      <x:c r="F26" s="27"/>
+      <x:c r="G26" s="27"/>
+      <x:c r="H26" s="27"/>
+      <x:c r="I26" s="27"/>
+      <x:c r="J26" s="27"/>
+      <x:c r="K26" s="27"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="B12:D12"/>
+    <x:mergeCell ref="A14:K14"/>
+    <x:mergeCell ref="A15:K15"/>
+    <x:mergeCell ref="A25:K25"/>
+    <x:mergeCell ref="A26:K26"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BOM and manufacturing files for RheoBoard v1.05. Adjusted component values, added new components, and corrected designator placements. Updated creation timestamps for Gerber and manufacturing files to reflect the latest changes.
</commit_message>
<xml_diff>
--- a/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
+++ b/RheoBoard_PCB/RheoBoard_v1.05/BOM/BOM_RheoBoard_v1.05.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb4aff1c3d8994bd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="R72a9e9467a424203"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="Reac696242ad74b35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts cost" sheetId="4" r:id="R84eca56fb32b48f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R4ca0e844c0814f8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual accessories" sheetId="2" r:id="R6fe2f546394a44be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLCPCB SMT only" sheetId="3" r:id="R72436f23782f4389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts cost" sheetId="4" r:id="R6c5d9654e071452a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -280,15 +280,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:Q51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="RheoBoard105Parts" displayName="RheoBoard105Parts" ref="A1:Q53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
     <x:tableColumn id="3" name="Footprint"/>
     <x:tableColumn id="4" name="LCSC / JLCPCB part"/>
     <x:tableColumn id="5" name="Qty"/>
-    <x:tableColumn id="6" name="JLC unit USD (5 boards)"/>
-    <x:tableColumn id="7" name="SMT parts / board USD"/>
+    <x:tableColumn id="6" name="Unit USD (5-board order)"/>
+    <x:tableColumn id="7" name="Fitted parts / board USD"/>
     <x:tableColumn id="8" name="Selected part source"/>
     <x:tableColumn id="9" name="Datasheet / specification"/>
     <x:tableColumn id="10" name="Manufacturer part number"/>
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="RheoBoard105SMT" displayName="RheoBoard105SMT" ref="A1:D46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="RheoBoard105SMT" displayName="RheoBoard105SMT" ref="A1:D48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Comment"/>
     <x:tableColumn id="2" name="Designator"/>
@@ -665,11 +665,11 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="F3" s="9" t="n">
-        <x:v>0.0087</x:v>
+        <x:v>0.0081</x:v>
       </x:c>
       <x:c r="G3" s="9" t="n">
         <x:f>IF(ISNUMBER(F3),E3*F3,"")</x:f>
-        <x:v>0.1566</x:v>
+        <x:v>0.14579999999999999</x:v>
       </x:c>
       <x:c r="H3" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C14663</x:v>
@@ -717,11 +717,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
-        <x:v>0.0051</x:v>
+        <x:v>0.0050999999999999995</x:v>
       </x:c>
       <x:c r="G4" s="9" t="n">
         <x:f>IF(ISNUMBER(F4),E4*F4,"")</x:f>
-        <x:v>0.0051</x:v>
+        <x:v>0.0050999999999999995</x:v>
       </x:c>
       <x:c r="H4" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C5360811</x:v>
@@ -817,11 +817,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="10" t="n">
-        <x:v>0.1789</x:v>
+        <x:v>0.179</x:v>
       </x:c>
       <x:c r="G6" s="9" t="n">
         <x:f>IF(ISNUMBER(F6),E6*F6,"")</x:f>
-        <x:v>0.7156</x:v>
+        <x:v>0.716</x:v>
       </x:c>
       <x:c r="H6" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C128458</x:v>
@@ -871,11 +871,11 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>0.1333</x:v>
+        <x:v>0.1334</x:v>
       </x:c>
       <x:c r="G7" s="9" t="n">
         <x:f>IF(ISNUMBER(F7),E7*F7,"")</x:f>
-        <x:v>0.7998000000000001</x:v>
+        <x:v>0.8004</x:v>
       </x:c>
       <x:c r="H7" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C20416420</x:v>
@@ -909,7 +909,7 @@
         <x:v>18pF 50V C0G ±5%</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>C55, C58</x:v>
+        <x:v>C55</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
@@ -918,14 +918,14 @@
         <x:v>C107040</x:v>
       </x:c>
       <x:c r="E8" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
         <x:v>0.0067</x:v>
       </x:c>
       <x:c r="G8" s="9" t="n">
         <x:f>IF(ISNUMBER(F8),E8*F8,"")</x:f>
-        <x:v>0.0134</x:v>
+        <x:v>0.0067</x:v>
       </x:c>
       <x:c r="H8" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C107040</x:v>
@@ -1119,7 +1119,7 @@
         <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>C66</x:v>
+        <x:v>C66, C70</x:v>
       </x:c>
       <x:c r="C12" s="7" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
@@ -1128,14 +1128,14 @@
         <x:v>C14663</x:v>
       </x:c>
       <x:c r="E12" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F12" s="10" t="n">
-        <x:v>0.0087</x:v>
+        <x:v>0.0081</x:v>
       </x:c>
       <x:c r="G12" s="9" t="n">
         <x:f>IF(ISNUMBER(F12),E12*F12,"")</x:f>
-        <x:v>0.0087</x:v>
+        <x:v>0.0162</x:v>
       </x:c>
       <x:c r="H12" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C14663</x:v>
@@ -1151,7 +1151,7 @@
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="M12" s="7" t="str">
-        <x:v>New local input high-frequency bypass for U12.</x:v>
+        <x:v>Local high-frequency bypass for U12 and U14.</x:v>
       </x:c>
       <x:c r="N12" s="31" t="n">
         <x:v>0.1</x:v>
@@ -1237,11 +1237,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F14" s="9" t="n">
-        <x:v>0.6237</x:v>
+        <x:v>0.624</x:v>
       </x:c>
       <x:c r="G14" s="9" t="n">
         <x:f>IF(ISNUMBER(F14),E14*F14,"")</x:f>
-        <x:v>0.6237</x:v>
+        <x:v>0.624</x:v>
       </x:c>
       <x:c r="H14" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C154901</x:v>
@@ -1337,11 +1337,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F16" s="9" t="n">
-        <x:v>0.0377</x:v>
+        <x:v>0.037700000000000004</x:v>
       </x:c>
       <x:c r="G16" s="9" t="n">
         <x:f>IF(ISNUMBER(F16),E16*F16,"")</x:f>
-        <x:v>0.1508</x:v>
+        <x:v>0.15080000000000002</x:v>
       </x:c>
       <x:c r="H16" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C115205</x:v>
@@ -1435,11 +1435,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F18" s="9" t="n">
-        <x:v>0.1425</x:v>
+        <x:v>0.14250000000000002</x:v>
       </x:c>
       <x:c r="G18" s="9" t="n">
         <x:f>IF(ISNUMBER(F18),E18*F18,"")</x:f>
-        <x:v>0.1425</x:v>
+        <x:v>0.14250000000000002</x:v>
       </x:c>
       <x:c r="H18" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C151252</x:v>
@@ -1485,11 +1485,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F19" s="9" t="n">
-        <x:v>0.2937</x:v>
+        <x:v>0.2938</x:v>
       </x:c>
       <x:c r="G19" s="9" t="n">
         <x:f>IF(ISNUMBER(F19),E19*F19,"")</x:f>
-        <x:v>0.2937</x:v>
+        <x:v>0.2938</x:v>
       </x:c>
       <x:c r="H19" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C53035082</x:v>
@@ -1535,11 +1535,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F20" s="13" t="n">
-        <x:v>0.2148</x:v>
+        <x:v>0.2149</x:v>
       </x:c>
       <x:c r="G20" s="13" t="n">
         <x:f>IF(ISNUMBER(F20),E20*F20,"")</x:f>
-        <x:v>0.8592</x:v>
+        <x:v>0.8596</x:v>
       </x:c>
       <x:c r="H20" s="11" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C160404</x:v>
@@ -1679,11 +1679,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F23" s="9" t="n">
-        <x:v>0.1244</x:v>
+        <x:v>0.1245</x:v>
       </x:c>
       <x:c r="G23" s="9" t="n">
         <x:f>IF(ISNUMBER(F23),E23*F23,"")</x:f>
-        <x:v>0.3732</x:v>
+        <x:v>0.3735</x:v>
       </x:c>
       <x:c r="H23" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C177246</x:v>
@@ -1731,11 +1731,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F24" s="9" t="n">
-        <x:v>0.0889</x:v>
+        <x:v>0.08900000000000001</x:v>
       </x:c>
       <x:c r="G24" s="9" t="n">
         <x:f>IF(ISNUMBER(F24),E24*F24,"")</x:f>
-        <x:v>0.26670000000000005</x:v>
+        <x:v>0.267</x:v>
       </x:c>
       <x:c r="H24" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C20917</x:v>
@@ -1933,11 +1933,11 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="F28" s="9" t="n">
-        <x:v>0.0017</x:v>
+        <x:v>0.0017000000000000001</x:v>
       </x:c>
       <x:c r="G28" s="9" t="n">
         <x:f>IF(ISNUMBER(F28),E28*F28,"")</x:f>
-        <x:v>0.0136</x:v>
+        <x:v>0.013600000000000001</x:v>
       </x:c>
       <x:c r="H28" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C21190</x:v>
@@ -1983,11 +1983,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F29" s="9" t="n">
-        <x:v>0.0023</x:v>
+        <x:v>0.0023000000000000004</x:v>
       </x:c>
       <x:c r="G29" s="9" t="n">
         <x:f>IF(ISNUMBER(F29),E29*F29,"")</x:f>
-        <x:v>0.0092</x:v>
+        <x:v>0.009200000000000002</x:v>
       </x:c>
       <x:c r="H29" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C22775</x:v>
@@ -2185,11 +2185,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F33" s="9" t="n">
-        <x:v>0.0042</x:v>
+        <x:v>0.004200000000000001</x:v>
       </x:c>
       <x:c r="G33" s="9" t="n">
         <x:f>IF(ISNUMBER(F33),E33*F33,"")</x:f>
-        <x:v>0.0042</x:v>
+        <x:v>0.004200000000000001</x:v>
       </x:c>
       <x:c r="H33" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C31850</x:v>
@@ -2222,7 +2222,7 @@
     </x:row>
     <x:row r="34" ht="72" customHeight="1">
       <x:c r="A34" s="7" t="str">
-        <x:v>270K/0603/1%</x:v>
+        <x:v>240k ±1%</x:v>
       </x:c>
       <x:c r="B34" s="7" t="str">
         <x:v>R60</x:v>
@@ -2231,7 +2231,7 @@
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D34" s="7" t="str">
-        <x:v>C22965</x:v>
+        <x:v>C4197</x:v>
       </x:c>
       <x:c r="E34" s="8" t="n">
         <x:v>1</x:v>
@@ -2244,11 +2244,11 @@
         <x:v>0.0018</x:v>
       </x:c>
       <x:c r="H34" s="7" t="str">
-        <x:v>https://jlcpcb.com/partdetail/component/C22965</x:v>
+        <x:v>https://jlcpcb.com/partdetail/component/C4197</x:v>
       </x:c>
       <x:c r="I34" s="7"/>
       <x:c r="J34" s="7" t="str">
-        <x:v>0603WAF2703T5E</x:v>
+        <x:v>0603WAF2403T5E</x:v>
       </x:c>
       <x:c r="K34" s="7" t="str">
         <x:v>UNI-ROYAL</x:v>
@@ -2256,18 +2256,20 @@
       <x:c r="L34" s="7" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="M34" s="7"/>
+      <x:c r="M34" s="7" t="str">
+        <x:v>Valve buck divider: 240k / 30k gives nominal 5.4 V.</x:v>
+      </x:c>
       <x:c r="N34" s="31" t="n">
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="O34" s="32" t="str">
-        <x:v>Feedback/protection: 1% or better. Same value, package, ratings and TCR.</x:v>
+        <x:v>1% or better; 240 kohm, 0603. Preserve divider ratio.</x:v>
       </x:c>
       <x:c r="P34" s="32" t="str">
         <x:v>Extended</x:v>
       </x:c>
       <x:c r="Q34" s="32" t="n">
-        <x:v>220840</x:v>
+        <x:v>101020</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="72" customHeight="1">
@@ -2339,11 +2341,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F36" s="9" t="n">
-        <x:v>0.0034</x:v>
+        <x:v>0.0034000000000000002</x:v>
       </x:c>
       <x:c r="G36" s="9" t="n">
         <x:f>IF(ISNUMBER(F36),E36*F36,"")</x:f>
-        <x:v>0.0034</x:v>
+        <x:v>0.0034000000000000002</x:v>
       </x:c>
       <x:c r="H36" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C23204</x:v>
@@ -2491,11 +2493,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F39" s="9" t="n">
-        <x:v>0.0022</x:v>
+        <x:v>0.0021999999999999997</x:v>
       </x:c>
       <x:c r="G39" s="9" t="n">
         <x:f>IF(ISNUMBER(F39),E39*F39,"")</x:f>
-        <x:v>0.0022</x:v>
+        <x:v>0.0021999999999999997</x:v>
       </x:c>
       <x:c r="H39" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C2759410</x:v>
@@ -2591,11 +2593,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F41" s="9" t="n">
-        <x:v>0.2657</x:v>
+        <x:v>0.2658</x:v>
       </x:c>
       <x:c r="G41" s="9" t="n">
         <x:f>IF(ISNUMBER(F41),E41*F41,"")</x:f>
-        <x:v>1.0628</x:v>
+        <x:v>1.0632</x:v>
       </x:c>
       <x:c r="H41" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C273527</x:v>
@@ -2637,11 +2639,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F42" s="9" t="n">
-        <x:v>0.1197</x:v>
+        <x:v>0.11979999999999999</x:v>
       </x:c>
       <x:c r="G42" s="9" t="n">
         <x:f>IF(ISNUMBER(F42),E42*F42,"")</x:f>
-        <x:v>0.3591</x:v>
+        <x:v>0.35939999999999994</x:v>
       </x:c>
       <x:c r="H42" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C22445512</x:v>
@@ -2685,11 +2687,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F43" s="13" t="n">
-        <x:v>10.4036</x:v>
+        <x:v>10.409099999999999</x:v>
       </x:c>
       <x:c r="G43" s="13" t="n">
         <x:f>IF(ISNUMBER(F43),E43*F43,"")</x:f>
-        <x:v>10.4036</x:v>
+        <x:v>10.409099999999999</x:v>
       </x:c>
       <x:c r="H43" s="11" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C3257154</x:v>
@@ -2733,11 +2735,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F44" s="10" t="n">
-        <x:v>3.3359</x:v>
+        <x:v>3.3375999999999997</x:v>
       </x:c>
       <x:c r="G44" s="13" t="n">
         <x:f>IF(ISNUMBER(F44),E44*F44,"")</x:f>
-        <x:v>3.3359</x:v>
+        <x:v>3.3375999999999997</x:v>
       </x:c>
       <x:c r="H44" s="11" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C2678753</x:v>
@@ -2873,11 +2875,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F47" s="10" t="n">
-        <x:v>1.0754</x:v>
+        <x:v>1.076</x:v>
       </x:c>
       <x:c r="G47" s="9" t="n">
         <x:f>IF(ISNUMBER(F47),E47*F47,"")</x:f>
-        <x:v>1.0754</x:v>
+        <x:v>1.076</x:v>
       </x:c>
       <x:c r="H47" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C3662789</x:v>
@@ -2923,11 +2925,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F48" s="10" t="n">
-        <x:v>0.4878</x:v>
+        <x:v>0.48810000000000003</x:v>
       </x:c>
       <x:c r="G48" s="13" t="n">
         <x:f>IF(ISNUMBER(F48),E48*F48,"")</x:f>
-        <x:v>0.4878</x:v>
+        <x:v>0.48810000000000003</x:v>
       </x:c>
       <x:c r="H48" s="11" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C201698</x:v>
@@ -2973,11 +2975,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F49" s="9" t="n">
-        <x:v>0.0542</x:v>
+        <x:v>0.0543</x:v>
       </x:c>
       <x:c r="G49" s="9" t="n">
         <x:f>IF(ISNUMBER(F49),E49*F49,"")</x:f>
-        <x:v>0.0542</x:v>
+        <x:v>0.0543</x:v>
       </x:c>
       <x:c r="H49" s="7" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C155227</x:v>
@@ -3072,11 +3074,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F51" s="36" t="n">
-        <x:v>0.0889</x:v>
+        <x:v>0.08900000000000001</x:v>
       </x:c>
       <x:c r="G51" s="36" t="n">
         <x:f>IF(ISNUMBER(F51),E51*F51,"")</x:f>
-        <x:v>0.0889</x:v>
+        <x:v>0.08900000000000001</x:v>
       </x:c>
       <x:c r="H51" s="33" t="str">
         <x:v>https://jlcpcb.com/partdetail/component/C20917</x:v>
@@ -3104,64 +3106,125 @@
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
-      <x:c r="A52" s="16" t="str">
-        <x:v>Total fitted parts / cost (valves extra)</x:v>
-      </x:c>
-      <x:c r="B52" s="16"/>
-      <x:c r="C52" s="16"/>
-      <x:c r="D52" s="16"/>
-      <x:c r="E52" s="16" t="n">
-        <x:f>SUM(E2:E51)</x:f>
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="F52" s="37"/>
-      <x:c r="G52" s="37" t="n">
-        <x:f>SUM(G2:G51)</x:f>
-        <x:v>39.1486</x:v>
-      </x:c>
-      <x:c r="H52" s="16"/>
-      <x:c r="I52" s="16"/>
-      <x:c r="J52" s="16"/>
-      <x:c r="K52" s="16"/>
-      <x:c r="L52" s="16"/>
-      <x:c r="M52" s="16"/>
-      <x:c r="N52" s="26"/>
-      <x:c r="O52" s="27"/>
+      <x:c r="A52" s="7" t="str">
+        <x:v>20pF 50V C0G ±5%</x:v>
+      </x:c>
+      <x:c r="B52" s="7" t="str">
+        <x:v>C58</x:v>
+      </x:c>
+      <x:c r="C52" s="7" t="str">
+        <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
+      </x:c>
+      <x:c r="D52" s="7" t="str">
+        <x:v>C1648</x:v>
+      </x:c>
+      <x:c r="E52" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F52" s="9" t="n">
+        <x:v>0.006900000000000001</x:v>
+      </x:c>
+      <x:c r="G52" s="9" t="n">
+        <x:f>IF(ISNUMBER(F52),E52*F52,"")</x:f>
+        <x:v>0.006900000000000001</x:v>
+      </x:c>
+      <x:c r="H52" s="7" t="str">
+        <x:v>https://jlcpcb.com/partdetail/component/C1648</x:v>
+      </x:c>
+      <x:c r="I52" s="7"/>
+      <x:c r="J52" s="7" t="str">
+        <x:v>CL10C200JB8NNNC</x:v>
+      </x:c>
+      <x:c r="K52" s="7" t="str">
+        <x:v>Samsung Electro-Mechanics</x:v>
+      </x:c>
+      <x:c r="L52" s="7" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M52" s="7" t="str">
+        <x:v>Valve buck feed-forward capacitor matched to 240k divider.</x:v>
+      </x:c>
+      <x:c r="N52" s="31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O52" s="32" t="str">
+        <x:v>5% or better, 20 pF C0G/NP0, &gt;=50 V, 0603.</x:v>
+      </x:c>
+      <x:c r="P52" s="32" t="str">
+        <x:v>Basic</x:v>
+      </x:c>
+      <x:c r="Q52" s="32" t="n">
+        <x:v>1638769</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
-      <x:c r="A53" s="16" t="str">
-        <x:v>Fitted parts for 5 boards (valves extra)</x:v>
-      </x:c>
-      <x:c r="B53" s="16"/>
-      <x:c r="C53" s="16"/>
-      <x:c r="D53" s="16"/>
-      <x:c r="E53" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F53"/>
-      <x:c r="G53" s="28" t="n">
-        <x:f>G52*E53</x:f>
-        <x:v>195.743</x:v>
-      </x:c>
-      <x:c r="H53"/>
-      <x:c r="I53"/>
-      <x:c r="J53"/>
-      <x:c r="K53"/>
-      <x:c r="L53"/>
-      <x:c r="M53"/>
-      <x:c r="N53" s="26"/>
-      <x:c r="O53" s="27"/>
+      <x:c r="A53" s="11" t="str">
+        <x:v>TLV803EA29DBZR</x:v>
+      </x:c>
+      <x:c r="B53" s="11" t="str">
+        <x:v>U14</x:v>
+      </x:c>
+      <x:c r="C53" s="11" t="str">
+        <x:v>Package_TO_SOT_SMD:SOT-23</x:v>
+      </x:c>
+      <x:c r="D53" s="11" t="str">
+        <x:v>C1852114</x:v>
+      </x:c>
+      <x:c r="E53" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F53" s="10" t="n">
+        <x:v>0.4373</x:v>
+      </x:c>
+      <x:c r="G53" s="13" t="n">
+        <x:f>IF(ISNUMBER(F53),E53*F53,"")</x:f>
+        <x:v>0.4373</x:v>
+      </x:c>
+      <x:c r="H53" s="11" t="str">
+        <x:v>https://jlcpcb.com/partdetail/component/C1852114</x:v>
+      </x:c>
+      <x:c r="I53" s="11" t="str">
+        <x:v>https://www.ti.com/lit/ds/symlink/tlv803e.pdf</x:v>
+      </x:c>
+      <x:c r="J53" s="11" t="str">
+        <x:v>TLV803EA29DBZR</x:v>
+      </x:c>
+      <x:c r="K53" s="11" t="str">
+        <x:v>Texas Instruments</x:v>
+      </x:c>
+      <x:c r="L53" s="11" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="M53" s="11" t="str">
+        <x:v>2.93 V supervisor, open-drain reset, nominal 200 ms delay. Pin 1 GND, 2 RESET, 3 VDD.</x:v>
+      </x:c>
+      <x:c r="N53" s="31"/>
+      <x:c r="O53" s="32" t="str">
+        <x:v>Exact EA29DBZR variant and pinout required.</x:v>
+      </x:c>
+      <x:c r="P53" s="32" t="str">
+        <x:v>Extended</x:v>
+      </x:c>
+      <x:c r="Q53" s="32" t="n">
+        <x:v>2979</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="40" customHeight="1">
       <x:c r="A54" s="16" t="str">
-        <x:v>See Parts cost for the FULL board parts total: fitted parts plus external valves, and minimum-pack purchase budget. Prices checked 2026-10-27. Excludes PCB, assembly, SMT attrition, shipping, tax and system accessories.</x:v>
+        <x:v>Total fitted parts / cost (valves extra)</x:v>
       </x:c>
       <x:c r="B54" s="16"/>
       <x:c r="C54" s="16"/>
       <x:c r="D54" s="16"/>
-      <x:c r="E54" s="16"/>
-      <x:c r="F54" s="16"/>
-      <x:c r="G54" s="16"/>
+      <x:c r="E54" s="16" t="n">
+        <x:f>SUM(E2:E53)</x:f>
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="F54" s="37"/>
+      <x:c r="G54" s="37" t="n">
+        <x:f>SUM(G2:G53)</x:f>
+        <x:v>39.5942</x:v>
+      </x:c>
       <x:c r="H54" s="16"/>
       <x:c r="I54" s="16"/>
       <x:c r="J54" s="16"/>
@@ -3170,16 +3233,63 @@
       <x:c r="M54" s="16"/>
       <x:c r="N54" s="26"/>
       <x:c r="O54" s="27"/>
-      <x:c r="P54" s="16"/>
-      <x:c r="Q54" s="16"/>
+      <x:c r="P54"/>
+      <x:c r="Q54"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="16" t="str">
+        <x:v>Fitted parts for 5 boards (valves extra)</x:v>
+      </x:c>
+      <x:c r="B55" s="16"/>
+      <x:c r="C55" s="16"/>
+      <x:c r="D55" s="16"/>
+      <x:c r="E55" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F55"/>
+      <x:c r="G55" s="28" t="n">
+        <x:f>G54*E55</x:f>
+        <x:v>197.971</x:v>
+      </x:c>
+      <x:c r="H55"/>
+      <x:c r="I55"/>
+      <x:c r="J55"/>
+      <x:c r="K55"/>
+      <x:c r="L55"/>
+      <x:c r="M55"/>
+      <x:c r="N55" s="26"/>
+      <x:c r="O55" s="27"/>
+      <x:c r="P55"/>
+      <x:c r="Q55"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="16" t="str">
+        <x:v>See Parts cost for the FULL board parts total: fitted parts plus external valves, and minimum-pack purchase budget. Prices checked 2026-10-27. Excludes PCB, assembly, SMT attrition, shipping, tax and system accessories.</x:v>
+      </x:c>
+      <x:c r="B56" s="16"/>
+      <x:c r="C56" s="16"/>
+      <x:c r="D56" s="16"/>
+      <x:c r="E56" s="16"/>
+      <x:c r="F56" s="16"/>
+      <x:c r="G56" s="16"/>
+      <x:c r="H56" s="16"/>
+      <x:c r="I56" s="16"/>
+      <x:c r="J56" s="16"/>
+      <x:c r="K56" s="16"/>
+      <x:c r="L56" s="16"/>
+      <x:c r="M56" s="16"/>
+      <x:c r="N56" s="26"/>
+      <x:c r="O56" s="27"/>
+      <x:c r="P56" s="16"/>
+      <x:c r="Q56" s="16"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A54:Q54"/>
+    <x:mergeCell ref="A56:Q56"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05cc8c22dba84215"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0cdbc7342154a4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3370,7 +3480,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R377052dac96a4745"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12e175ce0abf4b72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3496,7 +3606,7 @@
         <x:v>18pF 50V C0G ±5%</x:v>
       </x:c>
       <x:c r="B8" s="3" t="str">
-        <x:v>C55, C58</x:v>
+        <x:v>C55</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
@@ -3556,7 +3666,7 @@
         <x:v>100nF 50V X7R ±10%</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
-        <x:v>C66</x:v>
+        <x:v>C66, C70</x:v>
       </x:c>
       <x:c r="C12" s="3" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
@@ -3853,7 +3963,7 @@
     </x:row>
     <x:row r="32" ht="48" customHeight="1">
       <x:c r="A32" s="3" t="str">
-        <x:v>270K/0603/1%</x:v>
+        <x:v>240k ±1%</x:v>
       </x:c>
       <x:c r="B32" s="3" t="str">
         <x:v>R60</x:v>
@@ -3862,7 +3972,7 @@
         <x:v>Resistor_SMD:R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</x:v>
       </x:c>
       <x:c r="D32" s="3" t="str">
-        <x:v>C22965</x:v>
+        <x:v>C4197</x:v>
       </x:c>
       <x:c r="E32" s="24"/>
     </x:row>
@@ -4076,10 +4186,38 @@
       </x:c>
       <x:c r="E46" s="24"/>
     </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="3" t="str">
+        <x:v>20pF 50V C0G ±5%</x:v>
+      </x:c>
+      <x:c r="B47" s="3" t="str">
+        <x:v>C58</x:v>
+      </x:c>
+      <x:c r="C47" s="3" t="str">
+        <x:v>Capacitor_SMD:C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</x:v>
+      </x:c>
+      <x:c r="D47" s="3" t="str">
+        <x:v>C1648</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="3" t="str">
+        <x:v>TLV803EA29DBZR</x:v>
+      </x:c>
+      <x:c r="B48" s="3" t="str">
+        <x:v>U14</x:v>
+      </x:c>
+      <x:c r="C48" s="3" t="str">
+        <x:v>Package_TO_SOT_SMD:SOT-23</x:v>
+      </x:c>
+      <x:c r="D48" s="3" t="str">
+        <x:v>C1852114</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R802152188f2640d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09894e4f6a55405e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4198,12 +4336,12 @@
         <x:v>JLCPCB SMT components</x:v>
       </x:c>
       <x:c r="B7" s="46" t="n">
-        <x:f>SUMIFS(Sheet1!G2:G51,Sheet1!L2:L51,"SMT")</x:f>
-        <x:v>22.021199999999997</x:v>
+        <x:f>SUMIFS(Sheet1!G2:G53,Sheet1!L2:L53,"SMT")</x:f>
+        <x:v>22.4668</x:v>
       </x:c>
       <x:c r="C7" s="46" t="n">
         <x:f>B7*$B$4</x:f>
-        <x:v>110.10599999999998</x:v>
+        <x:v>112.334</x:v>
       </x:c>
       <x:c r="D7" s="38"/>
       <x:c r="E7" s="38"/>
@@ -4241,11 +4379,11 @@
       </x:c>
       <x:c r="B9" s="47" t="n">
         <x:f>SUM(B7:B8)</x:f>
-        <x:v>44.468599999999995</x:v>
+        <x:v>44.9142</x:v>
       </x:c>
       <x:c r="C9" s="47" t="n">
         <x:f>SUM(C7:C8)</x:f>
-        <x:v>222.343</x:v>
+        <x:v>224.57100000000003</x:v>
       </x:c>
       <x:c r="D9" s="38"/>
       <x:c r="E9" s="38"/>
@@ -4283,11 +4421,11 @@
       </x:c>
       <x:c r="B11" s="48" t="n">
         <x:f>C11/$B$4</x:f>
-        <x:v>44.66799999999999</x:v>
+        <x:v>45.1136</x:v>
       </x:c>
       <x:c r="C11" s="48" t="n">
         <x:f>SUM(C9:C10)</x:f>
-        <x:v>223.33999999999997</x:v>
+        <x:v>225.56799999999998</x:v>
       </x:c>
       <x:c r="D11" s="38"/>
       <x:c r="E11" s="38"/>
@@ -4330,7 +4468,7 @@
     </x:row>
     <x:row r="14" ht="32" customHeight="1">
       <x:c r="A14" s="27" t="str">
-        <x:v>Includes all 142 fitted BOM parts plus two external valves per board. Prices below use the five-board order tiers. Per-board costs are allocations of that batch, not a one-board shopping quote.</x:v>
+        <x:v>Includes all 144 fitted BOM parts plus two external valves per board. Prices below use the five-board order tiers. Per-board costs are allocations of that batch, not a one-board shopping quote.</x:v>
       </x:c>
       <x:c r="B14" s="27"/>
       <x:c r="C14" s="27"/>

</xml_diff>